<commit_message>
Add shelter draft login pilot
</commit_message>
<xml_diff>
--- a/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
+++ b/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="Rabedb891f48d46e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="R6cda112468394d41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="Rc2eaca78143d466f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="R8876b4b68335425f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="15">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -99,8 +99,55 @@
       <x:color rgb="FF4F4338"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF4F4338"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF2F7D32"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF6F6256"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFB42318"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFA96617"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF2F7D32"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFA96617"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFB42318"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -170,6 +217,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F1EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B4D40"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD88C24"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8ECD8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -201,7 +288,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="93">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -285,6 +372,92 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="13" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="21" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="22" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -516,502 +689,502 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="7" t="str">
+      <x:c r="A2" s="46" t="str">
         <x:v>Admin gate / password</x:v>
       </x:c>
-      <x:c r="B2" s="7" t="str">
+      <x:c r="B2" s="46" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="C2" s="7" t="str">
+      <x:c r="C2" s="46" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D2" s="10" t="str">
+      <x:c r="D2" s="48" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E2" s="7" t="str">
+      <x:c r="E2" s="46" t="str">
         <x:v>Keep temporary phrase gate until real login logic</x:v>
       </x:c>
-      <x:c r="F2" s="12" t="str">
+      <x:c r="F2" s="50" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="7" t="str">
+      <x:c r="A3" s="46" t="str">
         <x:v>Main PawJai admin umbrella</x:v>
       </x:c>
-      <x:c r="B3" s="7" t="str">
+      <x:c r="B3" s="46" t="str">
         <x:v>scattered across /admin/*</x:v>
       </x:c>
-      <x:c r="C3" s="7" t="str">
+      <x:c r="C3" s="46" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D3" s="10" t="str">
+      <x:c r="D3" s="48" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E3" s="7" t="str">
+      <x:c r="E3" s="46" t="str">
         <x:v>Continue moving remaining old admin tools into draft-native routes</x:v>
       </x:c>
-      <x:c r="F3" s="14" t="str">
+      <x:c r="F3" s="52" t="str">
         <x:v>High</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="7" t="str">
+      <x:c r="A4" s="46" t="str">
         <x:v>Partner shelters overview</x:v>
       </x:c>
-      <x:c r="B4" s="7" t="str">
+      <x:c r="B4" s="46" t="str">
         <x:v>mostly inside /admin/bookings</x:v>
       </x:c>
-      <x:c r="C4" s="7" t="str">
+      <x:c r="C4" s="46" t="str">
         <x:v>/admindraft &gt; Partner shelters</x:v>
       </x:c>
-      <x:c r="D4" s="10" t="str">
+      <x:c r="D4" s="48" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E4" s="7" t="str">
+      <x:c r="E4" s="46" t="str">
         <x:v>Add deeper shelter metrics later if wanted</x:v>
       </x:c>
-      <x:c r="F4" s="16" t="str">
+      <x:c r="F4" s="54" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="7" t="str">
+      <x:c r="A5" s="46" t="str">
         <x:v>Shelter profile edit</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="str">
+      <x:c r="B5" s="46" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C5" s="7" t="str">
+      <x:c r="C5" s="46" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D5" s="10" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E5" s="7" t="str">
+      <x:c r="D5" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E5" s="46" t="str">
         <x:v>Real-world save testing per shelter</x:v>
       </x:c>
-      <x:c r="F5" s="12" t="str">
+      <x:c r="F5" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="7" t="str">
+      <x:c r="A6" s="46" t="str">
         <x:v>Shelter logo upload</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="str">
+      <x:c r="B6" s="46" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="str">
+      <x:c r="C6" s="46" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D6" s="10" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="str">
+      <x:c r="D6" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E6" s="46" t="str">
         <x:v>Real-world upload testing per shelter</x:v>
       </x:c>
-      <x:c r="F6" s="12" t="str">
+      <x:c r="F6" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="7" t="str">
+      <x:c r="A7" s="46" t="str">
         <x:v>Shelter donation details</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="str">
+      <x:c r="B7" s="46" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C7" s="7" t="str">
+      <x:c r="C7" s="46" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D7" s="10" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E7" s="7" t="str">
+      <x:c r="D7" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E7" s="46" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F7" s="12" t="str">
+      <x:c r="F7" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="7" t="str">
+      <x:c r="A8" s="46" t="str">
         <x:v>Shelter operating hours</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="str">
+      <x:c r="B8" s="46" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="str">
+      <x:c r="C8" s="46" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D8" s="10" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E8" s="7" t="str">
+      <x:c r="D8" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E8" s="46" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F8" s="12" t="str">
+      <x:c r="F8" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="7" t="str">
+      <x:c r="A9" s="46" t="str">
         <x:v>Shelter blockout dates</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="str">
+      <x:c r="B9" s="46" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C9" s="7" t="str">
+      <x:c r="C9" s="46" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D9" s="10" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E9" s="7" t="str">
+      <x:c r="D9" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E9" s="46" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F9" s="12" t="str">
+      <x:c r="F9" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="7" t="str">
+      <x:c r="A10" s="46" t="str">
         <x:v>Shelter dog listings</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="str">
+      <x:c r="B10" s="46" t="str">
         <x:v>/admin/bookings?view=dogs, /admin/listings</x:v>
       </x:c>
-      <x:c r="C10" s="7" t="str">
+      <x:c r="C10" s="46" t="str">
         <x:v>/admindraft &gt; Dog listings</x:v>
       </x:c>
-      <x:c r="D10" s="17" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E10" s="7" t="str">
+      <x:c r="D10" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E10" s="46" t="str">
         <x:v>Search/status view is enough for shelter listing management; edit remains separate</x:v>
       </x:c>
-      <x:c r="F10" s="14" t="str">
+      <x:c r="F10" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="7" t="str">
+      <x:c r="A11" s="46" t="str">
         <x:v>Create dog listing</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="str">
+      <x:c r="B11" s="46" t="str">
         <x:v>/admin, /admin/dogs/new</x:v>
       </x:c>
-      <x:c r="C11" s="7" t="str">
+      <x:c r="C11" s="46" t="str">
         <x:v>/admindraft/dog-creation</x:v>
       </x:c>
-      <x:c r="D11" s="17" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E11" s="7" t="str">
+      <x:c r="D11" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E11" s="46" t="str">
         <x:v>Draft-native create flow exists; real-world save/photo testing remains</x:v>
       </x:c>
-      <x:c r="F11" s="14" t="str">
+      <x:c r="F11" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="7" t="str">
+      <x:c r="A12" s="46" t="str">
         <x:v>Edit dog listing</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="str">
+      <x:c r="B12" s="46" t="str">
         <x:v>/admin/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="C12" s="7" t="str">
+      <x:c r="C12" s="46" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D12" s="18" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E12" s="7" t="str">
+      <x:c r="D12" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E12" s="46" t="str">
         <x:v>Draft-native edit route reuses the full old edit form; real-world save/photo testing remains</x:v>
       </x:c>
-      <x:c r="F12" s="14" t="str">
+      <x:c r="F12" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="7" t="str">
+      <x:c r="A13" s="46" t="str">
         <x:v>Dog photos / cover order</x:v>
       </x:c>
-      <x:c r="B13" s="7" t="str">
+      <x:c r="B13" s="46" t="str">
         <x:v>/admin, /admin/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="C13" s="7" t="str">
+      <x:c r="C13" s="46" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D13" s="17" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="str">
+      <x:c r="D13" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E13" s="46" t="str">
         <x:v>Edit route now includes existing upload, reorder, cover, and remove tools</x:v>
       </x:c>
-      <x:c r="F13" s="14" t="str">
+      <x:c r="F13" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="7" t="str">
+      <x:c r="A14" s="46" t="str">
         <x:v>All dog listings across shelters</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="str">
+      <x:c r="B14" s="46" t="str">
         <x:v>/admin/listings</x:v>
       </x:c>
-      <x:c r="C14" s="7" t="str">
+      <x:c r="C14" s="46" t="str">
         <x:v>/admindraft &gt; All dog listings</x:v>
       </x:c>
-      <x:c r="D14" s="17" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E14" s="7" t="str">
+      <x:c r="D14" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E14" s="46" t="str">
         <x:v>Filters exist and edit buttons now open draft-native dog edit pages</x:v>
       </x:c>
-      <x:c r="F14" s="14" t="str">
+      <x:c r="F14" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="7" t="str">
+      <x:c r="A15" s="46" t="str">
         <x:v>Booking visits list</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="str">
+      <x:c r="B15" s="46" t="str">
         <x:v>/admin/bookings</x:v>
       </x:c>
-      <x:c r="C15" s="7" t="str">
+      <x:c r="C15" s="46" t="str">
         <x:v>/admindraft &gt; Bookings</x:v>
       </x:c>
-      <x:c r="D15" s="17" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="str">
+      <x:c r="D15" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E15" s="46" t="str">
         <x:v>Old low-friction booking card flow duplicated; real staff testing remains</x:v>
       </x:c>
-      <x:c r="F15" s="14" t="str">
+      <x:c r="F15" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="7" t="str">
+      <x:c r="A16" s="46" t="str">
         <x:v>Booking decision actions</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="str">
+      <x:c r="B16" s="46" t="str">
         <x:v>/admin/bookings, /admin/bookings/[id]</x:v>
       </x:c>
-      <x:c r="C16" s="7" t="str">
+      <x:c r="C16" s="46" t="str">
         <x:v>/admindraft &gt; Bookings</x:v>
       </x:c>
-      <x:c r="D16" s="18" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E16" s="7" t="str">
+      <x:c r="D16" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E16" s="46" t="str">
         <x:v>Accept, deny, and date-change actions are draft-native; final status edge cases can be polished later</x:v>
       </x:c>
-      <x:c r="F16" s="14" t="str">
+      <x:c r="F16" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="7" t="str">
+      <x:c r="A17" s="46" t="str">
         <x:v>Booking detail page</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="str">
+      <x:c r="B17" s="46" t="str">
         <x:v>/admin/bookings/[id]</x:v>
       </x:c>
-      <x:c r="C17" s="7" t="str">
+      <x:c r="C17" s="46" t="str">
         <x:v>/admindraft/bookings/[id]</x:v>
       </x:c>
-      <x:c r="D17" s="18" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E17" s="7" t="str">
+      <x:c r="D17" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E17" s="46" t="str">
         <x:v>QR scan can land here; refine isolated detail page only if needed</x:v>
       </x:c>
-      <x:c r="F17" s="16" t="str">
+      <x:c r="F17" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="7" t="str">
+      <x:c r="A18" s="46" t="str">
         <x:v>QR check-in</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="str">
+      <x:c r="B18" s="46" t="str">
         <x:v>/admin/bookings/check-in</x:v>
       </x:c>
-      <x:c r="C18" s="7" t="str">
+      <x:c r="C18" s="46" t="str">
         <x:v>/admindraft/bookings/check-in</x:v>
       </x:c>
-      <x:c r="D18" s="18" t="str">
+      <x:c r="D18" s="48" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E18" s="7" t="str">
+      <x:c r="E18" s="46" t="str">
         <x:v>Needs real QR/camera device testing</x:v>
       </x:c>
-      <x:c r="F18" s="16" t="str">
+      <x:c r="F18" s="54" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="7" t="str">
+      <x:c r="A19" s="46" t="str">
         <x:v>Visitor profile</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="str">
+      <x:c r="B19" s="46" t="str">
         <x:v>/admin/bookings/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="C19" s="7" t="str">
+      <x:c r="C19" s="46" t="str">
         <x:v>/admindraft/bookings/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="D19" s="18" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="E19" s="7" t="str">
+      <x:c r="D19" s="48" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E19" s="46" t="str">
         <x:v>Draft-native profile/documents view exists; real document review testing remains</x:v>
       </x:c>
-      <x:c r="F19" s="16" t="str">
+      <x:c r="F19" s="48" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="7" t="str">
+      <x:c r="A20" s="46" t="str">
         <x:v>Shelter messaging</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="str">
+      <x:c r="B20" s="46" t="str">
         <x:v>/admin/bookings?view=messages</x:v>
       </x:c>
-      <x:c r="C20" s="7" t="str">
+      <x:c r="C20" s="46" t="str">
         <x:v>/admindraft &gt; Messaging</x:v>
       </x:c>
-      <x:c r="D20" s="17" t="str">
+      <x:c r="D20" s="52" t="str">
         <x:v>Visual only</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="str">
+      <x:c r="E20" s="46" t="str">
         <x:v>Transfer real message thread and send reply in separate messaging session</x:v>
       </x:c>
-      <x:c r="F20" s="14" t="str">
+      <x:c r="F20" s="52" t="str">
         <x:v>High</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="7" t="str">
+      <x:c r="A21" s="46" t="str">
         <x:v>Ads management</x:v>
       </x:c>
-      <x:c r="B21" s="7" t="str">
+      <x:c r="B21" s="46" t="str">
         <x:v>/admin/ads</x:v>
       </x:c>
-      <x:c r="C21" s="7" t="str">
+      <x:c r="C21" s="46" t="str">
         <x:v>/admindraft &gt; Ads</x:v>
       </x:c>
-      <x:c r="D21" s="17" t="str">
+      <x:c r="D21" s="54" t="str">
         <x:v>Read only</x:v>
       </x:c>
-      <x:c r="E21" s="7" t="str">
+      <x:c r="E21" s="46" t="str">
         <x:v>Transfer create ad, edit dates, pause/resume, delete</x:v>
       </x:c>
-      <x:c r="F21" s="16" t="str">
+      <x:c r="F21" s="54" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="7" t="str">
+      <x:c r="A22" s="46" t="str">
         <x:v>About content</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="str">
+      <x:c r="B22" s="46" t="str">
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
-      <x:c r="C22" s="7" t="str">
+      <x:c r="C22" s="46" t="str">
         <x:v>/admindraft &gt; About content</x:v>
       </x:c>
-      <x:c r="D22" s="17" t="str">
+      <x:c r="D22" s="54" t="str">
         <x:v>Read only</x:v>
       </x:c>
-      <x:c r="E22" s="7" t="str">
+      <x:c r="E22" s="46" t="str">
         <x:v>Transfer full About editor/save action</x:v>
       </x:c>
-      <x:c r="F22" s="16" t="str">
+      <x:c r="F22" s="54" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="7" t="str">
+      <x:c r="A23" s="46" t="str">
         <x:v>Admin accounts</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="str">
+      <x:c r="B23" s="46" t="str">
         <x:v>/admin/accounts</x:v>
       </x:c>
-      <x:c r="C23" s="7" t="str">
+      <x:c r="C23" s="46" t="str">
         <x:v>not yet</x:v>
       </x:c>
-      <x:c r="D23" s="18" t="str">
+      <x:c r="D23" s="52" t="str">
         <x:v>Missing</x:v>
       </x:c>
-      <x:c r="E23" s="7" t="str">
+      <x:c r="E23" s="46" t="str">
         <x:v>Transfer PawJai/shelter admin account creation</x:v>
       </x:c>
-      <x:c r="F23" s="12" t="str">
+      <x:c r="F23" s="50" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="7" t="str">
+      <x:c r="A24" s="46" t="str">
         <x:v>Audit log</x:v>
       </x:c>
-      <x:c r="B24" s="7" t="str">
+      <x:c r="B24" s="46" t="str">
         <x:v>/admin/audit</x:v>
       </x:c>
-      <x:c r="C24" s="7" t="str">
+      <x:c r="C24" s="46" t="str">
         <x:v>not yet</x:v>
       </x:c>
-      <x:c r="D24" s="18" t="str">
+      <x:c r="D24" s="52" t="str">
         <x:v>Missing</x:v>
       </x:c>
-      <x:c r="E24" s="7" t="str">
+      <x:c r="E24" s="46" t="str">
         <x:v>Transfer audit table view</x:v>
       </x:c>
-      <x:c r="F24" s="12" t="str">
+      <x:c r="F24" s="50" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="7" t="str">
+      <x:c r="A25" s="46" t="str">
         <x:v>Admin login page</x:v>
       </x:c>
-      <x:c r="B25" s="7" t="str">
+      <x:c r="B25" s="46" t="str">
         <x:v>/admin/login</x:v>
       </x:c>
-      <x:c r="C25" s="7" t="str">
+      <x:c r="C25" s="46" t="str">
         <x:v>temporary phrase gate</x:v>
       </x:c>
-      <x:c r="D25" s="17" t="str">
+      <x:c r="D25" s="54" t="str">
         <x:v>Temporary</x:v>
       </x:c>
-      <x:c r="E25" s="7" t="str">
+      <x:c r="E25" s="46" t="str">
         <x:v>Later replace phrase gates with real auth</x:v>
       </x:c>
-      <x:c r="F25" s="12" t="str">
+      <x:c r="F25" s="50" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="7" t="str">
+      <x:c r="A26" s="46" t="str">
         <x:v>Legacy draft alias</x:v>
       </x:c>
-      <x:c r="B26" s="7" t="str">
+      <x:c r="B26" s="46" t="str">
         <x:v>/admin/reorg-draft</x:v>
       </x:c>
-      <x:c r="C26" s="7" t="str">
+      <x:c r="C26" s="46" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D26" s="10" t="str">
+      <x:c r="D26" s="48" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E26" s="7" t="str">
+      <x:c r="E26" s="46" t="str">
         <x:v>Remove after /admindraft becomes canonical</x:v>
       </x:c>
-      <x:c r="F26" s="12" t="str">
+      <x:c r="F26" s="50" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
@@ -1031,33 +1204,33 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="35" t="str">
+      <x:c r="A1" s="64" t="str">
         <x:v>PAWJAI Admin Draft Transfer Progress</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="43" t="str">
+      <x:c r="A3" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="43" t="str">
+      <x:c r="B3" s="81" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C3" s="43" t="str">
+      <x:c r="C3" s="81" t="str">
         <x:v>% of workflows</x:v>
       </x:c>
-      <x:c r="D3" s="43" t="str">
+      <x:c r="D3" s="81" t="str">
         <x:v>Meaning</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="33" t="str">
-        <x:v>Functional</x:v>
-      </x:c>
-      <x:c r="B4" s="30" t="n">
+      <x:c r="A4" s="88" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="B4" s="82" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A4)</x:f>
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C4" s="32" t="n">
+      <x:c r="C4" s="86" t="n">
         <x:f>B4/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.56</x:v>
       </x:c>
@@ -1066,14 +1239,14 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="33" t="str">
+      <x:c r="A5" s="88" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="B5" s="30" t="n">
+      <x:c r="B5" s="82" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A5)</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C5" s="32" t="n">
+      <x:c r="C5" s="86" t="n">
         <x:f>B5/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.2</x:v>
       </x:c>
@@ -1082,14 +1255,14 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="33" t="str">
+      <x:c r="A6" s="89" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="B6" s="30" t="n">
+      <x:c r="B6" s="83" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C6" s="32" t="n">
+      <x:c r="C6" s="91" t="n">
         <x:f>B6/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1098,14 +1271,14 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="33" t="str">
+      <x:c r="A7" s="89" t="str">
         <x:v>Read only</x:v>
       </x:c>
-      <x:c r="B7" s="30" t="n">
+      <x:c r="B7" s="83" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A7)</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C7" s="32" t="n">
+      <x:c r="C7" s="91" t="n">
         <x:f>B7/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.08</x:v>
       </x:c>
@@ -1114,14 +1287,14 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="33" t="str">
+      <x:c r="A8" s="90" t="str">
         <x:v>Visual only</x:v>
       </x:c>
-      <x:c r="B8" s="30" t="n">
+      <x:c r="B8" s="84" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A8)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="32" t="n">
+      <x:c r="C8" s="92" t="n">
         <x:f>B8/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
@@ -1130,14 +1303,14 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="33" t="str">
+      <x:c r="A9" s="89" t="str">
         <x:v>Temporary</x:v>
       </x:c>
-      <x:c r="B9" s="30" t="n">
+      <x:c r="B9" s="83" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C9" s="32" t="n">
+      <x:c r="C9" s="91" t="n">
         <x:f>B9/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
@@ -1146,14 +1319,14 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="33" t="str">
+      <x:c r="A10" s="90" t="str">
         <x:v>Missing</x:v>
       </x:c>
-      <x:c r="B10" s="30" t="n">
+      <x:c r="B10" s="84" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A10)</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C10" s="32" t="n">
+      <x:c r="C10" s="92" t="n">
         <x:f>B10/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.08</x:v>
       </x:c>
@@ -1162,51 +1335,51 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="44" t="str">
+      <x:c r="A13" s="85" t="str">
         <x:v>Metric</x:v>
       </x:c>
-      <x:c r="B13" s="44" t="str">
+      <x:c r="B13" s="85" t="str">
         <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="33" t="str">
+      <x:c r="A14" s="88" t="str">
         <x:v>Functional workflows</x:v>
       </x:c>
-      <x:c r="B14" s="30" t="n">
+      <x:c r="B14" s="82" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Functional")</x:f>
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="33" t="str">
+      <x:c r="A15" s="88" t="str">
         <x:v>Functional + Exists</x:v>
       </x:c>
-      <x:c r="B15" s="32" t="n">
+      <x:c r="B15" s="86" t="n">
         <x:f>(COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Functional")+COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Exists"))/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.76</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="33" t="str">
+      <x:c r="A16" s="90" t="str">
         <x:v>Still high priority</x:v>
       </x:c>
-      <x:c r="B16" s="30" t="n">
+      <x:c r="B16" s="84" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$F$2:$F$26,"High")</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="33" t="str">
+      <x:c r="A17" s="87" t="str">
         <x:v>Total workflows</x:v>
       </x:c>
-      <x:c r="B17" s="30" t="n">
+      <x:c r="B17" s="87" t="n">
         <x:f>COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
-      <x:c r="A20" s="42" t="str">
+      <x:c r="A20" s="80" t="str">
         <x:v>Current read: shelter profile, dog creation/listing, and booking flows are now the strongest draft areas. Messaging is intentionally left for a separate session.</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Update admin architecture tracker workbook
</commit_message>
<xml_diff>
--- a/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
+++ b/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
@@ -2,10 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="R8e7570dd618e4e1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="Re8f04ed224d44482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="3" r:id="R9f82e309f1384cfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="4" r:id="R0d989a35cd9a45d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="R486035d6a5b74154"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="Rfd35a65c4a834ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="3" r:id="R74a05e29588c4806"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="4" r:id="R76ab6849f6a04757"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="5" r:id="R981289aaddef42dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="6" r:id="R1c4736847d474a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="7" r:id="Rbe1519db220f45b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="8" r:id="Rcc1730b9bc7249c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="9" r:id="R65519966cf804bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="10" r:id="R7d1cffe454e84578"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="11" r:id="R01e20ca402904def"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -377,7 +384,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="17">
+  <x:fonts count="20">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -477,8 +484,25 @@
       <x:color rgb="FF9A3129"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF8A5825"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFB77624"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF5B4D40"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="81">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -580,8 +604,308 @@
         <x:fgColor rgb="FFEAF6DF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4F4338"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDFA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE8E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF6DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1DC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9F2FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFAF3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8DFB8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6EFE6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7E3E1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4F4338"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDFA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE8E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF6DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1DC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9F2FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFAF3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8DFB8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6EFE6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7E3E1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4F4338"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDFA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE8E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF6DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1DC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9F2FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFAF3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8DFB8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6EFE6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7E3E1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4F4338"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDFA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE8E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF6DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1DC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9F2FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFAF3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8DFB8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6EFE6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7E3E1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4F4338"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDFA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE8E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF6DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1DC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9F2FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFAF3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8DFB8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6EFE6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7E3E1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="11">
+  <x:borders count="13">
     <x:border/>
     <x:border>
       <x:top style="thin">
@@ -681,11 +1005,21 @@
         <x:color rgb="FFEADFCE"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFEADFCE"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFEADFCE"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="110">
+  <x:cellXfs count="541">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -952,11 +1286,1123 @@
     <x:xf numFmtId="0" fontId="16" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="24" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="24" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="25" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="26" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="27" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="28" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="26" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="30" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="32" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="26" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="25" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="26" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="24" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="26" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="26" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="37" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="37" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="38" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="38" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="42" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="44" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="38" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="37" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="38" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="38" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="45" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="45" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="45" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="48" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="48" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="49" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="48" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="48" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="48" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="48" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="49" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="50" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="52" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="50" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="54" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="56" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="46" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="46" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="46" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="50" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="49" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="50" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="48" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="48" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="50" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="57" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="57" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="57" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="60" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="60" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="61" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="60" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="60" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="60" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="60" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="61" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="62" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="64" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="62" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="66" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="68" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="58" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="58" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="58" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="62" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="61" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="62" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="60" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="60" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="62" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="62" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="69" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="69" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="69" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="72" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="73" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="72" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="72" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="73" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="74" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="74" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="78" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="79" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="80" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="70" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="70" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="70" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="74" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="73" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="74" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="72" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="74" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="74" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7239000" cy="4095750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="48fd0a8e-8f5f-439d-8f7a-fd98a22e40b7"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R84c8484b21db4309"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7239000" cy="4095750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="9e6d2b00-eee6-4c87-93c4-09fa62d9c950"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3db7df041d0842e2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1686,6 +3132,262 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="92" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="458" t="str">
+        <x:v>PAWJAI Architecture Advisory</x:v>
+      </x:c>
+      <x:c r="B1" s="458" t="str">
+        <x:v>PAWJAI Architecture Advisory</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>PAWJAI Architecture Advisory</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="461" t="str">
+        <x:v>Recommended long-term structure based on the current admin/shelter/booking reorganization.</x:v>
+      </x:c>
+      <x:c r="B2" s="461" t="str">
+        <x:v>Recommended long-term structure based on the current admin/shelter/booking reorganization.</x:v>
+      </x:c>
+      <x:c r="C2" s="461" t="str">
+        <x:v>Recommended long-term structure based on the current admin/shelter/booking reorganization.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="464" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+      <x:c r="B4" s="465" t="str">
+        <x:v>Recommendation</x:v>
+      </x:c>
+      <x:c r="C4" s="466" t="str">
+        <x:v>Reason</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="469" t="str">
+        <x:v>Keep separate route shells</x:v>
+      </x:c>
+      <x:c r="B5" s="470" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="C5" s="471" t="str">
+        <x:v>The two dog edit URLs are two interfaces around one shared form/action and one DB row. This is good long-term because permissions and navigation differ by role.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="472" t="str">
+        <x:v>Do not create duplicate dog tables</x:v>
+      </x:c>
+      <x:c r="B6" s="473" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="C6" s="474" t="str">
+        <x:v>Keep dogs, dog_photos, dog_traits as the single source of truth. Route duplication is okay; data duplication is not.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="472" t="str">
+        <x:v>Use /booking as shared internal booking workspace</x:v>
+      </x:c>
+      <x:c r="B7" s="473" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="C7" s="474" t="str">
+        <x:v>Booking intersects admin, shelter, and adopter data. Shared /booking avoids copying pages while safe returnTo preserves lanes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="472" t="str">
+        <x:v>Do not expose shelter/admin to indexing</x:v>
+      </x:c>
+      <x:c r="B8" s="473" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="C8" s="474" t="str">
+        <x:v>/shelter, /booking, /admin, and /admindraft are noindex/private route groups.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="472" t="str">
+        <x:v>Expect synced after navigation/refresh</x:v>
+      </x:c>
+      <x:c r="B9" s="473" t="str">
+        <x:v>Current</x:v>
+      </x:c>
+      <x:c r="C9" s="474" t="str">
+        <x:v>Both admin and shelter listings reload from Supabase. This is synced data but not live websocket realtime.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="472" t="str">
+        <x:v>Add Supabase Realtime only if needed</x:v>
+      </x:c>
+      <x:c r="B10" s="473" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="C10" s="474" t="str">
+        <x:v>Useful if two staff members need open pages to update instantly after someone else saves a dog/booking.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="475" t="str">
+        <x:v>Pilot-safe missing feature</x:v>
+      </x:c>
+      <x:c r="B11" s="476" t="str">
+        <x:v>Messaging</x:v>
+      </x:c>
+      <x:c r="C11" s="477" t="str">
+        <x:v>Messaging remains the main intentionally pending feature. Do not block dog-data onboarding on messaging unless shelter expects it.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:C1"/>
+    <x:mergeCell ref="A2:C2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="458" t="str">
+        <x:v>Embedded PNG diagram gallery</x:v>
+      </x:c>
+      <x:c r="B1" s="458" t="str">
+        <x:v>Embedded PNG diagram gallery</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>Embedded PNG diagram gallery</x:v>
+      </x:c>
+      <x:c r="D1" s="458" t="str">
+        <x:v>Embedded PNG diagram gallery</x:v>
+      </x:c>
+      <x:c r="E1" s="458" t="str">
+        <x:v>Embedded PNG diagram gallery</x:v>
+      </x:c>
+      <x:c r="F1" s="458" t="str">
+        <x:v>Embedded PNG diagram gallery</x:v>
+      </x:c>
+      <x:c r="G1" s="458" t="str">
+        <x:v>Embedded PNG diagram gallery</x:v>
+      </x:c>
+      <x:c r="H1" s="458" t="str">
+        <x:v>Embedded PNG diagram gallery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="526" t="str">
+        <x:v>These images are generated from the workbook's diagram sheets. Future Codex sessions can read the underlying diagram sheets as text/tables and view these snapshots visually.</x:v>
+      </x:c>
+      <x:c r="B2" s="527" t="str">
+        <x:v>These images are generated from the workbook's diagram sheets. Future Codex sessions can read the underlying diagram sheets as text/tables and view these snapshots visually.</x:v>
+      </x:c>
+      <x:c r="C2" s="527" t="str">
+        <x:v>These images are generated from the workbook's diagram sheets. Future Codex sessions can read the underlying diagram sheets as text/tables and view these snapshots visually.</x:v>
+      </x:c>
+      <x:c r="D2" s="527" t="str">
+        <x:v>These images are generated from the workbook's diagram sheets. Future Codex sessions can read the underlying diagram sheets as text/tables and view these snapshots visually.</x:v>
+      </x:c>
+      <x:c r="E2" s="527" t="str">
+        <x:v>These images are generated from the workbook's diagram sheets. Future Codex sessions can read the underlying diagram sheets as text/tables and view these snapshots visually.</x:v>
+      </x:c>
+      <x:c r="F2" s="527" t="str">
+        <x:v>These images are generated from the workbook's diagram sheets. Future Codex sessions can read the underlying diagram sheets as text/tables and view these snapshots visually.</x:v>
+      </x:c>
+      <x:c r="G2" s="527" t="str">
+        <x:v>These images are generated from the workbook's diagram sheets. Future Codex sessions can read the underlying diagram sheets as text/tables and view these snapshots visually.</x:v>
+      </x:c>
+      <x:c r="H2" s="528" t="str">
+        <x:v>These images are generated from the workbook's diagram sheets. Future Codex sessions can read the underlying diagram sheets as text/tables and view these snapshots visually.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="526" t="str">
+        <x:v>Codex note: if a workbook renderer does not display embedded drawings, use the DB Sync Diagram and Route Flow Diagram sheets as the readable source, or regenerate the PNG previews with workbook-build/update-route-tabs.mjs.</x:v>
+      </x:c>
+      <x:c r="B3" s="527" t="str">
+        <x:v>Codex note: if a workbook renderer does not display embedded drawings, use the DB Sync Diagram and Route Flow Diagram sheets as the readable source, or regenerate the PNG previews with workbook-build/update-route-tabs.mjs.</x:v>
+      </x:c>
+      <x:c r="C3" s="527" t="str">
+        <x:v>Codex note: if a workbook renderer does not display embedded drawings, use the DB Sync Diagram and Route Flow Diagram sheets as the readable source, or regenerate the PNG previews with workbook-build/update-route-tabs.mjs.</x:v>
+      </x:c>
+      <x:c r="D3" s="527" t="str">
+        <x:v>Codex note: if a workbook renderer does not display embedded drawings, use the DB Sync Diagram and Route Flow Diagram sheets as the readable source, or regenerate the PNG previews with workbook-build/update-route-tabs.mjs.</x:v>
+      </x:c>
+      <x:c r="E3" s="527" t="str">
+        <x:v>Codex note: if a workbook renderer does not display embedded drawings, use the DB Sync Diagram and Route Flow Diagram sheets as the readable source, or regenerate the PNG previews with workbook-build/update-route-tabs.mjs.</x:v>
+      </x:c>
+      <x:c r="F3" s="527" t="str">
+        <x:v>Codex note: if a workbook renderer does not display embedded drawings, use the DB Sync Diagram and Route Flow Diagram sheets as the readable source, or regenerate the PNG previews with workbook-build/update-route-tabs.mjs.</x:v>
+      </x:c>
+      <x:c r="G3" s="527" t="str">
+        <x:v>Codex note: if a workbook renderer does not display embedded drawings, use the DB Sync Diagram and Route Flow Diagram sheets as the readable source, or regenerate the PNG previews with workbook-build/update-route-tabs.mjs.</x:v>
+      </x:c>
+      <x:c r="H3" s="528" t="str">
+        <x:v>Codex note: if a workbook renderer does not display embedded drawings, use the DB Sync Diagram and Route Flow Diagram sheets as the readable source, or regenerate the PNG previews with workbook-build/update-route-tabs.mjs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4"/>
+      <x:c r="B4"/>
+      <x:c r="C4"/>
+      <x:c r="D4"/>
+      <x:c r="E4"/>
+      <x:c r="F4"/>
+      <x:c r="G4"/>
+      <x:c r="H4"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="464" t="str">
+        <x:v>DB Sync Diagram snapshot</x:v>
+      </x:c>
+      <x:c r="B5" s="465" t="str"/>
+      <x:c r="C5" s="465" t="str"/>
+      <x:c r="D5" s="465" t="str"/>
+      <x:c r="E5" s="465" t="str">
+        <x:v>Route Flow Diagram snapshot</x:v>
+      </x:c>
+      <x:c r="F5" s="465" t="str"/>
+      <x:c r="G5" s="465" t="str"/>
+      <x:c r="H5" s="466" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R533a6f1712924216"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
@@ -1908,363 +3610,383 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
-      <x:c r="A1" s="82" t="str">
+      <x:c r="A1" s="458" t="str">
         <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
       </x:c>
-      <x:c r="B1" s="82" t="str"/>
-      <x:c r="C1" s="82" t="str"/>
-      <x:c r="D1" s="82" t="str"/>
-      <x:c r="E1" s="82" t="str"/>
-      <x:c r="F1" s="82" t="str"/>
+      <x:c r="B1" s="458" t="str">
+        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
+      </x:c>
+      <x:c r="D1" s="458" t="str">
+        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
+      </x:c>
+      <x:c r="E1" s="458" t="str">
+        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
+      </x:c>
+      <x:c r="F1" s="458" t="str">
+        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="85" t="str">
+      <x:c r="A2" s="461" t="str">
         <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
       </x:c>
-      <x:c r="B2" s="85" t="str"/>
-      <x:c r="C2" s="85" t="str"/>
-      <x:c r="D2" s="85" t="str"/>
-      <x:c r="E2" s="85" t="str"/>
-      <x:c r="F2" s="85" t="str"/>
+      <x:c r="B2" s="461" t="str">
+        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
+      </x:c>
+      <x:c r="C2" s="461" t="str">
+        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
+      </x:c>
+      <x:c r="D2" s="461" t="str">
+        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
+      </x:c>
+      <x:c r="E2" s="461" t="str">
+        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
+      </x:c>
+      <x:c r="F2" s="461" t="str">
+        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="88" t="str">
+      <x:c r="A4" s="464" t="str">
         <x:v>Workflow</x:v>
       </x:c>
-      <x:c r="B4" s="89" t="str">
+      <x:c r="B4" s="465" t="str">
         <x:v>Old / current source</x:v>
       </x:c>
-      <x:c r="C4" s="89" t="str">
+      <x:c r="C4" s="465" t="str">
         <x:v>New canonical route</x:v>
       </x:c>
-      <x:c r="D4" s="89" t="str">
+      <x:c r="D4" s="465" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="E4" s="89" t="str">
+      <x:c r="E4" s="465" t="str">
         <x:v>What it does</x:v>
       </x:c>
-      <x:c r="F4" s="90" t="str">
+      <x:c r="F4" s="466" t="str">
         <x:v>Notes / next step</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="469" t="str">
         <x:v>Old production admin</x:v>
       </x:c>
-      <x:c r="B5" s="94" t="str">
+      <x:c r="B5" s="470" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="C5" s="94" t="str">
+      <x:c r="C5" s="470" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="D5" s="103" t="str">
+      <x:c r="D5" s="479" t="str">
         <x:v>Legacy active</x:v>
       </x:c>
-      <x:c r="E5" s="94" t="str">
+      <x:c r="E5" s="470" t="str">
         <x:v>Current live admin remains usable until /admindraft fully replaces it</x:v>
       </x:c>
-      <x:c r="F5" s="95" t="str">
+      <x:c r="F5" s="471" t="str">
         <x:v>Do not delete until every workflow is verified in /admindraft and /shelter</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A6" s="96" t="str">
+      <x:c r="A6" s="472" t="str">
         <x:v>PawJai umbrella dashboard</x:v>
       </x:c>
-      <x:c r="B6" s="97" t="str">
+      <x:c r="B6" s="473" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="C6" s="97" t="str">
+      <x:c r="C6" s="473" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D6" s="105" t="str">
+      <x:c r="D6" s="481" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E6" s="97" t="str">
+      <x:c r="E6" s="473" t="str">
         <x:v>PawJai HQ sees all shelters, dogs, bookings, ads, and about content</x:v>
       </x:c>
-      <x:c r="F6" s="98" t="str">
+      <x:c r="F6" s="474" t="str">
         <x:v>Keep as the admin umbrella; do not make shelter staff use this route</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="96" t="str">
+      <x:c r="A7" s="472" t="str">
         <x:v>Shelter login</x:v>
       </x:c>
-      <x:c r="B7" s="97" t="str">
+      <x:c r="B7" s="473" t="str">
         <x:v>not separated before</x:v>
       </x:c>
-      <x:c r="C7" s="97" t="str">
+      <x:c r="C7" s="473" t="str">
         <x:v>/shelter</x:v>
       </x:c>
-      <x:c r="D7" s="105" t="str">
+      <x:c r="D7" s="481" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E7" s="97" t="str">
+      <x:c r="E7" s="473" t="str">
         <x:v>Username/password login for partner shelters</x:v>
       </x:c>
-      <x:c r="F7" s="98" t="str">
+      <x:c r="F7" s="474" t="str">
         <x:v>Always redirect shelter users here when not signed in</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A8" s="96" t="str">
+      <x:c r="A8" s="472" t="str">
         <x:v>Shelter workspace</x:v>
       </x:c>
-      <x:c r="B8" s="97" t="str">
+      <x:c r="B8" s="473" t="str">
         <x:v>/admindraft view-as-shelter</x:v>
       </x:c>
-      <x:c r="C8" s="97" t="str">
+      <x:c r="C8" s="473" t="str">
         <x:v>/shelter/[slug]</x:v>
       </x:c>
-      <x:c r="D8" s="105" t="str">
+      <x:c r="D8" s="481" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E8" s="97" t="str">
+      <x:c r="E8" s="473" t="str">
         <x:v>Shelter-only workspace with profile, dog listings, create dog, bookings, messaging, account settings</x:v>
       </x:c>
-      <x:c r="F8" s="98" t="str">
+      <x:c r="F8" s="474" t="str">
         <x:v>Must never expose PawJai umbrella</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A9" s="96" t="str">
+      <x:c r="A9" s="472" t="str">
         <x:v>Shelter account settings</x:v>
       </x:c>
-      <x:c r="B9" s="97" t="str">
+      <x:c r="B9" s="473" t="str">
         <x:v>none</x:v>
       </x:c>
-      <x:c r="C9" s="97" t="str">
+      <x:c r="C9" s="473" t="str">
         <x:v>/shelter/[slug]/settings</x:v>
       </x:c>
-      <x:c r="D9" s="105" t="str">
+      <x:c r="D9" s="481" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E9" s="97" t="str">
+      <x:c r="E9" s="473" t="str">
         <x:v>Change shelter username, email, and password through real Supabase Auth + shelter_portal_accounts</x:v>
       </x:c>
-      <x:c r="F9" s="98" t="str">
+      <x:c r="F9" s="474" t="str">
         <x:v>Shared-login pilot only; later replace with employee accounts</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="96" t="str">
+      <x:c r="A10" s="472" t="str">
         <x:v>Dog listings inside shelter</x:v>
       </x:c>
-      <x:c r="B10" s="97" t="str">
+      <x:c r="B10" s="473" t="str">
         <x:v>/admindraft?view=dogs</x:v>
       </x:c>
-      <x:c r="C10" s="97" t="str">
+      <x:c r="C10" s="473" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
       </x:c>
-      <x:c r="D10" s="105" t="str">
+      <x:c r="D10" s="481" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E10" s="97" t="str">
+      <x:c r="E10" s="473" t="str">
         <x:v>Shelter can search and filter its own dogs</x:v>
       </x:c>
-      <x:c r="F10" s="98" t="str">
+      <x:c r="F10" s="474" t="str">
         <x:v>Open public dog profile is allowed to go to /dogs/[id]</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="96" t="str">
+      <x:c r="A11" s="472" t="str">
         <x:v>Create dog</x:v>
       </x:c>
-      <x:c r="B11" s="97" t="str">
+      <x:c r="B11" s="473" t="str">
         <x:v>/admindraft/dog-creation?shelter=:id</x:v>
       </x:c>
-      <x:c r="C11" s="97" t="str">
+      <x:c r="C11" s="473" t="str">
         <x:v>/shelter/[slug]/dogs/new</x:v>
       </x:c>
-      <x:c r="D11" s="105" t="str">
+      <x:c r="D11" s="481" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E11" s="97" t="str">
+      <x:c r="E11" s="473" t="str">
         <x:v>Reuses same live dog create form and buckets</x:v>
       </x:c>
-      <x:c r="F11" s="98" t="str">
+      <x:c r="F11" s="474" t="str">
         <x:v>Exit/success returns to /shelter/[slug]?view=dogs</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="96" t="str">
+      <x:c r="A12" s="472" t="str">
         <x:v>Edit dog</x:v>
       </x:c>
-      <x:c r="B12" s="97" t="str">
+      <x:c r="B12" s="473" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="C12" s="97" t="str">
+      <x:c r="C12" s="473" t="str">
         <x:v>/shelter/[slug]/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D12" s="105" t="str">
+      <x:c r="D12" s="481" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E12" s="97" t="str">
+      <x:c r="E12" s="473" t="str">
         <x:v>Reuses same live dog edit form, photos, traits, and storage</x:v>
       </x:c>
-      <x:c r="F12" s="98" t="str">
+      <x:c r="F12" s="474" t="str">
         <x:v>Dog must belong to logged-in shelter</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="96" t="str">
+      <x:c r="A13" s="472" t="str">
         <x:v>Public dog profile</x:v>
       </x:c>
-      <x:c r="B13" s="97" t="str">
+      <x:c r="B13" s="473" t="str">
         <x:v>/dogs/[id]</x:v>
       </x:c>
-      <x:c r="C13" s="97" t="str">
+      <x:c r="C13" s="473" t="str">
         <x:v>/dogs/[id]</x:v>
       </x:c>
-      <x:c r="D13" s="105" t="str">
+      <x:c r="D13" s="481" t="str">
         <x:v>Shared exception</x:v>
       </x:c>
-      <x:c r="E13" s="97" t="str">
+      <x:c r="E13" s="473" t="str">
         <x:v>Public adopter-facing profile</x:v>
       </x:c>
-      <x:c r="F13" s="98" t="str">
+      <x:c r="F13" s="474" t="str">
         <x:v>Only allowed cross-over from shelter portal to public UX</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="96" t="str">
+      <x:c r="A14" s="472" t="str">
         <x:v>Booking list</x:v>
       </x:c>
-      <x:c r="B14" s="97" t="str">
+      <x:c r="B14" s="473" t="str">
         <x:v>/admindraft?view=bookings</x:v>
       </x:c>
-      <x:c r="C14" s="97" t="str">
+      <x:c r="C14" s="473" t="str">
         <x:v>/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="D14" s="105" t="str">
+      <x:c r="D14" s="481" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E14" s="97" t="str">
+      <x:c r="E14" s="473" t="str">
         <x:v>Shelter booking list remains inside shelter workspace</x:v>
       </x:c>
-      <x:c r="F14" s="98" t="str">
+      <x:c r="F14" s="474" t="str">
         <x:v>Links open shared /booking detail with safe returnTo</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A15" s="96" t="str">
+      <x:c r="A15" s="472" t="str">
         <x:v>Booking detail</x:v>
       </x:c>
-      <x:c r="B15" s="97" t="str">
+      <x:c r="B15" s="473" t="str">
         <x:v>/admindraft/bookings/[id]</x:v>
       </x:c>
-      <x:c r="C15" s="97" t="str">
+      <x:c r="C15" s="473" t="str">
         <x:v>/booking/[id]</x:v>
       </x:c>
-      <x:c r="D15" s="105" t="str">
+      <x:c r="D15" s="481" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
-      <x:c r="E15" s="97" t="str">
+      <x:c r="E15" s="473" t="str">
         <x:v>Single internal booking detail page for PawJai admin and linked shelter</x:v>
       </x:c>
-      <x:c r="F15" s="98" t="str">
+      <x:c r="F15" s="474" t="str">
         <x:v>No new SQL table; reads same appointments/adopters/dogs/shelters</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="96" t="str">
+      <x:c r="A16" s="472" t="str">
         <x:v>Visitor profile / verification</x:v>
       </x:c>
-      <x:c r="B16" s="97" t="str">
+      <x:c r="B16" s="473" t="str">
         <x:v>/admindraft/bookings/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="C16" s="97" t="str">
+      <x:c r="C16" s="473" t="str">
         <x:v>/booking/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="D16" s="105" t="str">
+      <x:c r="D16" s="481" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
-      <x:c r="E16" s="97" t="str">
+      <x:c r="E16" s="473" t="str">
         <x:v>Single internal visitor profile and verification document page</x:v>
       </x:c>
-      <x:c r="F16" s="98" t="str">
+      <x:c r="F16" s="474" t="str">
         <x:v>Back links use safe returnTo</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="96" t="str">
+      <x:c r="A17" s="472" t="str">
         <x:v>QR check-in</x:v>
       </x:c>
-      <x:c r="B17" s="97" t="str">
+      <x:c r="B17" s="473" t="str">
         <x:v>/admindraft/bookings/check-in</x:v>
       </x:c>
-      <x:c r="C17" s="97" t="str">
+      <x:c r="C17" s="473" t="str">
         <x:v>/booking/check-in</x:v>
       </x:c>
-      <x:c r="D17" s="105" t="str">
+      <x:c r="D17" s="481" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
-      <x:c r="E17" s="97" t="str">
+      <x:c r="E17" s="473" t="str">
         <x:v>QR token resolves to shared booking detail</x:v>
       </x:c>
-      <x:c r="F17" s="98" t="str">
+      <x:c r="F17" s="474" t="str">
         <x:v>Generated QR URLs now use /booking/check-in</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="96" t="str">
+      <x:c r="A18" s="472" t="str">
         <x:v>Messaging</x:v>
       </x:c>
-      <x:c r="B18" s="97" t="str">
+      <x:c r="B18" s="473" t="str">
         <x:v>/admindraft shelter workspace</x:v>
       </x:c>
-      <x:c r="C18" s="97" t="str">
+      <x:c r="C18" s="473" t="str">
         <x:v>/shelter/[slug]?view=messages</x:v>
       </x:c>
-      <x:c r="D18" s="107" t="str">
+      <x:c r="D18" s="483" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E18" s="97" t="str">
+      <x:c r="E18" s="473" t="str">
         <x:v>Messaging is intentionally not completed in this session</x:v>
       </x:c>
-      <x:c r="F18" s="98" t="str">
+      <x:c r="F18" s="474" t="str">
         <x:v>Plan separately with API/provider choice</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="96" t="str">
+      <x:c r="A19" s="472" t="str">
         <x:v>Ads</x:v>
       </x:c>
-      <x:c r="B19" s="97" t="str">
+      <x:c r="B19" s="473" t="str">
         <x:v>/admin/ads</x:v>
       </x:c>
-      <x:c r="C19" s="97" t="str">
+      <x:c r="C19" s="473" t="str">
         <x:v>/admindraft &gt; Ads</x:v>
       </x:c>
-      <x:c r="D19" s="107" t="str">
+      <x:c r="D19" s="483" t="str">
         <x:v>Admin-only</x:v>
       </x:c>
-      <x:c r="E19" s="97" t="str">
+      <x:c r="E19" s="473" t="str">
         <x:v>PawJai-managed ads remain inside admin umbrella</x:v>
       </x:c>
-      <x:c r="F19" s="98" t="str">
+      <x:c r="F19" s="474" t="str">
         <x:v>No brand login yet</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="99" t="str">
+      <x:c r="A20" s="475" t="str">
         <x:v>About content</x:v>
       </x:c>
-      <x:c r="B20" s="100" t="str">
+      <x:c r="B20" s="476" t="str">
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
-      <x:c r="C20" s="100" t="str">
+      <x:c r="C20" s="476" t="str">
         <x:v>/admindraft &gt; About content</x:v>
       </x:c>
-      <x:c r="D20" s="109" t="str">
+      <x:c r="D20" s="485" t="str">
         <x:v>Admin-only</x:v>
       </x:c>
-      <x:c r="E20" s="100" t="str">
+      <x:c r="E20" s="476" t="str">
         <x:v>PawJai public content management</x:v>
       </x:c>
-      <x:c r="F20" s="101" t="str">
+      <x:c r="F20" s="477" t="str">
         <x:v>Not visible to shelters</x:v>
       </x:c>
     </x:row>
@@ -2290,283 +4012,303 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
-      <x:c r="A1" s="82" t="str">
+      <x:c r="A1" s="458" t="str">
         <x:v>PAWJAI Route Lane Connections</x:v>
       </x:c>
-      <x:c r="B1" s="82" t="str"/>
-      <x:c r="C1" s="82" t="str"/>
-      <x:c r="D1" s="82" t="str"/>
-      <x:c r="E1" s="82" t="str"/>
-      <x:c r="F1" s="82" t="str"/>
+      <x:c r="B1" s="458" t="str">
+        <x:v>PAWJAI Route Lane Connections</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>PAWJAI Route Lane Connections</x:v>
+      </x:c>
+      <x:c r="D1" s="458" t="str">
+        <x:v>PAWJAI Route Lane Connections</x:v>
+      </x:c>
+      <x:c r="E1" s="458" t="str">
+        <x:v>PAWJAI Route Lane Connections</x:v>
+      </x:c>
+      <x:c r="F1" s="458" t="str">
+        <x:v>PAWJAI Route Lane Connections</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="85" t="str">
+      <x:c r="A2" s="461" t="str">
         <x:v>Shows how admin, shelter, booking, and public dog-profile pages should connect without leaking shelter staff into PawJai admin.</x:v>
       </x:c>
-      <x:c r="B2" s="85" t="str"/>
-      <x:c r="C2" s="85" t="str"/>
-      <x:c r="D2" s="85" t="str"/>
-      <x:c r="E2" s="85" t="str"/>
-      <x:c r="F2" s="85" t="str"/>
+      <x:c r="B2" s="461" t="str">
+        <x:v>Shows how admin, shelter, booking, and public dog-profile pages should connect without leaking shelter staff into PawJai admin.</x:v>
+      </x:c>
+      <x:c r="C2" s="461" t="str">
+        <x:v>Shows how admin, shelter, booking, and public dog-profile pages should connect without leaking shelter staff into PawJai admin.</x:v>
+      </x:c>
+      <x:c r="D2" s="461" t="str">
+        <x:v>Shows how admin, shelter, booking, and public dog-profile pages should connect without leaking shelter staff into PawJai admin.</x:v>
+      </x:c>
+      <x:c r="E2" s="461" t="str">
+        <x:v>Shows how admin, shelter, booking, and public dog-profile pages should connect without leaking shelter staff into PawJai admin.</x:v>
+      </x:c>
+      <x:c r="F2" s="461" t="str">
+        <x:v>Shows how admin, shelter, booking, and public dog-profile pages should connect without leaking shelter staff into PawJai admin.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="88" t="str">
+      <x:c r="A4" s="464" t="str">
         <x:v>Scenario</x:v>
       </x:c>
-      <x:c r="B4" s="89" t="str">
+      <x:c r="B4" s="465" t="str">
         <x:v>Starts at</x:v>
       </x:c>
-      <x:c r="C4" s="89" t="str">
+      <x:c r="C4" s="465" t="str">
         <x:v>Deep route opened</x:v>
       </x:c>
-      <x:c r="D4" s="89" t="str">
+      <x:c r="D4" s="465" t="str">
         <x:v>Back / exit returns to</x:v>
       </x:c>
-      <x:c r="E4" s="89" t="str">
+      <x:c r="E4" s="465" t="str">
         <x:v>Safety status</x:v>
       </x:c>
-      <x:c r="F4" s="90" t="str">
+      <x:c r="F4" s="466" t="str">
         <x:v>Why it works</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="469" t="str">
         <x:v>PawJai admin opens booking</x:v>
       </x:c>
-      <x:c r="B5" s="94" t="str">
+      <x:c r="B5" s="470" t="str">
         <x:v>/admindraft?view=bookings</x:v>
       </x:c>
-      <x:c r="C5" s="94" t="str">
+      <x:c r="C5" s="470" t="str">
         <x:v>/booking/[id]?returnTo=/admindraft?view=bookings</x:v>
       </x:c>
-      <x:c r="D5" s="94" t="str">
+      <x:c r="D5" s="470" t="str">
         <x:v>/admindraft?view=bookings</x:v>
       </x:c>
-      <x:c r="E5" s="103" t="str">
+      <x:c r="E5" s="487" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F5" s="95" t="str">
+      <x:c r="F5" s="471" t="str">
         <x:v>Admin keeps umbrella context</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="96" t="str">
+      <x:c r="A6" s="472" t="str">
         <x:v>Old admin scans QR during migration</x:v>
       </x:c>
-      <x:c r="B6" s="97" t="str">
+      <x:c r="B6" s="473" t="str">
         <x:v>/admin/bookings</x:v>
       </x:c>
-      <x:c r="C6" s="97" t="str">
+      <x:c r="C6" s="473" t="str">
         <x:v>/booking/check-in?returnTo=/admin/bookings</x:v>
       </x:c>
-      <x:c r="D6" s="97" t="str">
+      <x:c r="D6" s="473" t="str">
         <x:v>/admin/bookings or /booking/[id]</x:v>
       </x:c>
-      <x:c r="E6" s="107" t="str">
+      <x:c r="E6" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F6" s="98" t="str">
+      <x:c r="F6" s="474" t="str">
         <x:v>Allowed for global admin only while old admin stays live</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="96" t="str">
+      <x:c r="A7" s="472" t="str">
         <x:v>Shelter opens booking</x:v>
       </x:c>
-      <x:c r="B7" s="97" t="str">
+      <x:c r="B7" s="473" t="str">
         <x:v>/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="C7" s="97" t="str">
+      <x:c r="C7" s="473" t="str">
         <x:v>/booking/[id]?returnTo=/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="D7" s="97" t="str">
+      <x:c r="D7" s="473" t="str">
         <x:v>/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="E7" s="107" t="str">
+      <x:c r="E7" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F7" s="98" t="str">
+      <x:c r="F7" s="474" t="str">
         <x:v>Shelter cannot leak into /admindraft</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="96" t="str">
+      <x:c r="A8" s="472" t="str">
         <x:v>PawJai admin opens visitor profile</x:v>
       </x:c>
-      <x:c r="B8" s="97" t="str">
+      <x:c r="B8" s="473" t="str">
         <x:v>/booking/[id]</x:v>
       </x:c>
-      <x:c r="C8" s="97" t="str">
+      <x:c r="C8" s="473" t="str">
         <x:v>/booking/[id]/visitor-profile?returnTo=/admindraft...</x:v>
       </x:c>
-      <x:c r="D8" s="97" t="str">
+      <x:c r="D8" s="473" t="str">
         <x:v>/booking/[id] or /admindraft...</x:v>
       </x:c>
-      <x:c r="E8" s="107" t="str">
+      <x:c r="E8" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F8" s="98" t="str">
+      <x:c r="F8" s="474" t="str">
         <x:v>Shared page preserves admin return path</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="96" t="str">
+      <x:c r="A9" s="472" t="str">
         <x:v>Shelter opens visitor profile</x:v>
       </x:c>
-      <x:c r="B9" s="97" t="str">
+      <x:c r="B9" s="473" t="str">
         <x:v>/booking/[id]</x:v>
       </x:c>
-      <x:c r="C9" s="97" t="str">
+      <x:c r="C9" s="473" t="str">
         <x:v>/booking/[id]/visitor-profile?returnTo=/shelter/[slug]...</x:v>
       </x:c>
-      <x:c r="D9" s="97" t="str">
+      <x:c r="D9" s="473" t="str">
         <x:v>/booking/[id] or /shelter/[slug]...</x:v>
       </x:c>
-      <x:c r="E9" s="107" t="str">
+      <x:c r="E9" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F9" s="98" t="str">
+      <x:c r="F9" s="474" t="str">
         <x:v>Shared page preserves shelter return path</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="96" t="str">
+      <x:c r="A10" s="472" t="str">
         <x:v>Shelter creates dog</x:v>
       </x:c>
-      <x:c r="B10" s="97" t="str">
+      <x:c r="B10" s="473" t="str">
         <x:v>/shelter/[slug]</x:v>
       </x:c>
-      <x:c r="C10" s="97" t="str">
+      <x:c r="C10" s="473" t="str">
         <x:v>/shelter/[slug]/dogs/new</x:v>
       </x:c>
-      <x:c r="D10" s="97" t="str">
+      <x:c r="D10" s="473" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
       </x:c>
-      <x:c r="E10" s="107" t="str">
+      <x:c r="E10" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F10" s="98" t="str">
+      <x:c r="F10" s="474" t="str">
         <x:v>Same create action, shelter-specific route shell</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="96" t="str">
+      <x:c r="A11" s="472" t="str">
         <x:v>Shelter edits dog</x:v>
       </x:c>
-      <x:c r="B11" s="97" t="str">
+      <x:c r="B11" s="473" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
       </x:c>
-      <x:c r="C11" s="97" t="str">
+      <x:c r="C11" s="473" t="str">
         <x:v>/shelter/[slug]/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D11" s="97" t="str">
+      <x:c r="D11" s="473" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
       </x:c>
-      <x:c r="E11" s="107" t="str">
+      <x:c r="E11" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F11" s="98" t="str">
+      <x:c r="F11" s="474" t="str">
         <x:v>Server checks dog.shelter_id before rendering</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="96" t="str">
+      <x:c r="A12" s="472" t="str">
         <x:v>PawJai admin edits dog</x:v>
       </x:c>
-      <x:c r="B12" s="97" t="str">
+      <x:c r="B12" s="473" t="str">
         <x:v>/admindraft?view=dogs</x:v>
       </x:c>
-      <x:c r="C12" s="97" t="str">
+      <x:c r="C12" s="473" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D12" s="97" t="str">
+      <x:c r="D12" s="473" t="str">
         <x:v>/admindraft?view=dogs</x:v>
       </x:c>
-      <x:c r="E12" s="107" t="str">
+      <x:c r="E12" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F12" s="98" t="str">
+      <x:c r="F12" s="474" t="str">
         <x:v>Admin keeps admin route context</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="96" t="str">
+      <x:c r="A13" s="472" t="str">
         <x:v>Shelter opens public dog profile</x:v>
       </x:c>
-      <x:c r="B13" s="97" t="str">
+      <x:c r="B13" s="473" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
       </x:c>
-      <x:c r="C13" s="97" t="str">
+      <x:c r="C13" s="473" t="str">
         <x:v>/dogs/[id]</x:v>
       </x:c>
-      <x:c r="D13" s="97" t="str">
+      <x:c r="D13" s="473" t="str">
         <x:v>Browser back or public page controls</x:v>
       </x:c>
-      <x:c r="E13" s="107" t="str">
+      <x:c r="E13" s="483" t="str">
         <x:v>Allowed exception</x:v>
       </x:c>
-      <x:c r="F13" s="98" t="str">
+      <x:c r="F13" s="474" t="str">
         <x:v>This is intentionally the adopter-facing dog profile</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="96" t="str">
+      <x:c r="A14" s="472" t="str">
         <x:v>QR scanner from shelter</x:v>
       </x:c>
-      <x:c r="B14" s="97" t="str">
+      <x:c r="B14" s="473" t="str">
         <x:v>/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="C14" s="97" t="str">
+      <x:c r="C14" s="473" t="str">
         <x:v>/booking/check-in?returnTo=/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="D14" s="97" t="str">
+      <x:c r="D14" s="473" t="str">
         <x:v>/booking/[id]?returnTo=/shelter/[slug]...</x:v>
       </x:c>
-      <x:c r="E14" s="107" t="str">
+      <x:c r="E14" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F14" s="98" t="str">
+      <x:c r="F14" s="474" t="str">
         <x:v>QR resolves into shared booking route</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="96" t="str">
+      <x:c r="A15" s="472" t="str">
         <x:v>Expired shelter session</x:v>
       </x:c>
-      <x:c r="B15" s="97" t="str">
+      <x:c r="B15" s="473" t="str">
         <x:v>any /shelter deep workflow</x:v>
       </x:c>
-      <x:c r="C15" s="97" t="str">
+      <x:c r="C15" s="473" t="str">
         <x:v>/shelter</x:v>
       </x:c>
-      <x:c r="D15" s="97" t="str">
+      <x:c r="D15" s="473" t="str">
         <x:v>/shelter</x:v>
       </x:c>
-      <x:c r="E15" s="107" t="str">
+      <x:c r="E15" s="481" t="str">
         <x:v>Safe</x:v>
       </x:c>
-      <x:c r="F15" s="98" t="str">
+      <x:c r="F15" s="474" t="str">
         <x:v>Shelter should log in through shelter portal, not admin login</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="99" t="str">
+      <x:c r="A16" s="475" t="str">
         <x:v>Unsafe edited returnTo</x:v>
       </x:c>
-      <x:c r="B16" s="100" t="str">
+      <x:c r="B16" s="476" t="str">
         <x:v>manually edited URL</x:v>
       </x:c>
-      <x:c r="C16" s="100" t="str">
+      <x:c r="C16" s="476" t="str">
         <x:v>shared booking route</x:v>
       </x:c>
-      <x:c r="D16" s="100" t="str">
+      <x:c r="D16" s="476" t="str">
         <x:v>role-based fallback</x:v>
       </x:c>
-      <x:c r="E16" s="109" t="str">
+      <x:c r="E16" s="489" t="str">
         <x:v>Guarded</x:v>
       </x:c>
-      <x:c r="F16" s="101" t="str">
+      <x:c r="F16" s="477" t="str">
         <x:v>External URLs and wrong-lane return paths are ignored</x:v>
       </x:c>
     </x:row>
@@ -2577,4 +4319,1601 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="458" t="str">
+        <x:v>PAWJAI Live Data Sync Diagram</x:v>
+      </x:c>
+      <x:c r="B1" s="458" t="str">
+        <x:v>PAWJAI Live Data Sync Diagram</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>PAWJAI Live Data Sync Diagram</x:v>
+      </x:c>
+      <x:c r="D1" s="458" t="str">
+        <x:v>PAWJAI Live Data Sync Diagram</x:v>
+      </x:c>
+      <x:c r="E1" s="458" t="str">
+        <x:v>PAWJAI Live Data Sync Diagram</x:v>
+      </x:c>
+      <x:c r="F1" s="458" t="str">
+        <x:v>PAWJAI Live Data Sync Diagram</x:v>
+      </x:c>
+      <x:c r="G1" s="458" t="str">
+        <x:v>PAWJAI Live Data Sync Diagram</x:v>
+      </x:c>
+      <x:c r="H1" s="458" t="str">
+        <x:v>PAWJAI Live Data Sync Diagram</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="461" t="str">
+        <x:v>Different route shells, same Supabase database, same storage bucket, same shared form/actions.</x:v>
+      </x:c>
+      <x:c r="B2" s="461" t="str">
+        <x:v>Different route shells, same Supabase database, same storage bucket, same shared form/actions.</x:v>
+      </x:c>
+      <x:c r="C2" s="461" t="str">
+        <x:v>Different route shells, same Supabase database, same storage bucket, same shared form/actions.</x:v>
+      </x:c>
+      <x:c r="D2" s="461" t="str">
+        <x:v>Different route shells, same Supabase database, same storage bucket, same shared form/actions.</x:v>
+      </x:c>
+      <x:c r="E2" s="461" t="str">
+        <x:v>Different route shells, same Supabase database, same storage bucket, same shared form/actions.</x:v>
+      </x:c>
+      <x:c r="F2" s="461" t="str">
+        <x:v>Different route shells, same Supabase database, same storage bucket, same shared form/actions.</x:v>
+      </x:c>
+      <x:c r="G2" s="461" t="str">
+        <x:v>Different route shells, same Supabase database, same storage bucket, same shared form/actions.</x:v>
+      </x:c>
+      <x:c r="H2" s="461" t="str">
+        <x:v>Different route shells, same Supabase database, same storage bucket, same shared form/actions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="464" t="str">
+        <x:v>Interface lane</x:v>
+      </x:c>
+      <x:c r="B4" s="465" t="str"/>
+      <x:c r="C4" s="465" t="str">
+        <x:v>Shared code</x:v>
+      </x:c>
+      <x:c r="D4" s="465" t="str"/>
+      <x:c r="E4" s="465" t="str">
+        <x:v>Live data layer</x:v>
+      </x:c>
+      <x:c r="F4" s="465" t="str"/>
+      <x:c r="G4" s="465" t="str">
+        <x:v>Updated surfaces</x:v>
+      </x:c>
+      <x:c r="H4" s="466" t="str">
+        <x:v>Sync rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="104" customHeight="1">
+      <x:c r="A5" s="493" t="str">
+        <x:v>Admin dog edit
+/admindraft/dogs/[id]/edit
+PawJai umbrella can edit any permitted shelter dog
+</x:v>
+      </x:c>
+      <x:c r="B5" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C5" s="499" t="str">
+        <x:v>DogEditForm
+updateDogProfileAction
+returnTo=/admindraft/dogs/[id]/edit
+</x:v>
+      </x:c>
+      <x:c r="D5" s="496" t="str">
+        <x:v>-&gt;
+reads/writes</x:v>
+      </x:c>
+      <x:c r="E5" s="503" t="str">
+        <x:v>Supabase tables
+dogs, dog_photos, dog_traits, shelters
+Storage bucket: dog-photos
+</x:v>
+      </x:c>
+      <x:c r="F5" s="496" t="str">
+        <x:v>-&gt;
+revalidates</x:v>
+      </x:c>
+      <x:c r="G5" s="507" t="str">
+        <x:v>/admindraft dog listings
+/shelter dog listings
+/dogs/[id] public profile
+</x:v>
+      </x:c>
+      <x:c r="H5" s="511" t="str">
+        <x:v>Same dog.id. No duplicate dog record. Navigation/refresh shows latest data on both sides.
+</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="104" customHeight="1">
+      <x:c r="A8" s="507" t="str">
+        <x:v>Shelter dog edit
+/shelter/[slug]/dogs/[id]/edit
+Shelter shell is scoped to that shelter only
+</x:v>
+      </x:c>
+      <x:c r="B8" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C8" s="499" t="str">
+        <x:v>DogEditForm
+updateDogProfileAction
+server checks dog.shelter_id before render
+</x:v>
+      </x:c>
+      <x:c r="D8" s="496" t="str">
+        <x:v>-&gt;
+reads/writes</x:v>
+      </x:c>
+      <x:c r="E8" s="503" t="str">
+        <x:v>Same Supabase rows and same media bucket as admin dog edit
+</x:v>
+      </x:c>
+      <x:c r="F8" s="496" t="str">
+        <x:v>-&gt;
+revalidates</x:v>
+      </x:c>
+      <x:c r="G8" s="507" t="str">
+        <x:v>/shelter/[slug]?view=dogs
+/admindraft?shelter=:id&amp;view=dogs
+/dogs/[id]
+</x:v>
+      </x:c>
+      <x:c r="H8" s="511" t="str">
+        <x:v>Editing here changes the same live PawJai listing that admin sees.
+</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="104" customHeight="1">
+      <x:c r="A11" s="515" t="str">
+        <x:v>Dog creation
+/admindraft/dog-creation?shelter=:id
+/shelter/[slug]/dogs/new
+</x:v>
+      </x:c>
+      <x:c r="B11" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C11" s="499" t="str">
+        <x:v>DogListingForm
+createDogProfileAction
+successListingsHref controls exit lane
+</x:v>
+      </x:c>
+      <x:c r="D11" s="496" t="str">
+        <x:v>-&gt;
+reads/writes</x:v>
+      </x:c>
+      <x:c r="E11" s="503" t="str">
+        <x:v>Creates dogs row
+Creates dog_photos rows
+Uploads to dog-photos bucket
+</x:v>
+      </x:c>
+      <x:c r="F11" s="496" t="str">
+        <x:v>-&gt;
+revalidates</x:v>
+      </x:c>
+      <x:c r="G11" s="507" t="str">
+        <x:v>Admin all dogs
+Shelter own dogs
+Public dog profile when available
+</x:v>
+      </x:c>
+      <x:c r="H11" s="511" t="str">
+        <x:v>Both create flows insert into the same production tables; route only changes who can choose shelter.
+</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="104" customHeight="1">
+      <x:c r="A14" s="519" t="str">
+        <x:v>Booking list and detail
+/admindraft?view=bookings
+/shelter/[slug]?view=bookings
+/booking/[id]
+</x:v>
+      </x:c>
+      <x:c r="B14" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C14" s="499" t="str">
+        <x:v>ShelterBookingsTab
+decideBookingAction
+checkInBookingAction
+safeBookingReturnTo
+</x:v>
+      </x:c>
+      <x:c r="D14" s="496" t="str">
+        <x:v>-&gt;
+reads/writes</x:v>
+      </x:c>
+      <x:c r="E14" s="503" t="str">
+        <x:v>appointments, adopters, dogs, shelters
+adopter_documents for verification view
+</x:v>
+      </x:c>
+      <x:c r="F14" s="496" t="str">
+        <x:v>-&gt;
+revalidates</x:v>
+      </x:c>
+      <x:c r="G14" s="507" t="str">
+        <x:v>Admin booking list
+Shelter booking list
+Shared /booking detail/profile
+</x:v>
+      </x:c>
+      <x:c r="H14" s="511" t="str">
+        <x:v>Single appointment record. Decisions and QR check-ins revalidate admin, shelter, shared booking, and adopter appointment views.
+</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="104" customHeight="1">
+      <x:c r="A17" s="523" t="str">
+        <x:v>Shelter profile/calendar
+/admindraft selected shelter
+/shelter/[slug]?view=profile
+</x:v>
+      </x:c>
+      <x:c r="B17" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C17" s="499" t="str">
+        <x:v>updateShelterProfileAction
+updateShelterOperatingDaysAction
+create/delete blockouts
+</x:v>
+      </x:c>
+      <x:c r="D17" s="496" t="str">
+        <x:v>-&gt;
+reads/writes</x:v>
+      </x:c>
+      <x:c r="E17" s="503" t="str">
+        <x:v>shelters
+shelter_regular_hours
+shelter_availability
+</x:v>
+      </x:c>
+      <x:c r="F17" s="496" t="str">
+        <x:v>-&gt;
+revalidates</x:v>
+      </x:c>
+      <x:c r="G17" s="507" t="str">
+        <x:v>Shelter profile card
+Booking availability
+Admin selected shelter profile
+</x:v>
+      </x:c>
+      <x:c r="H17" s="511" t="str">
+        <x:v>Same shelter.id; route-specific returnTo keeps staff out of PawJai admin lane.
+</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="526" t="str">
+        <x:v>See Architecture Advice sheet for the longer advisory: keep route shells separate, keep data/actions shared, and add Supabase Realtime later only if instant open-tab updates become important.</x:v>
+      </x:c>
+      <x:c r="B20" s="527" t="str">
+        <x:v>See Architecture Advice sheet for the longer advisory: keep route shells separate, keep data/actions shared, and add Supabase Realtime later only if instant open-tab updates become important.</x:v>
+      </x:c>
+      <x:c r="C20" s="527" t="str">
+        <x:v>See Architecture Advice sheet for the longer advisory: keep route shells separate, keep data/actions shared, and add Supabase Realtime later only if instant open-tab updates become important.</x:v>
+      </x:c>
+      <x:c r="D20" s="527" t="str">
+        <x:v>See Architecture Advice sheet for the longer advisory: keep route shells separate, keep data/actions shared, and add Supabase Realtime later only if instant open-tab updates become important.</x:v>
+      </x:c>
+      <x:c r="E20" s="527" t="str">
+        <x:v>See Architecture Advice sheet for the longer advisory: keep route shells separate, keep data/actions shared, and add Supabase Realtime later only if instant open-tab updates become important.</x:v>
+      </x:c>
+      <x:c r="F20" s="527" t="str">
+        <x:v>See Architecture Advice sheet for the longer advisory: keep route shells separate, keep data/actions shared, and add Supabase Realtime later only if instant open-tab updates become important.</x:v>
+      </x:c>
+      <x:c r="G20" s="527" t="str">
+        <x:v>See Architecture Advice sheet for the longer advisory: keep route shells separate, keep data/actions shared, and add Supabase Realtime later only if instant open-tab updates become important.</x:v>
+      </x:c>
+      <x:c r="H20" s="528" t="str">
+        <x:v>See Architecture Advice sheet for the longer advisory: keep route shells separate, keep data/actions shared, and add Supabase Realtime later only if instant open-tab updates become important.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+      <x:c r="G22"/>
+      <x:c r="H22"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A20:H20"/>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="458" t="str">
+        <x:v>PAWJAI Route Flow and Lane Separation</x:v>
+      </x:c>
+      <x:c r="B1" s="458" t="str">
+        <x:v>PAWJAI Route Flow and Lane Separation</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>PAWJAI Route Flow and Lane Separation</x:v>
+      </x:c>
+      <x:c r="D1" s="458" t="str">
+        <x:v>PAWJAI Route Flow and Lane Separation</x:v>
+      </x:c>
+      <x:c r="E1" s="458" t="str">
+        <x:v>PAWJAI Route Flow and Lane Separation</x:v>
+      </x:c>
+      <x:c r="F1" s="458" t="str">
+        <x:v>PAWJAI Route Flow and Lane Separation</x:v>
+      </x:c>
+      <x:c r="G1" s="458" t="str">
+        <x:v>PAWJAI Route Flow and Lane Separation</x:v>
+      </x:c>
+      <x:c r="H1" s="458" t="str">
+        <x:v>PAWJAI Route Flow and Lane Separation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="461" t="str">
+        <x:v>Deep pages can be shared only when the return path is validated. Shelter staff should never land in the PawJai admin umbrella.</x:v>
+      </x:c>
+      <x:c r="B2" s="461" t="str">
+        <x:v>Deep pages can be shared only when the return path is validated. Shelter staff should never land in the PawJai admin umbrella.</x:v>
+      </x:c>
+      <x:c r="C2" s="461" t="str">
+        <x:v>Deep pages can be shared only when the return path is validated. Shelter staff should never land in the PawJai admin umbrella.</x:v>
+      </x:c>
+      <x:c r="D2" s="461" t="str">
+        <x:v>Deep pages can be shared only when the return path is validated. Shelter staff should never land in the PawJai admin umbrella.</x:v>
+      </x:c>
+      <x:c r="E2" s="461" t="str">
+        <x:v>Deep pages can be shared only when the return path is validated. Shelter staff should never land in the PawJai admin umbrella.</x:v>
+      </x:c>
+      <x:c r="F2" s="461" t="str">
+        <x:v>Deep pages can be shared only when the return path is validated. Shelter staff should never land in the PawJai admin umbrella.</x:v>
+      </x:c>
+      <x:c r="G2" s="461" t="str">
+        <x:v>Deep pages can be shared only when the return path is validated. Shelter staff should never land in the PawJai admin umbrella.</x:v>
+      </x:c>
+      <x:c r="H2" s="461" t="str">
+        <x:v>Deep pages can be shared only when the return path is validated. Shelter staff should never land in the PawJai admin umbrella.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="464" t="str">
+        <x:v>Lane start</x:v>
+      </x:c>
+      <x:c r="B4" s="465" t="str"/>
+      <x:c r="C4" s="465" t="str">
+        <x:v>Workspace list</x:v>
+      </x:c>
+      <x:c r="D4" s="465" t="str"/>
+      <x:c r="E4" s="465" t="str">
+        <x:v>Deep workflow</x:v>
+      </x:c>
+      <x:c r="F4" s="465" t="str"/>
+      <x:c r="G4" s="465" t="str">
+        <x:v>Back/exit</x:v>
+      </x:c>
+      <x:c r="H4" s="466" t="str">
+        <x:v>Guardrail</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="104" customHeight="1">
+      <x:c r="A5" s="493" t="str">
+        <x:v>PawJai admin
+/admindraft
+phrase gate
+</x:v>
+      </x:c>
+      <x:c r="B5" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C5" s="499" t="str">
+        <x:v>/admindraft?shelter=:id&amp;view=dogs
+/admindraft?view=bookings
+</x:v>
+      </x:c>
+      <x:c r="D5" s="496" t="str">
+        <x:v>-&gt;
+opens</x:v>
+      </x:c>
+      <x:c r="E5" s="503" t="str">
+        <x:v>/admindraft/dogs/[id]/edit
+/booking/[id]?returnTo=/admindraft...
+</x:v>
+      </x:c>
+      <x:c r="F5" s="496" t="str">
+        <x:v>-&gt;
+returns</x:v>
+      </x:c>
+      <x:c r="G5" s="507" t="str">
+        <x:v>/admindraft?shelter=:id&amp;view=dogs
+/admindraft?view=bookings
+</x:v>
+      </x:c>
+      <x:c r="H5" s="511" t="str">
+        <x:v>Admin can see umbrella; booking returnTo accepts /admindraft for global admin.
+</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="104" customHeight="1">
+      <x:c r="A9" s="507" t="str">
+        <x:v>Shelter staff
+/shelter login
+Supabase account
+</x:v>
+      </x:c>
+      <x:c r="B9" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C9" s="499" t="str">
+        <x:v>/shelter/[slug]?view=profile
+/shelter/[slug]?view=dogs
+/shelter/[slug]?view=bookings
+</x:v>
+      </x:c>
+      <x:c r="D9" s="496" t="str">
+        <x:v>-&gt;
+opens</x:v>
+      </x:c>
+      <x:c r="E9" s="503" t="str">
+        <x:v>/shelter/[slug]/dogs/[id]/edit
+/booking/[id]?returnTo=/shelter/[slug]...
+</x:v>
+      </x:c>
+      <x:c r="F9" s="496" t="str">
+        <x:v>-&gt;
+returns</x:v>
+      </x:c>
+      <x:c r="G9" s="507" t="str">
+        <x:v>/shelter/[slug]?view=dogs
+/shelter/[slug]?view=bookings
+</x:v>
+      </x:c>
+      <x:c r="H9" s="511" t="str">
+        <x:v>Server checks shelter membership and dog.shelter_id. Wrong-lane returnTo falls back to shelter portal.
+</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="104" customHeight="1">
+      <x:c r="A13" s="515" t="str">
+        <x:v>Shared booking route
+/booking/[id]
+/booking/[id]/visitor-profile
+</x:v>
+      </x:c>
+      <x:c r="B13" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C13" s="499" t="str">
+        <x:v>Opened from admin or shelter list
+</x:v>
+      </x:c>
+      <x:c r="D13" s="496" t="str">
+        <x:v>-&gt;
+opens</x:v>
+      </x:c>
+      <x:c r="E13" s="503" t="str">
+        <x:v>safeBookingReturnTo(requestedReturnTo)
+canAccessShelter(context, shelter_id)
+</x:v>
+      </x:c>
+      <x:c r="F13" s="496" t="str">
+        <x:v>-&gt;
+returns</x:v>
+      </x:c>
+      <x:c r="G13" s="507" t="str">
+        <x:v>Returns to allowed /admindraft or /shelter path only
+</x:v>
+      </x:c>
+      <x:c r="H13" s="511" t="str">
+        <x:v>External URLs, // paths, and wrong role/lane return paths are ignored.
+</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="104" customHeight="1">
+      <x:c r="A17" s="523" t="str">
+        <x:v>Public dog profile exception
+</x:v>
+      </x:c>
+      <x:c r="B17" s="496" t="str">
+        <x:v>-&gt;
+flows to</x:v>
+      </x:c>
+      <x:c r="C17" s="499" t="str">
+        <x:v>/shelter/[slug]?view=dogs
+/admindraft?view=dogs
+</x:v>
+      </x:c>
+      <x:c r="D17" s="496" t="str">
+        <x:v>-&gt;
+opens</x:v>
+      </x:c>
+      <x:c r="E17" s="503" t="str">
+        <x:v>/dogs/[id]
+</x:v>
+      </x:c>
+      <x:c r="F17" s="496" t="str">
+        <x:v>-&gt;
+returns</x:v>
+      </x:c>
+      <x:c r="G17" s="507" t="str">
+        <x:v>Browser back or public navigation
+</x:v>
+      </x:c>
+      <x:c r="H17" s="511" t="str">
+        <x:v>This is the one intentional crossover into adopter-facing UX.
+</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="54" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="54" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="46" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="458" t="str">
+        <x:v>PAWJAI Back Behavior Matrix</x:v>
+      </x:c>
+      <x:c r="B1" s="458" t="str">
+        <x:v>PAWJAI Back Behavior Matrix</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>PAWJAI Back Behavior Matrix</x:v>
+      </x:c>
+      <x:c r="D1" s="458" t="str">
+        <x:v>PAWJAI Back Behavior Matrix</x:v>
+      </x:c>
+      <x:c r="E1" s="458" t="str">
+        <x:v>PAWJAI Back Behavior Matrix</x:v>
+      </x:c>
+      <x:c r="F1" s="458" t="str">
+        <x:v>PAWJAI Back Behavior Matrix</x:v>
+      </x:c>
+      <x:c r="G1" s="458" t="str">
+        <x:v>PAWJAI Back Behavior Matrix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="461" t="str">
+        <x:v>Documents the two back types: browser history is uncontrolled history, while app back/exit links and returnTo are controlled lane-aware behavior.</x:v>
+      </x:c>
+      <x:c r="B2" s="461" t="str">
+        <x:v>Documents the two back types: browser history is uncontrolled history, while app back/exit links and returnTo are controlled lane-aware behavior.</x:v>
+      </x:c>
+      <x:c r="C2" s="461" t="str">
+        <x:v>Documents the two back types: browser history is uncontrolled history, while app back/exit links and returnTo are controlled lane-aware behavior.</x:v>
+      </x:c>
+      <x:c r="D2" s="461" t="str">
+        <x:v>Documents the two back types: browser history is uncontrolled history, while app back/exit links and returnTo are controlled lane-aware behavior.</x:v>
+      </x:c>
+      <x:c r="E2" s="461" t="str">
+        <x:v>Documents the two back types: browser history is uncontrolled history, while app back/exit links and returnTo are controlled lane-aware behavior.</x:v>
+      </x:c>
+      <x:c r="F2" s="461" t="str">
+        <x:v>Documents the two back types: browser history is uncontrolled history, while app back/exit links and returnTo are controlled lane-aware behavior.</x:v>
+      </x:c>
+      <x:c r="G2" s="461" t="str">
+        <x:v>Documents the two back types: browser history is uncontrolled history, while app back/exit links and returnTo are controlled lane-aware behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="464" t="str">
+        <x:v>Back type</x:v>
+      </x:c>
+      <x:c r="B4" s="465" t="str">
+        <x:v>Trigger</x:v>
+      </x:c>
+      <x:c r="C4" s="465" t="str">
+        <x:v>Used from</x:v>
+      </x:c>
+      <x:c r="D4" s="465" t="str">
+        <x:v>How it behaves</x:v>
+      </x:c>
+      <x:c r="E4" s="465" t="str">
+        <x:v>Risk / guardrail</x:v>
+      </x:c>
+      <x:c r="F4" s="465" t="str">
+        <x:v>Recommendation</x:v>
+      </x:c>
+      <x:c r="G4" s="466" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="469" t="str">
+        <x:v>Browser back</x:v>
+      </x:c>
+      <x:c r="B5" s="470" t="str">
+        <x:v>Browser toolbar / trackpad / keyboard</x:v>
+      </x:c>
+      <x:c r="C5" s="470" t="str">
+        <x:v>Any page</x:v>
+      </x:c>
+      <x:c r="D5" s="470" t="str">
+        <x:v>Uses browser history exactly as the browser recorded it</x:v>
+      </x:c>
+      <x:c r="E5" s="470" t="str">
+        <x:v>Auth guards still protect restricted routes, but browser history can feel confusing if the user arrived from a different lane.</x:v>
+      </x:c>
+      <x:c r="F5" s="470" t="str">
+        <x:v>Use as fallback only; do not rely on it for shelter staff training.</x:v>
+      </x:c>
+      <x:c r="G5" s="530" t="str">
+        <x:v>Manual / watch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="472" t="str">
+        <x:v>App Back / Exit link</x:v>
+      </x:c>
+      <x:c r="B6" s="473" t="str">
+        <x:v>Visible Back, Exit, Booking list, Dog listings buttons</x:v>
+      </x:c>
+      <x:c r="C6" s="473" t="str">
+        <x:v>/shelter/[slug]/dogs/[id]/edit, /admindraft/dogs/[id]/edit, /booking/[id]</x:v>
+      </x:c>
+      <x:c r="D6" s="473" t="str">
+        <x:v>Hard-coded route for that lane: /shelter/[slug]?view=dogs, /admindraft?... or bookingListHref</x:v>
+      </x:c>
+      <x:c r="E6" s="473" t="str">
+        <x:v>Deterministic and role-aware. Best UX for shelter staff.</x:v>
+      </x:c>
+      <x:c r="F6" s="473" t="str">
+        <x:v>Primary path for training and QA.</x:v>
+      </x:c>
+      <x:c r="G6" s="532" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="472" t="str">
+        <x:v>Form returnTo</x:v>
+      </x:c>
+      <x:c r="B7" s="473" t="str">
+        <x:v>Hidden form input submitted with save/delete/profile/calendar forms</x:v>
+      </x:c>
+      <x:c r="C7" s="473" t="str">
+        <x:v>Dog create/edit, shelter profile, calendar, booking decisions</x:v>
+      </x:c>
+      <x:c r="D7" s="473" t="str">
+        <x:v>Server action redirects to returnTo only when it starts with allowed prefixes.</x:v>
+      </x:c>
+      <x:c r="E7" s="473" t="str">
+        <x:v>Keeps saved workflows inside the same lane after mutation.</x:v>
+      </x:c>
+      <x:c r="F7" s="473" t="str">
+        <x:v>Keep adding returnTo whenever a form is reused across admin/shelter.</x:v>
+      </x:c>
+      <x:c r="G7" s="532" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="472" t="str">
+        <x:v>Shared booking returnTo</x:v>
+      </x:c>
+      <x:c r="B8" s="473" t="str">
+        <x:v>Query param on /booking routes</x:v>
+      </x:c>
+      <x:c r="C8" s="473" t="str">
+        <x:v>/booking/[id], /booking/[id]/visitor-profile</x:v>
+      </x:c>
+      <x:c r="D8" s="473" t="str">
+        <x:v>safeBookingReturnTo validates /admindraft for global admin, /shelter/[slug] for shelter admin, /admin/bookings for legacy admin only.</x:v>
+      </x:c>
+      <x:c r="E8" s="473" t="str">
+        <x:v>Blocks wrong-lane or external return URLs.</x:v>
+      </x:c>
+      <x:c r="F8" s="473" t="str">
+        <x:v>This is the core fix for booking deep-page leaks.</x:v>
+      </x:c>
+      <x:c r="G8" s="532" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="472" t="str">
+        <x:v>QR check-in return</x:v>
+      </x:c>
+      <x:c r="B9" s="473" t="str">
+        <x:v>QR scanner link includes returnTo</x:v>
+      </x:c>
+      <x:c r="C9" s="473" t="str">
+        <x:v>/booking/check-in</x:v>
+      </x:c>
+      <x:c r="D9" s="473" t="str">
+        <x:v>Valid token redirects to /booking/[id]?token=...&amp;returnTo=...; invalid token shows card with Back to booking list.</x:v>
+      </x:c>
+      <x:c r="E9" s="473" t="str">
+        <x:v>Shelter session expires to /shelter; admin can return to admin lane.</x:v>
+      </x:c>
+      <x:c r="F9" s="473" t="str">
+        <x:v>Smoke test on a real phone before shelter pilot.</x:v>
+      </x:c>
+      <x:c r="G9" s="534" t="str">
+        <x:v>Manual / watch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="472" t="str">
+        <x:v>Public dog profile exception</x:v>
+      </x:c>
+      <x:c r="B10" s="473" t="str">
+        <x:v>Open public profile button</x:v>
+      </x:c>
+      <x:c r="C10" s="473" t="str">
+        <x:v>/dogs/[id]</x:v>
+      </x:c>
+      <x:c r="D10" s="473" t="str">
+        <x:v>No internal returnTo; use browser back/public navigation.</x:v>
+      </x:c>
+      <x:c r="E10" s="473" t="str">
+        <x:v>This is intentionally adopter-facing and public.</x:v>
+      </x:c>
+      <x:c r="F10" s="473" t="str">
+        <x:v>Only exception where shelter portal may leave private UI.</x:v>
+      </x:c>
+      <x:c r="G10" s="536" t="str">
+        <x:v>Allowed exception</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="472" t="str">
+        <x:v>Expired shelter session</x:v>
+      </x:c>
+      <x:c r="B11" s="473" t="str">
+        <x:v>User opens deep shelter/booking route after logout</x:v>
+      </x:c>
+      <x:c r="C11" s="473" t="str">
+        <x:v>/shelter/[slug]/..., /booking/[id]</x:v>
+      </x:c>
+      <x:c r="D11" s="473" t="str">
+        <x:v>Redirects to /shelter login or role fallback.</x:v>
+      </x:c>
+      <x:c r="E11" s="473" t="str">
+        <x:v>Should not show PawJai admin login to shelter staff.</x:v>
+      </x:c>
+      <x:c r="F11" s="473" t="str">
+        <x:v>Test in incognito before pilot.</x:v>
+      </x:c>
+      <x:c r="G11" s="534" t="str">
+        <x:v>Manual / watch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="475" t="str">
+        <x:v>Unsafe returnTo edit</x:v>
+      </x:c>
+      <x:c r="B12" s="476" t="str">
+        <x:v>User manually edits returnTo URL</x:v>
+      </x:c>
+      <x:c r="C12" s="476" t="str">
+        <x:v>/booking/[id]?returnTo=...</x:v>
+      </x:c>
+      <x:c r="D12" s="476" t="str">
+        <x:v>External URLs, // paths, and wrong-lane paths are ignored; fallback is role-based.</x:v>
+      </x:c>
+      <x:c r="E12" s="476" t="str">
+        <x:v>Prevents shelter staff from being bounced into admin umbrella.</x:v>
+      </x:c>
+      <x:c r="F12" s="476" t="str">
+        <x:v>Keep this pattern for future shared routes.</x:v>
+      </x:c>
+      <x:c r="G12" s="538" t="str">
+        <x:v>Guarded</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="46" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="458" t="str">
+        <x:v>PAWJAI Machine-Readable Route and Data Spec</x:v>
+      </x:c>
+      <x:c r="B1" s="458" t="str">
+        <x:v>PAWJAI Machine-Readable Route and Data Spec</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>PAWJAI Machine-Readable Route and Data Spec</x:v>
+      </x:c>
+      <x:c r="D1" s="458" t="str">
+        <x:v>PAWJAI Machine-Readable Route and Data Spec</x:v>
+      </x:c>
+      <x:c r="E1" s="458" t="str">
+        <x:v>PAWJAI Machine-Readable Route and Data Spec</x:v>
+      </x:c>
+      <x:c r="F1" s="458" t="str">
+        <x:v>PAWJAI Machine-Readable Route and Data Spec</x:v>
+      </x:c>
+      <x:c r="G1" s="458" t="str">
+        <x:v>PAWJAI Machine-Readable Route and Data Spec</x:v>
+      </x:c>
+      <x:c r="H1" s="458" t="str">
+        <x:v>PAWJAI Machine-Readable Route and Data Spec</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="461" t="str">
+        <x:v>Future Codex sessions should read this sheet to understand exact source files, route shells, shared actions, tables, buckets, and guardrails.</x:v>
+      </x:c>
+      <x:c r="B2" s="461" t="str">
+        <x:v>Future Codex sessions should read this sheet to understand exact source files, route shells, shared actions, tables, buckets, and guardrails.</x:v>
+      </x:c>
+      <x:c r="C2" s="461" t="str">
+        <x:v>Future Codex sessions should read this sheet to understand exact source files, route shells, shared actions, tables, buckets, and guardrails.</x:v>
+      </x:c>
+      <x:c r="D2" s="461" t="str">
+        <x:v>Future Codex sessions should read this sheet to understand exact source files, route shells, shared actions, tables, buckets, and guardrails.</x:v>
+      </x:c>
+      <x:c r="E2" s="461" t="str">
+        <x:v>Future Codex sessions should read this sheet to understand exact source files, route shells, shared actions, tables, buckets, and guardrails.</x:v>
+      </x:c>
+      <x:c r="F2" s="461" t="str">
+        <x:v>Future Codex sessions should read this sheet to understand exact source files, route shells, shared actions, tables, buckets, and guardrails.</x:v>
+      </x:c>
+      <x:c r="G2" s="461" t="str">
+        <x:v>Future Codex sessions should read this sheet to understand exact source files, route shells, shared actions, tables, buckets, and guardrails.</x:v>
+      </x:c>
+      <x:c r="H2" s="461" t="str">
+        <x:v>Future Codex sessions should read this sheet to understand exact source files, route shells, shared actions, tables, buckets, and guardrails.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="464" t="str">
+        <x:v>System area</x:v>
+      </x:c>
+      <x:c r="B4" s="465" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="C4" s="465" t="str">
+        <x:v>Source route / file</x:v>
+      </x:c>
+      <x:c r="D4" s="465" t="str">
+        <x:v>Reads</x:v>
+      </x:c>
+      <x:c r="E4" s="465" t="str">
+        <x:v>Writes / shared action</x:v>
+      </x:c>
+      <x:c r="F4" s="465" t="str">
+        <x:v>Return / back behavior</x:v>
+      </x:c>
+      <x:c r="G4" s="465" t="str">
+        <x:v>Guard</x:v>
+      </x:c>
+      <x:c r="H4" s="466" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="469" t="str">
+        <x:v>Dog edit - admin shell</x:v>
+      </x:c>
+      <x:c r="B5" s="470" t="str">
+        <x:v>Route shell</x:v>
+      </x:c>
+      <x:c r="C5" s="470" t="str">
+        <x:v>app/admindraft/dogs/[id]/edit/page.tsx</x:v>
+      </x:c>
+      <x:c r="D5" s="470" t="str">
+        <x:v>dogs, dog_photos, dog_traits, shelters</x:v>
+      </x:c>
+      <x:c r="E5" s="470" t="str">
+        <x:v>DogEditForm -&gt; updateDogProfileAction</x:v>
+      </x:c>
+      <x:c r="F5" s="470" t="str">
+        <x:v>returnTo=/admindraft/dogs/[id]/edit; deleteReturnTo=/admindraft?shelter=:id&amp;view=dogs</x:v>
+      </x:c>
+      <x:c r="G5" s="470" t="str">
+        <x:v>isAdminDraftUnlocked + requireShelterAccess(dog.shelter_id)</x:v>
+      </x:c>
+      <x:c r="H5" s="471" t="str">
+        <x:v>PawJai umbrella interface; same live dog row</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="472" t="str">
+        <x:v>Dog edit - shelter shell</x:v>
+      </x:c>
+      <x:c r="B6" s="473" t="str">
+        <x:v>Route shell</x:v>
+      </x:c>
+      <x:c r="C6" s="473" t="str">
+        <x:v>app/shelter/[slug]/dogs/[id]/edit/page.tsx</x:v>
+      </x:c>
+      <x:c r="D6" s="473" t="str">
+        <x:v>dogs, dog_photos, dog_traits, shelters</x:v>
+      </x:c>
+      <x:c r="E6" s="473" t="str">
+        <x:v>DogEditForm -&gt; updateDogProfileAction</x:v>
+      </x:c>
+      <x:c r="F6" s="473" t="str">
+        <x:v>returnTo=/shelter/[slug]/dogs/[id]/edit; deleteReturnTo=/shelter/[slug]?view=dogs</x:v>
+      </x:c>
+      <x:c r="G6" s="473" t="str">
+        <x:v>getAdminAuthContext(includePhraseGate:false) + dog.shelter_id === shelter.id</x:v>
+      </x:c>
+      <x:c r="H6" s="474" t="str">
+        <x:v>Shelter-only interface; same live dog row</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="472" t="str">
+        <x:v>Dog create - admin</x:v>
+      </x:c>
+      <x:c r="B7" s="473" t="str">
+        <x:v>Route shell</x:v>
+      </x:c>
+      <x:c r="C7" s="473" t="str">
+        <x:v>app/admindraft/dog-creation + app/admindraft/dogs/new/page.tsx</x:v>
+      </x:c>
+      <x:c r="D7" s="473" t="str">
+        <x:v>shelters, dog_traits</x:v>
+      </x:c>
+      <x:c r="E7" s="473" t="str">
+        <x:v>DogListingForm -&gt; createDogProfileAction</x:v>
+      </x:c>
+      <x:c r="F7" s="473" t="str">
+        <x:v>successListingsHref=/admindraft?shelter=:id&amp;view=dogs</x:v>
+      </x:c>
+      <x:c r="G7" s="473" t="str">
+        <x:v>isAdminDraftUnlocked + requireShelterAccess(selected shelter)</x:v>
+      </x:c>
+      <x:c r="H7" s="474" t="str">
+        <x:v>Admin can choose shelter</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="472" t="str">
+        <x:v>Dog create - shelter</x:v>
+      </x:c>
+      <x:c r="B8" s="473" t="str">
+        <x:v>Route shell</x:v>
+      </x:c>
+      <x:c r="C8" s="473" t="str">
+        <x:v>app/shelter/[slug]/dogs/new/page.tsx</x:v>
+      </x:c>
+      <x:c r="D8" s="473" t="str">
+        <x:v>shelters scoped to logged-in shelter, dog_traits</x:v>
+      </x:c>
+      <x:c r="E8" s="473" t="str">
+        <x:v>DogListingForm -&gt; createDogProfileAction</x:v>
+      </x:c>
+      <x:c r="F8" s="473" t="str">
+        <x:v>successListingsHref=/shelter/[slug]?view=dogs</x:v>
+      </x:c>
+      <x:c r="G8" s="473" t="str">
+        <x:v>getShelterByPortalSlug + shelter membership</x:v>
+      </x:c>
+      <x:c r="H8" s="474" t="str">
+        <x:v>Shelter cannot choose other shelters</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="472" t="str">
+        <x:v>Dog create/edit action</x:v>
+      </x:c>
+      <x:c r="B9" s="473" t="str">
+        <x:v>Server action</x:v>
+      </x:c>
+      <x:c r="C9" s="473" t="str">
+        <x:v>app/admin/dogs/new/actions.ts + app/admin/dogs/[id]/edit/actions.ts</x:v>
+      </x:c>
+      <x:c r="D9" s="473" t="str">
+        <x:v>dogs, dog_photos, dog_traits, appointments</x:v>
+      </x:c>
+      <x:c r="E9" s="473" t="str">
+        <x:v>insert/update/delete rows; upload/remove dog-photos storage</x:v>
+      </x:c>
+      <x:c r="F9" s="473" t="str">
+        <x:v>Accepts /admindraft and /shelter returnTo prefixes</x:v>
+      </x:c>
+      <x:c r="G9" s="473" t="str">
+        <x:v>requireShelterAccess(shelter_id)</x:v>
+      </x:c>
+      <x:c r="H9" s="474" t="str">
+        <x:v>Shared action is why both route shells sync</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="472" t="str">
+        <x:v>Admin/shelter listings</x:v>
+      </x:c>
+      <x:c r="B10" s="473" t="str">
+        <x:v>Data loader</x:v>
+      </x:c>
+      <x:c r="C10" s="473" t="str">
+        <x:v>utils/admin-draft-data.ts:loadAdminDraftData</x:v>
+      </x:c>
+      <x:c r="D10" s="473" t="str">
+        <x:v>dogs, dog_photos, appointments, shelters, ads, pawjai_profile</x:v>
+      </x:c>
+      <x:c r="E10" s="473" t="str">
+        <x:v>Read-only load for panel</x:v>
+      </x:c>
+      <x:c r="F10" s="473" t="str">
+        <x:v>Panel routes decide edit/create/detail links</x:v>
+      </x:c>
+      <x:c r="G10" s="473" t="str">
+        <x:v>Optional shelterIds scopes shelter portal</x:v>
+      </x:c>
+      <x:c r="H10" s="474" t="str">
+        <x:v>Same loader powers umbrella and shelter subset</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="472" t="str">
+        <x:v>Booking detail</x:v>
+      </x:c>
+      <x:c r="B11" s="473" t="str">
+        <x:v>Shared route</x:v>
+      </x:c>
+      <x:c r="C11" s="473" t="str">
+        <x:v>app/booking/[id]/page.tsx</x:v>
+      </x:c>
+      <x:c r="D11" s="473" t="str">
+        <x:v>appointments, adopters, dogs, shelters</x:v>
+      </x:c>
+      <x:c r="E11" s="473" t="str">
+        <x:v>decideBookingAction, checkInBookingAction</x:v>
+      </x:c>
+      <x:c r="F11" s="473" t="str">
+        <x:v>safeBookingReturnTo</x:v>
+      </x:c>
+      <x:c r="G11" s="473" t="str">
+        <x:v>getAdminAuthContext + canAccessShelter</x:v>
+      </x:c>
+      <x:c r="H11" s="474" t="str">
+        <x:v>No duplicate booking page/data table needed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="472" t="str">
+        <x:v>Visitor profile</x:v>
+      </x:c>
+      <x:c r="B12" s="473" t="str">
+        <x:v>Shared route</x:v>
+      </x:c>
+      <x:c r="C12" s="473" t="str">
+        <x:v>app/booking/[id]/visitor-profile/page.tsx</x:v>
+      </x:c>
+      <x:c r="D12" s="473" t="str">
+        <x:v>appointments, adopters, adopter_documents, adopter_profiles, adopter_preferences, dogs, shelters</x:v>
+      </x:c>
+      <x:c r="E12" s="473" t="str">
+        <x:v>Read profile/verification documents</x:v>
+      </x:c>
+      <x:c r="F12" s="473" t="str">
+        <x:v>Back to booking detail/list uses safe returnTo</x:v>
+      </x:c>
+      <x:c r="G12" s="473" t="str">
+        <x:v>getAdminAuthContext + canAccessShelter</x:v>
+      </x:c>
+      <x:c r="H12" s="474" t="str">
+        <x:v>Shared internal verification view</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A13" s="472" t="str">
+        <x:v>QR check-in</x:v>
+      </x:c>
+      <x:c r="B13" s="473" t="str">
+        <x:v>Shared route</x:v>
+      </x:c>
+      <x:c r="C13" s="473" t="str">
+        <x:v>app/booking/check-in/page.tsx + utils/booking.ts:buildCheckInUrl</x:v>
+      </x:c>
+      <x:c r="D13" s="473" t="str">
+        <x:v>appointments</x:v>
+      </x:c>
+      <x:c r="E13" s="473" t="str">
+        <x:v>checkInBookingAction updates appointments.checked_in_at/status</x:v>
+      </x:c>
+      <x:c r="F13" s="473" t="str">
+        <x:v>returnTo preserved into /booking/[id]</x:v>
+      </x:c>
+      <x:c r="G13" s="473" t="str">
+        <x:v>token validation + canAccessShelter</x:v>
+      </x:c>
+      <x:c r="H13" s="474" t="str">
+        <x:v>Generated QR now points to /booking/check-in</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="472" t="str">
+        <x:v>Shelter profile</x:v>
+      </x:c>
+      <x:c r="B14" s="473" t="str">
+        <x:v>Shared action reused</x:v>
+      </x:c>
+      <x:c r="C14" s="473" t="str">
+        <x:v>components/admin/AdminReorgDraftPanel.tsx + app/admin/bookings/actions.ts</x:v>
+      </x:c>
+      <x:c r="D14" s="473" t="str">
+        <x:v>shelters, shelter_regular_hours, shelter_availability</x:v>
+      </x:c>
+      <x:c r="E14" s="473" t="str">
+        <x:v>updateShelterProfileAction, operating days, blockouts</x:v>
+      </x:c>
+      <x:c r="F14" s="473" t="str">
+        <x:v>DraftReturnFields returnTo=/admindraft or /shelter/[slug]</x:v>
+      </x:c>
+      <x:c r="G14" s="473" t="str">
+        <x:v>requireShelterAccess(shelter_id)</x:v>
+      </x:c>
+      <x:c r="H14" s="474" t="str">
+        <x:v>Same shelter data in both admin and portal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="472" t="str">
+        <x:v>Public dog profile</x:v>
+      </x:c>
+      <x:c r="B15" s="473" t="str">
+        <x:v>Public route</x:v>
+      </x:c>
+      <x:c r="C15" s="473" t="str">
+        <x:v>app/dogs/[id]/page.tsx</x:v>
+      </x:c>
+      <x:c r="D15" s="473" t="str">
+        <x:v>dogs, dog_photos, dog_traits, shelters</x:v>
+      </x:c>
+      <x:c r="E15" s="473" t="str">
+        <x:v>Read-only public display</x:v>
+      </x:c>
+      <x:c r="F15" s="473" t="str">
+        <x:v>Browser/public navigation only</x:v>
+      </x:c>
+      <x:c r="G15" s="473" t="str">
+        <x:v>Public page; available dogs indexable</x:v>
+      </x:c>
+      <x:c r="H15" s="474" t="str">
+        <x:v>Only intentional shelter-to-public crossover</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="475" t="str">
+        <x:v>Not realtime yet</x:v>
+      </x:c>
+      <x:c r="B16" s="476" t="str">
+        <x:v>Architecture note</x:v>
+      </x:c>
+      <x:c r="C16" s="476" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="D16" s="476" t="str">
+        <x:v>Supabase tables are shared</x:v>
+      </x:c>
+      <x:c r="E16" s="476" t="str">
+        <x:v>Server actions revalidate key routes</x:v>
+      </x:c>
+      <x:c r="F16" s="476" t="str">
+        <x:v>Refresh/navigation shows latest DB state</x:v>
+      </x:c>
+      <x:c r="G16" s="476" t="str">
+        <x:v>No Supabase Realtime channel added yet</x:v>
+      </x:c>
+      <x:c r="H16" s="477" t="str">
+        <x:v>Add Realtime later if open tabs need instant updates</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="64" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="458" t="str">
+        <x:v>Shelter Pilot Readiness Checklist</x:v>
+      </x:c>
+      <x:c r="B1" s="458" t="str">
+        <x:v>Shelter Pilot Readiness Checklist</x:v>
+      </x:c>
+      <x:c r="C1" s="458" t="str">
+        <x:v>Shelter Pilot Readiness Checklist</x:v>
+      </x:c>
+      <x:c r="D1" s="458" t="str">
+        <x:v>Shelter Pilot Readiness Checklist</x:v>
+      </x:c>
+      <x:c r="E1" s="458" t="str">
+        <x:v>Shelter Pilot Readiness Checklist</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="461" t="str">
+        <x:v>Use this before giving shelter staff login credentials. The goal is to catch route leaks, sync issues, upload problems, and mobile friction before real data scaling.</x:v>
+      </x:c>
+      <x:c r="B2" s="461" t="str">
+        <x:v>Use this before giving shelter staff login credentials. The goal is to catch route leaks, sync issues, upload problems, and mobile friction before real data scaling.</x:v>
+      </x:c>
+      <x:c r="C2" s="461" t="str">
+        <x:v>Use this before giving shelter staff login credentials. The goal is to catch route leaks, sync issues, upload problems, and mobile friction before real data scaling.</x:v>
+      </x:c>
+      <x:c r="D2" s="461" t="str">
+        <x:v>Use this before giving shelter staff login credentials. The goal is to catch route leaks, sync issues, upload problems, and mobile friction before real data scaling.</x:v>
+      </x:c>
+      <x:c r="E2" s="461" t="str">
+        <x:v>Use this before giving shelter staff login credentials. The goal is to catch route leaks, sync issues, upload problems, and mobile friction before real data scaling.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="464" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="B4" s="465" t="str">
+        <x:v>What must be true</x:v>
+      </x:c>
+      <x:c r="C4" s="465" t="str">
+        <x:v>How to test</x:v>
+      </x:c>
+      <x:c r="D4" s="465" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E4" s="466" t="str">
+        <x:v>Owner / timing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="469" t="str">
+        <x:v>Login separation</x:v>
+      </x:c>
+      <x:c r="B5" s="470" t="str">
+        <x:v>Voice and Rescue Dog accounts route to their own /shelter/[slug] portal.</x:v>
+      </x:c>
+      <x:c r="C5" s="470" t="str">
+        <x:v>Use incognito; sign in as thevoice and rescuedog; verify no admin umbrella appears.</x:v>
+      </x:c>
+      <x:c r="D5" s="487" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
+      <x:c r="E5" s="471" t="str">
+        <x:v>Before sharing credentials</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="472" t="str">
+        <x:v>Shelter dog creation</x:v>
+      </x:c>
+      <x:c r="B6" s="473" t="str">
+        <x:v>Shelter can create dog with name, shelter, breed, matching fields, photos, cover order.</x:v>
+      </x:c>
+      <x:c r="C6" s="473" t="str">
+        <x:v>Create a test draft dog from /shelter/thevoicefoundation/dogs/new and confirm it appears in shelter and admin listings.</x:v>
+      </x:c>
+      <x:c r="D6" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E6" s="474" t="str">
+        <x:v>Before first staff upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="472" t="str">
+        <x:v>Shelter dog edit</x:v>
+      </x:c>
+      <x:c r="B7" s="473" t="str">
+        <x:v>Editing from /shelter/[slug]/dogs/[id]/edit updates same record admin sees.</x:v>
+      </x:c>
+      <x:c r="C7" s="473" t="str">
+        <x:v>Change a harmless field, return to shelter dog list, check /admindraft dog list and public dog page.</x:v>
+      </x:c>
+      <x:c r="D7" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E7" s="474" t="str">
+        <x:v>Before first staff upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="472" t="str">
+        <x:v>Photos and storage</x:v>
+      </x:c>
+      <x:c r="B8" s="473" t="str">
+        <x:v>Uploads land in dog-photos bucket and dog_photos rows; cover/order works.</x:v>
+      </x:c>
+      <x:c r="C8" s="473" t="str">
+        <x:v>Upload 2-3 small photos, set cover, save, reopen from both routes.</x:v>
+      </x:c>
+      <x:c r="D8" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E8" s="474" t="str">
+        <x:v>Before first real dog batch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="472" t="str">
+        <x:v>Back/exit behavior</x:v>
+      </x:c>
+      <x:c r="B9" s="473" t="str">
+        <x:v>Exit/back from dog create/edit and booking detail returns to the correct lane.</x:v>
+      </x:c>
+      <x:c r="C9" s="473" t="str">
+        <x:v>Click every visible Back, Exit, Dog listings, Booking list button from shelter and admin.</x:v>
+      </x:c>
+      <x:c r="D9" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E9" s="474" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="472" t="str">
+        <x:v>Booking list sync</x:v>
+      </x:c>
+      <x:c r="B10" s="473" t="str">
+        <x:v>Admin and shelter booking lists read same appointments and reflect status decisions.</x:v>
+      </x:c>
+      <x:c r="C10" s="473" t="str">
+        <x:v>Accept/deny/change one test booking from shelter; verify /admindraft booking list shows same status after reload.</x:v>
+      </x:c>
+      <x:c r="D10" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E10" s="474" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="472" t="str">
+        <x:v>Booking deep pages</x:v>
+      </x:c>
+      <x:c r="B11" s="473" t="str">
+        <x:v>Shared /booking detail and visitor profile never leak shelter to /admindraft.</x:v>
+      </x:c>
+      <x:c r="C11" s="473" t="str">
+        <x:v>Open booking detail/profile as shelter, use back buttons, edit returnTo manually once.</x:v>
+      </x:c>
+      <x:c r="D11" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E11" s="474" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="472" t="str">
+        <x:v>QR check-in</x:v>
+      </x:c>
+      <x:c r="B12" s="473" t="str">
+        <x:v>QR check-in opens /booking and preserves the correct return lane.</x:v>
+      </x:c>
+      <x:c r="C12" s="473" t="str">
+        <x:v>Scan or paste a test token from shelter booking list on phone.</x:v>
+      </x:c>
+      <x:c r="D12" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E12" s="474" t="str">
+        <x:v>Before shelter live visits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="472" t="str">
+        <x:v>Permission boundary</x:v>
+      </x:c>
+      <x:c r="B13" s="473" t="str">
+        <x:v>Voice cannot access Rescue Dog dog edit/booking routes and vice versa.</x:v>
+      </x:c>
+      <x:c r="C13" s="473" t="str">
+        <x:v>Copy a route from one shelter while signed into the other.</x:v>
+      </x:c>
+      <x:c r="D13" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E13" s="474" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="472" t="str">
+        <x:v>Mobile shelter UX</x:v>
+      </x:c>
+      <x:c r="B14" s="473" t="str">
+        <x:v>Dog create/edit and booking decisions are usable on phone width.</x:v>
+      </x:c>
+      <x:c r="C14" s="473" t="str">
+        <x:v>Test on mobile viewport or real phone for create dog, edit dog, booking decision.</x:v>
+      </x:c>
+      <x:c r="D14" s="540" t="str">
+        <x:v>Manual smoke test</x:v>
+      </x:c>
+      <x:c r="E14" s="474" t="str">
+        <x:v>Before staff training</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="472" t="str">
+        <x:v>Messaging</x:v>
+      </x:c>
+      <x:c r="B15" s="473" t="str">
+        <x:v>Messaging is intentionally not complete yet.</x:v>
+      </x:c>
+      <x:c r="C15" s="473" t="str">
+        <x:v>Do not promise messaging in the pilot unless built/tested in a separate session.</x:v>
+      </x:c>
+      <x:c r="D15" s="483" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E15" s="474" t="str">
+        <x:v>Separate build</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A16" s="472" t="str">
+        <x:v>Staff training note</x:v>
+      </x:c>
+      <x:c r="B16" s="473" t="str">
+        <x:v>Tell shelter staff to use visible Exit/Back buttons instead of relying on browser back.</x:v>
+      </x:c>
+      <x:c r="C16" s="473" t="str">
+        <x:v>Add this to onboarding SOP.</x:v>
+      </x:c>
+      <x:c r="D16" s="483" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="E16" s="474" t="str">
+        <x:v>Training</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="472" t="str">
+        <x:v>Temporary shared password</x:v>
+      </x:c>
+      <x:c r="B17" s="473" t="str">
+        <x:v>Shared login is okay for pilot but not long-term.</x:v>
+      </x:c>
+      <x:c r="C17" s="473" t="str">
+        <x:v>After pilot, move to employee accounts with audit history.</x:v>
+      </x:c>
+      <x:c r="D17" s="540" t="str">
+        <x:v>Watch</x:v>
+      </x:c>
+      <x:c r="E17" s="474" t="str">
+        <x:v>Post-pilot</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="475" t="str">
+        <x:v>Data backup/export</x:v>
+      </x:c>
+      <x:c r="B18" s="476" t="str">
+        <x:v>Before mass upload, export or snapshot dogs/shelters/appointments data.</x:v>
+      </x:c>
+      <x:c r="C18" s="476" t="str">
+        <x:v>Run Supabase export/dashboard backup process.</x:v>
+      </x:c>
+      <x:c r="D18" s="485" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="E18" s="477" t="str">
+        <x:v>Before large onboarding</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Migrate admin profile pages into admindraft
</commit_message>
<xml_diff>
--- a/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
+++ b/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
@@ -2,389 +2,31 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="R486035d6a5b74154"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="Rfd35a65c4a834ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="3" r:id="R74a05e29588c4806"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="4" r:id="R76ab6849f6a04757"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="5" r:id="R981289aaddef42dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="6" r:id="R1c4736847d474a1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="7" r:id="Rbe1519db220f45b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="8" r:id="Rcc1730b9bc7249c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="9" r:id="R65519966cf804bdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="10" r:id="R7d1cffe454e84578"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="11" r:id="R01e20ca402904def"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="Ra329004d8c1e4c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="Rccbb6f959970486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="3" r:id="R912cb7bc43c14d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="4" r:id="R0c10d944a4c74c96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="5" r:id="R99a26ce92d8f4833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="6" r:id="Rf7cd2d3c02fc4878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="7" r:id="R2c8ccf797d8146e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="8" r:id="R579aec150b2342f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="9" r:id="R5ef2e7432ee1424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="10" r:id="R4ee0a127d9954ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="11" r:id="Rc2c599a9435a493b"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:si>
-    <x:t xml:space="preserve">Area / Workflow</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Old Admin Route</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">New Admin Draft Location</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Status</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">What Is Left To Transfer</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Priority</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Admin gate / password</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Exists</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Keep temporary phrase gate until real login logic</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Later</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Main PawJai admin umbrella</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">scattered across /admin/*</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Continue moving remaining old admin tools into draft-native routes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">High</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Partner shelters overview</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">mostly inside /admin/bookings</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft &gt; Partner shelters</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Add deeper shelter metrics later if wanted</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Medium</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shelter profile edit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/bookings?view=profile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft &gt; Shelter profile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Functional</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Real-world save testing per shelter</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Done-ish</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shelter logo upload</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Real-world upload testing per shelter</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shelter donation details</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mostly transferred now</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shelter operating hours</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shelter blockout dates</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shelter dog listings</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/bookings?view=dogs, /admin/listings</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft &gt; Dog listings</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Search/status view is enough for shelter listing management; edit remains separate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Create dog listing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin, /admin/dogs/new</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft/dog-creation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Draft-native create flow exists; real-world save/photo testing remains</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Edit dog listing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/dogs/[id]/edit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft/dogs/[id]/edit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Draft-native edit route reuses the full old edit form; real-world save/photo testing remains</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Dog photos / cover order</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin, /admin/dogs/[id]/edit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Edit route now includes existing upload, reorder, cover, and remove tools</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">All dog listings across shelters</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/listings</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft &gt; All dog listings</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Filters exist and edit buttons now open draft-native dog edit pages</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Booking visits list</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/bookings</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft &gt; Bookings</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Old low-friction booking card flow duplicated; real staff testing remains</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Booking decision actions</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/bookings, /admin/bookings/[id]</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Accept, deny, and date-change actions are draft-native; final status edge cases can be polished later</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Booking detail page</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/bookings/[id]</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft/bookings/[id]</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QR scan can land here; refine isolated detail page only if needed</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QR check-in</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/bookings/check-in</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft/bookings/check-in</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs real QR/camera device testing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Visitor profile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/bookings/[id]/visitor-profile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft/bookings/[id]/visitor-profile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Draft-native profile/documents view exists; real document review testing remains</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shelter messaging</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/bookings?view=messages</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft &gt; Messaging</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Visual only</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Transfer real message thread and send reply in separate messaging session</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ads management</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/ads</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft &gt; Ads</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Read only</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Transfer create ad, edit dates, pause/resume, delete</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">About content</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/pawjaiprofile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admindraft &gt; About content</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Transfer full About editor/save action</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Admin accounts</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/accounts</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">not yet</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Missing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Transfer PawJai/shelter admin account creation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Audit log</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/audit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Transfer audit table view</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Admin login page</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/login</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">temporary phrase gate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Temporary</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Later replace phrase gates with real auth</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Legacy draft alias</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/admin/reorg-draft</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Remove after /admindraft becomes canonical</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PAWJAI Admin Draft Transfer Progress</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Count</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">% of workflows</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Meaning</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Moved into draft and connected enough to use/test</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Present in draft, but may still need deeper behavior</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Partial</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Some behavior moved, still depends on old admin or missing pieces</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Real data visible, write controls not transferred</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Layout placeholder only</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Temporary bridge until real auth/login</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Not moved yet</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Metric</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Value</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Functional workflows</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Functional + Exists</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Still high priority</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Total workflows</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Current read: shelter profile, dog creation/listing, and booking flows are now the strongest draft areas. Messaging is intentionally left for a separate session.</x:t>
-  </x:si>
-</x:sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="20">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0%"/>
+  </x:numFmts>
+  <x:fonts count="22">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -501,8 +143,19 @@
       <x:color rgb="FF5B4D40"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF4F4338"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="81">
+  <x:fills count="113">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -902,6 +555,166 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7E3E1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F1EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B4D40"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD88C24"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8ECD8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F1EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B4D40"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD88C24"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8ECD8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F1EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B4D40"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD88C24"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8ECD8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F1EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B4D40"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD88C24"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8ECD8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1019,7 +832,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="541">
+  <x:cellXfs count="735">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -2337,6 +2150,342 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="17" fillId="74" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="81" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="82" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="83" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="84" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="85" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="82" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="82" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="82" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="87" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="85" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="88" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="83" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="85" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="12" fillId="85" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="13" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="89" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="90" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="91" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="92" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="93" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="94" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="94" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="95" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="95" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="92" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="92" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="96" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="96" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="91" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="91" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="95" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="90" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="93" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="92" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="96" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="90" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="91" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="90" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="93" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="92" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="12" fillId="93" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="13" fillId="92" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="94" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="94" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="96" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="96" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="95" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="95" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="95" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="95" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="93" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="93" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="90" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="90" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="92" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="92" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="90" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="97" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="98" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="99" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="100" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="101" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="102" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="102" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="103" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="103" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="98" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="98" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="101" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="101" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="100" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="100" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="104" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="104" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="98" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="98" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="99" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="99" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="101" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="101" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="103" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="98" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="100" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="104" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="98" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="99" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="98" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="100" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="13" fillId="100" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="102" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="104" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="104" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="98" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="98" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="100" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="100" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="105" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="106" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="107" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="108" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="109" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="110" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="110" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="111" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="111" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="106" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="106" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="108" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="108" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="112" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="112" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="106" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="106" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="111" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="106" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="109" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="108" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="112" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="106" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="107" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="106" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="109" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="108" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="12" fillId="109" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="13" fillId="108" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="110" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="112" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="112" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="109" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="109" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="106" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="106" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="108" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="108" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2358,13 +2507,13 @@
     <xdr:ext cx="7239000" cy="4095750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="48fd0a8e-8f5f-439d-8f7a-fd98a22e40b7"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R84c8484b21db4309"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6c71fcbcd5df4aac"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2385,13 +2534,13 @@
     <xdr:ext cx="7239000" cy="4095750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="9e6d2b00-eee6-4c87-93c4-09fa62d9c950"/>
+        <xdr:cNvPr id="2" name="/xl/media/image2.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3db7df041d0842e2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re6d86f2eb7774373"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2600,531 +2749,532 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <x:cols>
-    <x:col min="1" max="1" width="30" customWidth="1"/>
-    <x:col min="2" max="3" width="34" customWidth="1"/>
-    <x:col min="4" max="4" width="15" customWidth="1"/>
-    <x:col min="5" max="5" width="58" customWidth="1"/>
-    <x:col min="6" max="6" width="14" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="1" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="1" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C1" s="1" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D1" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E1" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F1" s="1" t="s">
-        <x:v>5</x:v>
+      <x:c r="A1" s="1" t="str">
+        <x:v>Area / Workflow</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="str">
+        <x:v>Old Admin Route</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="str">
+        <x:v>New Admin Draft Location</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="str">
+        <x:v>What Is Left To Transfer</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="str">
+        <x:v>Priority</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="16">
-      <x:c r="A2" s="3" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B2" s="3" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C2" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D2" s="4" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E2" s="3" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F2" s="5" t="s">
-        <x:v>11</x:v>
+      <x:c r="A2" s="691" t="str">
+        <x:v>Admin gate / password</x:v>
+      </x:c>
+      <x:c r="B2" s="691" t="str">
+        <x:v>/admin</x:v>
+      </x:c>
+      <x:c r="C2" s="691" t="str">
+        <x:v>/admindraft</x:v>
+      </x:c>
+      <x:c r="D2" s="692" t="str">
+        <x:v>Exists</x:v>
+      </x:c>
+      <x:c r="E2" s="691" t="str">
+        <x:v>Keep temporary phrase gate until real login logic</x:v>
+      </x:c>
+      <x:c r="F2" s="693" t="str">
+        <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="16">
-      <x:c r="A3" s="3" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B3" s="3" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C3" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D3" s="4" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E3" s="3" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F3" s="6" t="s">
-        <x:v>15</x:v>
+      <x:c r="A3" s="691" t="str">
+        <x:v>Main PawJai admin umbrella</x:v>
+      </x:c>
+      <x:c r="B3" s="691" t="str">
+        <x:v>scattered across /admin/*</x:v>
+      </x:c>
+      <x:c r="C3" s="691" t="str">
+        <x:v>/admindraft</x:v>
+      </x:c>
+      <x:c r="D3" s="692" t="str">
+        <x:v>Exists</x:v>
+      </x:c>
+      <x:c r="E3" s="691" t="str">
+        <x:v>About, Accounts, and Audit now have draft-native pages; Ads write controls and Messaging remain the main gaps</x:v>
+      </x:c>
+      <x:c r="F3" s="694" t="str">
+        <x:v>High</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="16">
-      <x:c r="A4" s="3" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B4" s="3" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C4" s="3" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="D4" s="4" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E4" s="3" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="F4" s="7" t="s">
-        <x:v>20</x:v>
+      <x:c r="A4" s="691" t="str">
+        <x:v>Partner shelters overview</x:v>
+      </x:c>
+      <x:c r="B4" s="691" t="str">
+        <x:v>mostly inside /admin/bookings</x:v>
+      </x:c>
+      <x:c r="C4" s="691" t="str">
+        <x:v>/admindraft &gt; Partner shelters</x:v>
+      </x:c>
+      <x:c r="D4" s="692" t="str">
+        <x:v>Exists</x:v>
+      </x:c>
+      <x:c r="E4" s="691" t="str">
+        <x:v>Add deeper shelter metrics later if wanted</x:v>
+      </x:c>
+      <x:c r="F4" s="695" t="str">
+        <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="16">
-      <x:c r="A5" s="3" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C5" s="3" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E5" s="3" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A5" s="691" t="str">
+        <x:v>Shelter profile edit</x:v>
+      </x:c>
+      <x:c r="B5" s="691" t="str">
+        <x:v>/admin/bookings?view=profile</x:v>
+      </x:c>
+      <x:c r="C5" s="691" t="str">
+        <x:v>/admindraft &gt; Shelter profile</x:v>
+      </x:c>
+      <x:c r="D5" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E5" s="691" t="str">
+        <x:v>Real-world save testing per shelter</x:v>
+      </x:c>
+      <x:c r="F5" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16">
-      <x:c r="A6" s="3" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D6" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="F6" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A6" s="691" t="str">
+        <x:v>Shelter logo upload</x:v>
+      </x:c>
+      <x:c r="B6" s="691" t="str">
+        <x:v>/admin/bookings?view=profile</x:v>
+      </x:c>
+      <x:c r="C6" s="691" t="str">
+        <x:v>/admindraft &gt; Shelter profile</x:v>
+      </x:c>
+      <x:c r="D6" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E6" s="691" t="str">
+        <x:v>Real-world upload testing per shelter</x:v>
+      </x:c>
+      <x:c r="F6" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="16">
-      <x:c r="A7" s="3" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C7" s="3" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D7" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E7" s="3" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="F7" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A7" s="691" t="str">
+        <x:v>Shelter donation details</x:v>
+      </x:c>
+      <x:c r="B7" s="691" t="str">
+        <x:v>/admin/bookings?view=profile</x:v>
+      </x:c>
+      <x:c r="C7" s="691" t="str">
+        <x:v>/admindraft &gt; Shelter profile</x:v>
+      </x:c>
+      <x:c r="D7" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E7" s="691" t="str">
+        <x:v>Mostly transferred now</x:v>
+      </x:c>
+      <x:c r="F7" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="16">
-      <x:c r="A8" s="3" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D8" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="F8" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A8" s="691" t="str">
+        <x:v>Shelter operating hours</x:v>
+      </x:c>
+      <x:c r="B8" s="691" t="str">
+        <x:v>/admin/bookings?view=profile</x:v>
+      </x:c>
+      <x:c r="C8" s="691" t="str">
+        <x:v>/admindraft &gt; Shelter profile</x:v>
+      </x:c>
+      <x:c r="D8" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E8" s="691" t="str">
+        <x:v>Mostly transferred now</x:v>
+      </x:c>
+      <x:c r="F8" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
-      <x:c r="A9" s="3" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B9" s="3" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C9" s="3" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D9" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E9" s="3" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="F9" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A9" s="691" t="str">
+        <x:v>Shelter blockout dates</x:v>
+      </x:c>
+      <x:c r="B9" s="691" t="str">
+        <x:v>/admin/bookings?view=profile</x:v>
+      </x:c>
+      <x:c r="C9" s="691" t="str">
+        <x:v>/admindraft &gt; Shelter profile</x:v>
+      </x:c>
+      <x:c r="D9" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E9" s="691" t="str">
+        <x:v>Mostly transferred now</x:v>
+      </x:c>
+      <x:c r="F9" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32">
-      <x:c r="A10" s="3" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="C10" s="3" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="D10" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E10" s="3" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F10" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A10" s="691" t="str">
+        <x:v>Shelter dog listings</x:v>
+      </x:c>
+      <x:c r="B10" s="691" t="str">
+        <x:v>/admin/bookings?view=dogs, /admin/listings</x:v>
+      </x:c>
+      <x:c r="C10" s="691" t="str">
+        <x:v>/admindraft &gt; Dog listings</x:v>
+      </x:c>
+      <x:c r="D10" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E10" s="691" t="str">
+        <x:v>Search/status view is enough for shelter listing management; edit remains separate</x:v>
+      </x:c>
+      <x:c r="F10" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="16">
-      <x:c r="A11" s="3" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C11" s="3" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D11" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E11" s="3" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="F11" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A11" s="691" t="str">
+        <x:v>Create dog listing</x:v>
+      </x:c>
+      <x:c r="B11" s="691" t="str">
+        <x:v>/admin, /admin/dogs/new</x:v>
+      </x:c>
+      <x:c r="C11" s="691" t="str">
+        <x:v>/admindraft/dog-creation</x:v>
+      </x:c>
+      <x:c r="D11" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E11" s="691" t="str">
+        <x:v>Draft-native create flow exists; real-world save/photo testing remains</x:v>
+      </x:c>
+      <x:c r="F11" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32">
-      <x:c r="A12" s="3" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="C12" s="3" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="D12" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E12" s="3" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F12" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A12" s="691" t="str">
+        <x:v>Edit dog listing</x:v>
+      </x:c>
+      <x:c r="B12" s="691" t="str">
+        <x:v>/admin/dogs/[id]/edit</x:v>
+      </x:c>
+      <x:c r="C12" s="691" t="str">
+        <x:v>/admindraft/dogs/[id]/edit</x:v>
+      </x:c>
+      <x:c r="D12" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E12" s="691" t="str">
+        <x:v>Draft-native edit route reuses the full old edit form; real-world save/photo testing remains</x:v>
+      </x:c>
+      <x:c r="F12" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="32">
-      <x:c r="A13" s="3" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="B13" s="3" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="C13" s="3" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="D13" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E13" s="3" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="F13" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A13" s="691" t="str">
+        <x:v>Dog photos / cover order</x:v>
+      </x:c>
+      <x:c r="B13" s="691" t="str">
+        <x:v>/admin, /admin/dogs/[id]/edit</x:v>
+      </x:c>
+      <x:c r="C13" s="691" t="str">
+        <x:v>/admindraft/dogs/[id]/edit</x:v>
+      </x:c>
+      <x:c r="D13" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E13" s="691" t="str">
+        <x:v>Edit route now includes existing upload, reorder, cover, and remove tools</x:v>
+      </x:c>
+      <x:c r="F13" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16">
-      <x:c r="A14" s="3" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="C14" s="3" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="D14" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E14" s="3" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F14" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A14" s="691" t="str">
+        <x:v>All dog listings across shelters</x:v>
+      </x:c>
+      <x:c r="B14" s="691" t="str">
+        <x:v>/admin/listings</x:v>
+      </x:c>
+      <x:c r="C14" s="691" t="str">
+        <x:v>/admindraft &gt; All dog listings</x:v>
+      </x:c>
+      <x:c r="D14" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E14" s="691" t="str">
+        <x:v>Filters exist and edit buttons now open draft-native dog edit pages</x:v>
+      </x:c>
+      <x:c r="F14" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32">
-      <x:c r="A15" s="3" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="B15" s="3" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="C15" s="3" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="D15" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E15" s="3" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F15" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A15" s="691" t="str">
+        <x:v>Booking visits list</x:v>
+      </x:c>
+      <x:c r="B15" s="691" t="str">
+        <x:v>/admin/bookings</x:v>
+      </x:c>
+      <x:c r="C15" s="691" t="str">
+        <x:v>/admindraft &gt; Bookings</x:v>
+      </x:c>
+      <x:c r="D15" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E15" s="691" t="str">
+        <x:v>Old low-friction booking card flow duplicated; real staff testing remains</x:v>
+      </x:c>
+      <x:c r="F15" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="32">
-      <x:c r="A16" s="3" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B16" s="3" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="C16" s="3" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="D16" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E16" s="3" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="F16" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A16" s="691" t="str">
+        <x:v>Booking decision actions</x:v>
+      </x:c>
+      <x:c r="B16" s="691" t="str">
+        <x:v>/admin/bookings, /admin/bookings/[id]</x:v>
+      </x:c>
+      <x:c r="C16" s="691" t="str">
+        <x:v>/admindraft &gt; Bookings</x:v>
+      </x:c>
+      <x:c r="D16" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E16" s="691" t="str">
+        <x:v>Accept, deny, and date-change actions are draft-native; final status edge cases can be polished later</x:v>
+      </x:c>
+      <x:c r="F16" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="16">
-      <x:c r="A17" s="3" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B17" s="3" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="C17" s="3" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="D17" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E17" s="3" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="F17" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A17" s="691" t="str">
+        <x:v>Booking detail page</x:v>
+      </x:c>
+      <x:c r="B17" s="691" t="str">
+        <x:v>/admin/bookings/[id]</x:v>
+      </x:c>
+      <x:c r="C17" s="691" t="str">
+        <x:v>/admindraft/bookings/[id]</x:v>
+      </x:c>
+      <x:c r="D17" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E17" s="691" t="str">
+        <x:v>QR scan can land here; refine isolated detail page only if needed</x:v>
+      </x:c>
+      <x:c r="F17" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="16">
-      <x:c r="A18" s="3" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="B18" s="3" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="C18" s="3" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="D18" s="4" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E18" s="3" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="F18" s="7" t="s">
-        <x:v>20</x:v>
+      <x:c r="A18" s="691" t="str">
+        <x:v>QR check-in</x:v>
+      </x:c>
+      <x:c r="B18" s="691" t="str">
+        <x:v>/admin/bookings/check-in</x:v>
+      </x:c>
+      <x:c r="C18" s="691" t="str">
+        <x:v>/admindraft/bookings/check-in</x:v>
+      </x:c>
+      <x:c r="D18" s="692" t="str">
+        <x:v>Exists</x:v>
+      </x:c>
+      <x:c r="E18" s="691" t="str">
+        <x:v>Needs real QR/camera device testing</x:v>
+      </x:c>
+      <x:c r="F18" s="695" t="str">
+        <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32">
-      <x:c r="A19" s="3" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="B19" s="3" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="C19" s="3" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="D19" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E19" s="3" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="F19" s="4" t="s">
-        <x:v>26</x:v>
+      <x:c r="A19" s="691" t="str">
+        <x:v>Visitor profile</x:v>
+      </x:c>
+      <x:c r="B19" s="691" t="str">
+        <x:v>/admin/bookings/[id]/visitor-profile</x:v>
+      </x:c>
+      <x:c r="C19" s="691" t="str">
+        <x:v>/admindraft/bookings/[id]/visitor-profile</x:v>
+      </x:c>
+      <x:c r="D19" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E19" s="691" t="str">
+        <x:v>Draft-native profile/documents view exists; real document review testing remains</x:v>
+      </x:c>
+      <x:c r="F19" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="32">
-      <x:c r="A20" s="3" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="B20" s="3" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="C20" s="3" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="D20" s="6" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="E20" s="3" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="F20" s="6" t="s">
-        <x:v>15</x:v>
+      <x:c r="A20" s="691" t="str">
+        <x:v>Shelter messaging</x:v>
+      </x:c>
+      <x:c r="B20" s="691" t="str">
+        <x:v>/admin/bookings?view=messages</x:v>
+      </x:c>
+      <x:c r="C20" s="691" t="str">
+        <x:v>/admindraft &gt; Messaging</x:v>
+      </x:c>
+      <x:c r="D20" s="694" t="str">
+        <x:v>Visual only</x:v>
+      </x:c>
+      <x:c r="E20" s="691" t="str">
+        <x:v>Transfer real message thread and send reply in separate messaging session</x:v>
+      </x:c>
+      <x:c r="F20" s="694" t="str">
+        <x:v>High</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16">
-      <x:c r="A21" s="3" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="B21" s="3" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="C21" s="3" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="D21" s="7" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="E21" s="3" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="F21" s="7" t="s">
-        <x:v>20</x:v>
+      <x:c r="A21" s="691" t="str">
+        <x:v>Ads management</x:v>
+      </x:c>
+      <x:c r="B21" s="691" t="str">
+        <x:v>/admin/ads</x:v>
+      </x:c>
+      <x:c r="C21" s="691" t="str">
+        <x:v>/admindraft &gt; Ads</x:v>
+      </x:c>
+      <x:c r="D21" s="695" t="str">
+        <x:v>Read only</x:v>
+      </x:c>
+      <x:c r="E21" s="691" t="str">
+        <x:v>Transfer create ad, edit dates, pause/resume, delete</x:v>
+      </x:c>
+      <x:c r="F21" s="695" t="str">
+        <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="16">
-      <x:c r="A22" s="3" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="B22" s="3" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="C22" s="3" t="s">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="D22" s="7" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="E22" s="3" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="F22" s="7" t="s">
-        <x:v>20</x:v>
+      <x:c r="A22" s="691" t="str">
+        <x:v>About content</x:v>
+      </x:c>
+      <x:c r="B22" s="691" t="str">
+        <x:v>/admin/pawjaiprofile</x:v>
+      </x:c>
+      <x:c r="C22" s="691" t="str">
+        <x:v>/admindraft/pawjaiprofile</x:v>
+      </x:c>
+      <x:c r="D22" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E22" s="691" t="str">
+        <x:v>Draft-native About editor exists and saves through the same pawjai_profile table; live save smoke test remains</x:v>
+      </x:c>
+      <x:c r="F22" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="16">
-      <x:c r="A23" s="3" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="B23" s="3" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="C23" s="3" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="D23" s="6" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="E23" s="3" t="s">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="F23" s="5" t="s">
-        <x:v>11</x:v>
+      <x:c r="A23" s="691" t="str">
+        <x:v>Admin accounts</x:v>
+      </x:c>
+      <x:c r="B23" s="691" t="str">
+        <x:v>/admin/accounts</x:v>
+      </x:c>
+      <x:c r="C23" s="691" t="str">
+        <x:v>/admindraft/accounts</x:v>
+      </x:c>
+      <x:c r="D23" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E23" s="691" t="str">
+        <x:v>Draft-native account creation/revoke exists and uses the same Supabase Auth, profiles, and shelter_users logic</x:v>
+      </x:c>
+      <x:c r="F23" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="16">
-      <x:c r="A24" s="3" t="s">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="B24" s="3" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="C24" s="3" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="D24" s="6" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="E24" s="3" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="F24" s="5" t="s">
-        <x:v>11</x:v>
+      <x:c r="A24" s="691" t="str">
+        <x:v>Audit log</x:v>
+      </x:c>
+      <x:c r="B24" s="691" t="str">
+        <x:v>/admin/audit</x:v>
+      </x:c>
+      <x:c r="C24" s="691" t="str">
+        <x:v>/admindraft/audit</x:v>
+      </x:c>
+      <x:c r="D24" s="692" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="E24" s="691" t="str">
+        <x:v>Draft-native audit table exists; keep testing with real admin changes</x:v>
+      </x:c>
+      <x:c r="F24" s="692" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="16">
-      <x:c r="A25" s="3" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="B25" s="3" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="C25" s="3" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="D25" s="7" t="s">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="E25" s="3" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="F25" s="5" t="s">
-        <x:v>11</x:v>
+      <x:c r="A25" s="691" t="str">
+        <x:v>Admin login page</x:v>
+      </x:c>
+      <x:c r="B25" s="691" t="str">
+        <x:v>/admin/login</x:v>
+      </x:c>
+      <x:c r="C25" s="691" t="str">
+        <x:v>temporary phrase gate</x:v>
+      </x:c>
+      <x:c r="D25" s="695" t="str">
+        <x:v>Temporary</x:v>
+      </x:c>
+      <x:c r="E25" s="691" t="str">
+        <x:v>Later replace phrase gates with real auth</x:v>
+      </x:c>
+      <x:c r="F25" s="693" t="str">
+        <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="16">
-      <x:c r="A26" s="3" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="B26" s="3" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="C26" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D26" s="4" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E26" s="3" t="s">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="F26" s="5" t="s">
-        <x:v>11</x:v>
+      <x:c r="A26" s="691" t="str">
+        <x:v>Legacy draft alias</x:v>
+      </x:c>
+      <x:c r="B26" s="691" t="str">
+        <x:v>/admin/reorg-draft</x:v>
+      </x:c>
+      <x:c r="C26" s="691" t="str">
+        <x:v>/admindraft</x:v>
+      </x:c>
+      <x:c r="D26" s="692" t="str">
+        <x:v>Exists</x:v>
+      </x:c>
+      <x:c r="E26" s="691" t="str">
+        <x:v>Remove after /admindraft becomes canonical</x:v>
+      </x:c>
+      <x:c r="F26" s="693" t="str">
+        <x:v>Later</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3384,7 +3534,7 @@
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R533a6f1712924216"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ac0f56048d54379"/>
 </x:worksheet>
 </file>
 
@@ -3392,201 +3542,201 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <x:cols>
-    <x:col min="1" max="1" width="113.1640625" customWidth="1"/>
-    <x:col min="2" max="2" width="4.83203125" customWidth="1"/>
-    <x:col min="3" max="3" width="11.83203125" customWidth="1"/>
-    <x:col min="4" max="4" width="64" customWidth="1"/>
+    <x:col min="1" max="1" width="154.77999877929688" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="4.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="64" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21">
-      <x:c r="A1" s="20" t="s">
-        <x:v>101</x:v>
-      </x:c>
-      <x:c r="B1" s="21"/>
-      <x:c r="C1" s="21"/>
-      <x:c r="D1" s="21"/>
-      <x:c r="E1" s="21"/>
-      <x:c r="F1" s="21"/>
+      <x:c r="A1" s="697" t="str">
+        <x:v>PAWJAI Admin Draft Transfer Progress</x:v>
+      </x:c>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
     </x:row>
     <x:row r="3" ht="15">
-      <x:c r="A3" s="8" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="8" t="s">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="C3" s="8" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="D3" s="8" t="s">
-        <x:v>104</x:v>
+      <x:c r="A3" s="714" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="B3" s="714" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+      <x:c r="C3" s="714" t="str">
+        <x:v>% of workflows</x:v>
+      </x:c>
+      <x:c r="D3" s="714" t="str">
+        <x:v>Meaning</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15">
-      <x:c r="A4" s="15" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="n">
+      <x:c r="A4" s="721" t="str">
+        <x:v>Functional</x:v>
+      </x:c>
+      <x:c r="B4" s="715" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A4)</x:f>
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C4" s="13" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C4" s="719" t="n">
         <x:f>B4/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
-        <x:v>0.56</x:v>
-      </x:c>
-      <x:c r="D4" s="2" t="s">
-        <x:v>105</x:v>
+        <x:v>0.68</x:v>
+      </x:c>
+      <x:c r="D4" s="570" t="str">
+        <x:v>Moved into draft and connected enough to use/test</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15">
-      <x:c r="A5" s="15" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="n">
+      <x:c r="A5" s="721" t="str">
+        <x:v>Exists</x:v>
+      </x:c>
+      <x:c r="B5" s="715" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A5)</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="n">
+      <x:c r="C5" s="719" t="n">
         <x:f>B5/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="D5" s="2" t="s">
-        <x:v>106</x:v>
+      <x:c r="D5" s="570" t="str">
+        <x:v>Present in draft, but may still need deeper behavior</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15">
-      <x:c r="A6" s="16" t="s">
-        <x:v>107</x:v>
-      </x:c>
-      <x:c r="B6" s="10" t="n">
+      <x:c r="A6" s="722" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="B6" s="716" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C6" s="18" t="n">
+      <x:c r="C6" s="724" t="n">
         <x:f>B6/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D6" s="2" t="s">
-        <x:v>108</x:v>
+      <x:c r="D6" s="570" t="str">
+        <x:v>Some behavior moved, still depends on old admin or missing pieces</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15">
-      <x:c r="A7" s="16" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="B7" s="10" t="n">
+      <x:c r="A7" s="722" t="str">
+        <x:v>Read only</x:v>
+      </x:c>
+      <x:c r="B7" s="716" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A7)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C7" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="724" t="n">
         <x:f>B7/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="D7" s="2" t="s">
-        <x:v>109</x:v>
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="D7" s="570" t="str">
+        <x:v>Real data visible, write controls not transferred</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15">
-      <x:c r="A8" s="17" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="B8" s="11" t="n">
+      <x:c r="A8" s="723" t="str">
+        <x:v>Visual only</x:v>
+      </x:c>
+      <x:c r="B8" s="717" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A8)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="19" t="n">
+      <x:c r="C8" s="725" t="n">
         <x:f>B8/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
-      <x:c r="D8" s="2" t="s">
-        <x:v>110</x:v>
+      <x:c r="D8" s="570" t="str">
+        <x:v>Layout placeholder only</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15">
-      <x:c r="A9" s="16" t="s">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="B9" s="10" t="n">
+      <x:c r="A9" s="722" t="str">
+        <x:v>Temporary</x:v>
+      </x:c>
+      <x:c r="B9" s="716" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C9" s="18" t="n">
+      <x:c r="C9" s="724" t="n">
         <x:f>B9/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
-      <x:c r="D9" s="2" t="s">
-        <x:v>111</x:v>
+      <x:c r="D9" s="570" t="str">
+        <x:v>Temporary bridge until real auth/login</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15">
-      <x:c r="A10" s="17" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="B10" s="11" t="n">
+      <x:c r="A10" s="723" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="B10" s="717" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A10)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C10" s="19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C10" s="725" t="n">
         <x:f>B10/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="D10" s="2" t="s">
-        <x:v>112</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="570" t="str">
+        <x:v>Not moved yet</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15">
-      <x:c r="A13" s="12" t="s">
-        <x:v>113</x:v>
-      </x:c>
-      <x:c r="B13" s="12" t="s">
-        <x:v>114</x:v>
+      <x:c r="A13" s="718" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B13" s="718" t="str">
+        <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15">
-      <x:c r="A14" s="15" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="B14" s="9" t="n">
+      <x:c r="A14" s="721" t="str">
+        <x:v>Functional workflows</x:v>
+      </x:c>
+      <x:c r="B14" s="715" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Functional")</x:f>
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15">
-      <x:c r="A15" s="15" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="B15" s="13" t="n">
+      <x:c r="A15" s="721" t="str">
+        <x:v>Functional + Exists</x:v>
+      </x:c>
+      <x:c r="B15" s="719" t="n">
         <x:f>(COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Functional")+COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Exists"))/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
-        <x:v>0.76</x:v>
+        <x:v>0.88</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15">
-      <x:c r="A16" s="17" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="B16" s="11" t="n">
+      <x:c r="A16" s="723" t="str">
+        <x:v>Still high priority</x:v>
+      </x:c>
+      <x:c r="B16" s="717" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$F$2:$F$26,"High")</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15">
-      <x:c r="A17" s="14" t="s">
-        <x:v>118</x:v>
-      </x:c>
-      <x:c r="B17" s="14" t="n">
+      <x:c r="A17" s="720" t="str">
+        <x:v>Total workflows</x:v>
+      </x:c>
+      <x:c r="B17" s="720" t="n">
         <x:f>COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
-      <x:c r="A20" s="22" t="s">
-        <x:v>119</x:v>
-      </x:c>
-      <x:c r="B20" s="21"/>
-      <x:c r="C20" s="21"/>
-      <x:c r="D20" s="21"/>
-      <x:c r="E20" s="21"/>
-      <x:c r="F20" s="21"/>
+      <x:c r="A20" s="713" t="str">
+        <x:v>Current read: shelter profile, dog creation/listing, booking flows, About content, Accounts, and Audit are now draft-native. Messaging is intentionally left for a separate session; Ads still needs write controls moved.</x:v>
+      </x:c>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3602,392 +3752,412 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="54" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
-      <x:c r="A1" s="458" t="str">
-        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
-      </x:c>
-      <x:c r="B1" s="458" t="str">
-        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
-      </x:c>
-      <x:c r="C1" s="458" t="str">
-        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
-      </x:c>
-      <x:c r="D1" s="458" t="str">
-        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
-      </x:c>
-      <x:c r="E1" s="458" t="str">
-        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
-      </x:c>
-      <x:c r="F1" s="458" t="str">
-        <x:v>PAWJAI Admin → Shelter → Booking Route Migration Map</x:v>
-      </x:c>
+      <x:c r="A1" s="726" t="str">
+        <x:v>PAWJAI Admin -&gt; Shelter -&gt; Booking Route Migration Map</x:v>
+      </x:c>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="461" t="str">
+      <x:c r="A2" s="728" t="str">
         <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
       </x:c>
-      <x:c r="B2" s="461" t="str">
-        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
-      </x:c>
-      <x:c r="C2" s="461" t="str">
-        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
-      </x:c>
-      <x:c r="D2" s="461" t="str">
-        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
-      </x:c>
-      <x:c r="E2" s="461" t="str">
-        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
-      </x:c>
-      <x:c r="F2" s="461" t="str">
-        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
-      </x:c>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="464" t="str">
+      <x:c r="A4" s="714" t="str">
         <x:v>Workflow</x:v>
       </x:c>
-      <x:c r="B4" s="465" t="str">
+      <x:c r="B4" s="714" t="str">
         <x:v>Old / current source</x:v>
       </x:c>
-      <x:c r="C4" s="465" t="str">
+      <x:c r="C4" s="714" t="str">
         <x:v>New canonical route</x:v>
       </x:c>
-      <x:c r="D4" s="465" t="str">
+      <x:c r="D4" s="714" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="E4" s="465" t="str">
+      <x:c r="E4" s="714" t="str">
         <x:v>What it does</x:v>
       </x:c>
-      <x:c r="F4" s="466" t="str">
+      <x:c r="F4" s="714" t="str">
         <x:v>Notes / next step</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A5" s="469" t="str">
+      <x:c r="A5" s="639" t="str">
         <x:v>Old production admin</x:v>
       </x:c>
-      <x:c r="B5" s="470" t="str">
+      <x:c r="B5" s="639" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="C5" s="470" t="str">
+      <x:c r="C5" s="639" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="D5" s="479" t="str">
+      <x:c r="D5" s="730" t="str">
         <x:v>Legacy active</x:v>
       </x:c>
-      <x:c r="E5" s="470" t="str">
+      <x:c r="E5" s="639" t="str">
         <x:v>Current live admin remains usable until /admindraft fully replaces it</x:v>
       </x:c>
-      <x:c r="F5" s="471" t="str">
+      <x:c r="F5" s="639" t="str">
         <x:v>Do not delete until every workflow is verified in /admindraft and /shelter</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A6" s="472" t="str">
+      <x:c r="A6" s="639" t="str">
         <x:v>PawJai umbrella dashboard</x:v>
       </x:c>
-      <x:c r="B6" s="473" t="str">
+      <x:c r="B6" s="639" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="C6" s="473" t="str">
+      <x:c r="C6" s="639" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D6" s="481" t="str">
+      <x:c r="D6" s="732" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E6" s="473" t="str">
-        <x:v>PawJai HQ sees all shelters, dogs, bookings, ads, and about content</x:v>
-      </x:c>
-      <x:c r="F6" s="474" t="str">
+      <x:c r="E6" s="639" t="str">
+        <x:v>PawJai HQ sees all shelters, dogs, bookings, ads, about content, accounts, and audit</x:v>
+      </x:c>
+      <x:c r="F6" s="639" t="str">
         <x:v>Keep as the admin umbrella; do not make shelter staff use this route</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="472" t="str">
+      <x:c r="A7" s="639" t="str">
         <x:v>Shelter login</x:v>
       </x:c>
-      <x:c r="B7" s="473" t="str">
+      <x:c r="B7" s="639" t="str">
         <x:v>not separated before</x:v>
       </x:c>
-      <x:c r="C7" s="473" t="str">
+      <x:c r="C7" s="639" t="str">
         <x:v>/shelter</x:v>
       </x:c>
-      <x:c r="D7" s="481" t="str">
+      <x:c r="D7" s="732" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E7" s="473" t="str">
+      <x:c r="E7" s="639" t="str">
         <x:v>Username/password login for partner shelters</x:v>
       </x:c>
-      <x:c r="F7" s="474" t="str">
+      <x:c r="F7" s="639" t="str">
         <x:v>Always redirect shelter users here when not signed in</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A8" s="472" t="str">
+      <x:c r="A8" s="639" t="str">
         <x:v>Shelter workspace</x:v>
       </x:c>
-      <x:c r="B8" s="473" t="str">
+      <x:c r="B8" s="639" t="str">
         <x:v>/admindraft view-as-shelter</x:v>
       </x:c>
-      <x:c r="C8" s="473" t="str">
+      <x:c r="C8" s="639" t="str">
         <x:v>/shelter/[slug]</x:v>
       </x:c>
-      <x:c r="D8" s="481" t="str">
+      <x:c r="D8" s="732" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E8" s="473" t="str">
+      <x:c r="E8" s="639" t="str">
         <x:v>Shelter-only workspace with profile, dog listings, create dog, bookings, messaging, account settings</x:v>
       </x:c>
-      <x:c r="F8" s="474" t="str">
+      <x:c r="F8" s="639" t="str">
         <x:v>Must never expose PawJai umbrella</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A9" s="472" t="str">
+      <x:c r="A9" s="639" t="str">
         <x:v>Shelter account settings</x:v>
       </x:c>
-      <x:c r="B9" s="473" t="str">
+      <x:c r="B9" s="639" t="str">
         <x:v>none</x:v>
       </x:c>
-      <x:c r="C9" s="473" t="str">
+      <x:c r="C9" s="639" t="str">
         <x:v>/shelter/[slug]/settings</x:v>
       </x:c>
-      <x:c r="D9" s="481" t="str">
+      <x:c r="D9" s="732" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E9" s="473" t="str">
+      <x:c r="E9" s="639" t="str">
         <x:v>Change shelter username, email, and password through real Supabase Auth + shelter_portal_accounts</x:v>
       </x:c>
-      <x:c r="F9" s="474" t="str">
+      <x:c r="F9" s="639" t="str">
         <x:v>Shared-login pilot only; later replace with employee accounts</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="472" t="str">
+      <x:c r="A10" s="639" t="str">
         <x:v>Dog listings inside shelter</x:v>
       </x:c>
-      <x:c r="B10" s="473" t="str">
+      <x:c r="B10" s="639" t="str">
         <x:v>/admindraft?view=dogs</x:v>
       </x:c>
-      <x:c r="C10" s="473" t="str">
+      <x:c r="C10" s="639" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
       </x:c>
-      <x:c r="D10" s="481" t="str">
+      <x:c r="D10" s="732" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E10" s="473" t="str">
+      <x:c r="E10" s="639" t="str">
         <x:v>Shelter can search and filter its own dogs</x:v>
       </x:c>
-      <x:c r="F10" s="474" t="str">
+      <x:c r="F10" s="639" t="str">
         <x:v>Open public dog profile is allowed to go to /dogs/[id]</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="472" t="str">
+      <x:c r="A11" s="639" t="str">
         <x:v>Create dog</x:v>
       </x:c>
-      <x:c r="B11" s="473" t="str">
+      <x:c r="B11" s="639" t="str">
         <x:v>/admindraft/dog-creation?shelter=:id</x:v>
       </x:c>
-      <x:c r="C11" s="473" t="str">
+      <x:c r="C11" s="639" t="str">
         <x:v>/shelter/[slug]/dogs/new</x:v>
       </x:c>
-      <x:c r="D11" s="481" t="str">
+      <x:c r="D11" s="732" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E11" s="473" t="str">
+      <x:c r="E11" s="639" t="str">
         <x:v>Reuses same live dog create form and buckets</x:v>
       </x:c>
-      <x:c r="F11" s="474" t="str">
+      <x:c r="F11" s="639" t="str">
         <x:v>Exit/success returns to /shelter/[slug]?view=dogs</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="472" t="str">
+      <x:c r="A12" s="639" t="str">
         <x:v>Edit dog</x:v>
       </x:c>
-      <x:c r="B12" s="473" t="str">
+      <x:c r="B12" s="639" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="C12" s="473" t="str">
+      <x:c r="C12" s="639" t="str">
         <x:v>/shelter/[slug]/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D12" s="481" t="str">
+      <x:c r="D12" s="732" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E12" s="473" t="str">
+      <x:c r="E12" s="639" t="str">
         <x:v>Reuses same live dog edit form, photos, traits, and storage</x:v>
       </x:c>
-      <x:c r="F12" s="474" t="str">
+      <x:c r="F12" s="639" t="str">
         <x:v>Dog must belong to logged-in shelter</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="472" t="str">
+      <x:c r="A13" s="639" t="str">
         <x:v>Public dog profile</x:v>
       </x:c>
-      <x:c r="B13" s="473" t="str">
+      <x:c r="B13" s="639" t="str">
         <x:v>/dogs/[id]</x:v>
       </x:c>
-      <x:c r="C13" s="473" t="str">
+      <x:c r="C13" s="639" t="str">
         <x:v>/dogs/[id]</x:v>
       </x:c>
-      <x:c r="D13" s="481" t="str">
+      <x:c r="D13" s="732" t="str">
         <x:v>Shared exception</x:v>
       </x:c>
-      <x:c r="E13" s="473" t="str">
+      <x:c r="E13" s="639" t="str">
         <x:v>Public adopter-facing profile</x:v>
       </x:c>
-      <x:c r="F13" s="474" t="str">
+      <x:c r="F13" s="639" t="str">
         <x:v>Only allowed cross-over from shelter portal to public UX</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="472" t="str">
+      <x:c r="A14" s="639" t="str">
         <x:v>Booking list</x:v>
       </x:c>
-      <x:c r="B14" s="473" t="str">
+      <x:c r="B14" s="639" t="str">
         <x:v>/admindraft?view=bookings</x:v>
       </x:c>
-      <x:c r="C14" s="473" t="str">
+      <x:c r="C14" s="639" t="str">
         <x:v>/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="D14" s="481" t="str">
+      <x:c r="D14" s="732" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
-      <x:c r="E14" s="473" t="str">
+      <x:c r="E14" s="639" t="str">
         <x:v>Shelter booking list remains inside shelter workspace</x:v>
       </x:c>
-      <x:c r="F14" s="474" t="str">
+      <x:c r="F14" s="639" t="str">
         <x:v>Links open shared /booking detail with safe returnTo</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A15" s="472" t="str">
+      <x:c r="A15" s="639" t="str">
         <x:v>Booking detail</x:v>
       </x:c>
-      <x:c r="B15" s="473" t="str">
+      <x:c r="B15" s="639" t="str">
         <x:v>/admindraft/bookings/[id]</x:v>
       </x:c>
-      <x:c r="C15" s="473" t="str">
+      <x:c r="C15" s="639" t="str">
         <x:v>/booking/[id]</x:v>
       </x:c>
-      <x:c r="D15" s="481" t="str">
+      <x:c r="D15" s="732" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
-      <x:c r="E15" s="473" t="str">
+      <x:c r="E15" s="639" t="str">
         <x:v>Single internal booking detail page for PawJai admin and linked shelter</x:v>
       </x:c>
-      <x:c r="F15" s="474" t="str">
+      <x:c r="F15" s="639" t="str">
         <x:v>No new SQL table; reads same appointments/adopters/dogs/shelters</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="472" t="str">
+      <x:c r="A16" s="639" t="str">
         <x:v>Visitor profile / verification</x:v>
       </x:c>
-      <x:c r="B16" s="473" t="str">
+      <x:c r="B16" s="639" t="str">
         <x:v>/admindraft/bookings/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="C16" s="473" t="str">
+      <x:c r="C16" s="639" t="str">
         <x:v>/booking/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="D16" s="481" t="str">
+      <x:c r="D16" s="732" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
-      <x:c r="E16" s="473" t="str">
+      <x:c r="E16" s="639" t="str">
         <x:v>Single internal visitor profile and verification document page</x:v>
       </x:c>
-      <x:c r="F16" s="474" t="str">
+      <x:c r="F16" s="639" t="str">
         <x:v>Back links use safe returnTo</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="472" t="str">
+      <x:c r="A17" s="639" t="str">
         <x:v>QR check-in</x:v>
       </x:c>
-      <x:c r="B17" s="473" t="str">
+      <x:c r="B17" s="639" t="str">
         <x:v>/admindraft/bookings/check-in</x:v>
       </x:c>
-      <x:c r="C17" s="473" t="str">
+      <x:c r="C17" s="639" t="str">
         <x:v>/booking/check-in</x:v>
       </x:c>
-      <x:c r="D17" s="481" t="str">
+      <x:c r="D17" s="732" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
-      <x:c r="E17" s="473" t="str">
+      <x:c r="E17" s="639" t="str">
         <x:v>QR token resolves to shared booking detail</x:v>
       </x:c>
-      <x:c r="F17" s="474" t="str">
+      <x:c r="F17" s="639" t="str">
         <x:v>Generated QR URLs now use /booking/check-in</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="472" t="str">
+      <x:c r="A18" s="639" t="str">
         <x:v>Messaging</x:v>
       </x:c>
-      <x:c r="B18" s="473" t="str">
+      <x:c r="B18" s="639" t="str">
         <x:v>/admindraft shelter workspace</x:v>
       </x:c>
-      <x:c r="C18" s="473" t="str">
+      <x:c r="C18" s="639" t="str">
         <x:v>/shelter/[slug]?view=messages</x:v>
       </x:c>
-      <x:c r="D18" s="483" t="str">
+      <x:c r="D18" s="734" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E18" s="473" t="str">
+      <x:c r="E18" s="639" t="str">
         <x:v>Messaging is intentionally not completed in this session</x:v>
       </x:c>
-      <x:c r="F18" s="474" t="str">
+      <x:c r="F18" s="639" t="str">
         <x:v>Plan separately with API/provider choice</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="472" t="str">
+      <x:c r="A19" s="639" t="str">
         <x:v>Ads</x:v>
       </x:c>
-      <x:c r="B19" s="473" t="str">
+      <x:c r="B19" s="639" t="str">
         <x:v>/admin/ads</x:v>
       </x:c>
-      <x:c r="C19" s="473" t="str">
+      <x:c r="C19" s="639" t="str">
         <x:v>/admindraft &gt; Ads</x:v>
       </x:c>
-      <x:c r="D19" s="483" t="str">
-        <x:v>Admin-only</x:v>
-      </x:c>
-      <x:c r="E19" s="473" t="str">
-        <x:v>PawJai-managed ads remain inside admin umbrella</x:v>
-      </x:c>
-      <x:c r="F19" s="474" t="str">
-        <x:v>No brand login yet</x:v>
+      <x:c r="D19" s="730" t="str">
+        <x:v>Admin-only partial</x:v>
+      </x:c>
+      <x:c r="E19" s="639" t="str">
+        <x:v>PawJai-managed ads are visible inside the admin umbrella</x:v>
+      </x:c>
+      <x:c r="F19" s="639" t="str">
+        <x:v>Write controls still need draft-native migration</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="475" t="str">
+      <x:c r="A20" s="639" t="str">
         <x:v>About content</x:v>
       </x:c>
-      <x:c r="B20" s="476" t="str">
+      <x:c r="B20" s="639" t="str">
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
-      <x:c r="C20" s="476" t="str">
-        <x:v>/admindraft &gt; About content</x:v>
-      </x:c>
-      <x:c r="D20" s="485" t="str">
-        <x:v>Admin-only</x:v>
-      </x:c>
-      <x:c r="E20" s="476" t="str">
-        <x:v>PawJai public content management</x:v>
-      </x:c>
-      <x:c r="F20" s="477" t="str">
-        <x:v>Not visible to shelters</x:v>
+      <x:c r="C20" s="639" t="str">
+        <x:v>/admindraft/pawjaiprofile</x:v>
+      </x:c>
+      <x:c r="D20" s="732" t="str">
+        <x:v>Moved / live</x:v>
+      </x:c>
+      <x:c r="E20" s="639" t="str">
+        <x:v>Full PawJai public content editor and save action</x:v>
+      </x:c>
+      <x:c r="F20" s="639" t="str">
+        <x:v>Uses the same pawjai_profile table and revalidates /about</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="639" t="str">
+        <x:v>Admin accounts</x:v>
+      </x:c>
+      <x:c r="B21" s="639" t="str">
+        <x:v>/admin/accounts</x:v>
+      </x:c>
+      <x:c r="C21" s="639" t="str">
+        <x:v>/admindraft/accounts</x:v>
+      </x:c>
+      <x:c r="D21" s="732" t="str">
+        <x:v>Moved / live</x:v>
+      </x:c>
+      <x:c r="E21" s="639" t="str">
+        <x:v>PawJai/shelter admin account creation and revoke controls</x:v>
+      </x:c>
+      <x:c r="F21" s="639" t="str">
+        <x:v>Uses Supabase Auth, profiles, and shelter_users</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="639" t="str">
+        <x:v>Audit log</x:v>
+      </x:c>
+      <x:c r="B22" s="639" t="str">
+        <x:v>/admin/audit</x:v>
+      </x:c>
+      <x:c r="C22" s="639" t="str">
+        <x:v>/admindraft/audit</x:v>
+      </x:c>
+      <x:c r="D22" s="732" t="str">
+        <x:v>Moved / live</x:v>
+      </x:c>
+      <x:c r="E22" s="639" t="str">
+        <x:v>Privileged admin activity table</x:v>
+      </x:c>
+      <x:c r="F22" s="639" t="str">
+        <x:v>Reads admin_audit_events and scopes by admin context</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update admin draft migration tracker
</commit_message>
<xml_diff>
--- a/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
+++ b/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="Ra329004d8c1e4c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="Rccbb6f959970486c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="3" r:id="R912cb7bc43c14d08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="4" r:id="R0c10d944a4c74c96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="5" r:id="R99a26ce92d8f4833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="6" r:id="Rf7cd2d3c02fc4878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="7" r:id="R2c8ccf797d8146e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="8" r:id="R579aec150b2342f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="9" r:id="R5ef2e7432ee1424c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="10" r:id="R4ee0a127d9954ceb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="11" r:id="Rc2c599a9435a493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="R37ca281a7e5b49fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="R834fc9a42c3a4068"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="3" r:id="R725865e42076487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="4" r:id="R675fdf0a802248b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="5" r:id="Rff2c2854f7fc4e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="6" r:id="R319929d7d4d94681"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="7" r:id="R6ab9f289d2734597"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="8" r:id="R52f9de93ebde443d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="9" r:id="Rd2ee569d37f9409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="10" r:id="Radd1d96d92f74ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="11" r:id="R62718852a80944fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Route Gap Audit" sheetId="12" r:id="Rf1e639c0d5c844a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +27,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="22">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -154,8 +155,14 @@
       <x:color rgb="FF4F4338"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF6F6256"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="113">
+  <x:fills count="121">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -555,6 +562,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7E3E1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F1EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B4D40"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD88C24"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8ECD8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -832,7 +879,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="735">
+  <x:cellXfs count="781">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -2486,6 +2533,82 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="13" fillId="108" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="113" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="114" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="115" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="116" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="117" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="118" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="118" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="119" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="119" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="114" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="114" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="117" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="117" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="116" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="116" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="120" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="120" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="114" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="114" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="115" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="115" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="117" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="117" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="119" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="114" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="117" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="116" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="120" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="114" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="115" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="114" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="117" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="116" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="12" fillId="117" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="13" fillId="116" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="118" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="120" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="120" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="117" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="117" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="114" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="114" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="116" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="116" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="115" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="115" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2513,7 +2636,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6c71fcbcd5df4aac"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2c7c44a5ea9f4781"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2540,7 +2663,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re6d86f2eb7774373"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R91362363a42d4f9d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2778,502 +2901,502 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="16">
-      <x:c r="A2" s="691" t="str">
+      <x:c r="A2" s="735" t="str">
         <x:v>Admin gate / password</x:v>
       </x:c>
-      <x:c r="B2" s="691" t="str">
+      <x:c r="B2" s="735" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="C2" s="691" t="str">
+      <x:c r="C2" s="735" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D2" s="692" t="str">
+      <x:c r="D2" s="736" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E2" s="691" t="str">
+      <x:c r="E2" s="735" t="str">
         <x:v>Keep temporary phrase gate until real login logic</x:v>
       </x:c>
-      <x:c r="F2" s="693" t="str">
+      <x:c r="F2" s="737" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="16">
-      <x:c r="A3" s="691" t="str">
+      <x:c r="A3" s="735" t="str">
         <x:v>Main PawJai admin umbrella</x:v>
       </x:c>
-      <x:c r="B3" s="691" t="str">
+      <x:c r="B3" s="735" t="str">
         <x:v>scattered across /admin/*</x:v>
       </x:c>
-      <x:c r="C3" s="691" t="str">
+      <x:c r="C3" s="735" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D3" s="692" t="str">
+      <x:c r="D3" s="736" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E3" s="691" t="str">
+      <x:c r="E3" s="735" t="str">
         <x:v>About, Accounts, and Audit now have draft-native pages; Ads write controls and Messaging remain the main gaps</x:v>
       </x:c>
-      <x:c r="F3" s="694" t="str">
+      <x:c r="F3" s="738" t="str">
         <x:v>High</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="16">
-      <x:c r="A4" s="691" t="str">
+      <x:c r="A4" s="735" t="str">
         <x:v>Partner shelters overview</x:v>
       </x:c>
-      <x:c r="B4" s="691" t="str">
+      <x:c r="B4" s="735" t="str">
         <x:v>mostly inside /admin/bookings</x:v>
       </x:c>
-      <x:c r="C4" s="691" t="str">
+      <x:c r="C4" s="735" t="str">
         <x:v>/admindraft &gt; Partner shelters</x:v>
       </x:c>
-      <x:c r="D4" s="692" t="str">
+      <x:c r="D4" s="736" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E4" s="691" t="str">
+      <x:c r="E4" s="735" t="str">
         <x:v>Add deeper shelter metrics later if wanted</x:v>
       </x:c>
-      <x:c r="F4" s="695" t="str">
+      <x:c r="F4" s="739" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="16">
-      <x:c r="A5" s="691" t="str">
+      <x:c r="A5" s="735" t="str">
         <x:v>Shelter profile edit</x:v>
       </x:c>
-      <x:c r="B5" s="691" t="str">
+      <x:c r="B5" s="735" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C5" s="691" t="str">
+      <x:c r="C5" s="735" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D5" s="692" t="str">
+      <x:c r="D5" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E5" s="691" t="str">
+      <x:c r="E5" s="735" t="str">
         <x:v>Real-world save testing per shelter</x:v>
       </x:c>
-      <x:c r="F5" s="692" t="str">
+      <x:c r="F5" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16">
-      <x:c r="A6" s="691" t="str">
+      <x:c r="A6" s="735" t="str">
         <x:v>Shelter logo upload</x:v>
       </x:c>
-      <x:c r="B6" s="691" t="str">
+      <x:c r="B6" s="735" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C6" s="691" t="str">
+      <x:c r="C6" s="735" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D6" s="692" t="str">
+      <x:c r="D6" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E6" s="691" t="str">
+      <x:c r="E6" s="735" t="str">
         <x:v>Real-world upload testing per shelter</x:v>
       </x:c>
-      <x:c r="F6" s="692" t="str">
+      <x:c r="F6" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="16">
-      <x:c r="A7" s="691" t="str">
+      <x:c r="A7" s="735" t="str">
         <x:v>Shelter donation details</x:v>
       </x:c>
-      <x:c r="B7" s="691" t="str">
+      <x:c r="B7" s="735" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C7" s="691" t="str">
+      <x:c r="C7" s="735" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D7" s="692" t="str">
+      <x:c r="D7" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E7" s="691" t="str">
+      <x:c r="E7" s="735" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F7" s="692" t="str">
+      <x:c r="F7" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="16">
-      <x:c r="A8" s="691" t="str">
+      <x:c r="A8" s="735" t="str">
         <x:v>Shelter operating hours</x:v>
       </x:c>
-      <x:c r="B8" s="691" t="str">
+      <x:c r="B8" s="735" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C8" s="691" t="str">
+      <x:c r="C8" s="735" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D8" s="692" t="str">
+      <x:c r="D8" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E8" s="691" t="str">
+      <x:c r="E8" s="735" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F8" s="692" t="str">
+      <x:c r="F8" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
-      <x:c r="A9" s="691" t="str">
+      <x:c r="A9" s="735" t="str">
         <x:v>Shelter blockout dates</x:v>
       </x:c>
-      <x:c r="B9" s="691" t="str">
+      <x:c r="B9" s="735" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C9" s="691" t="str">
+      <x:c r="C9" s="735" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D9" s="692" t="str">
+      <x:c r="D9" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E9" s="691" t="str">
+      <x:c r="E9" s="735" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F9" s="692" t="str">
+      <x:c r="F9" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32">
-      <x:c r="A10" s="691" t="str">
+      <x:c r="A10" s="735" t="str">
         <x:v>Shelter dog listings</x:v>
       </x:c>
-      <x:c r="B10" s="691" t="str">
+      <x:c r="B10" s="735" t="str">
         <x:v>/admin/bookings?view=dogs, /admin/listings</x:v>
       </x:c>
-      <x:c r="C10" s="691" t="str">
+      <x:c r="C10" s="735" t="str">
         <x:v>/admindraft &gt; Dog listings</x:v>
       </x:c>
-      <x:c r="D10" s="692" t="str">
+      <x:c r="D10" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E10" s="691" t="str">
+      <x:c r="E10" s="735" t="str">
         <x:v>Search/status view is enough for shelter listing management; edit remains separate</x:v>
       </x:c>
-      <x:c r="F10" s="692" t="str">
+      <x:c r="F10" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="16">
-      <x:c r="A11" s="691" t="str">
+      <x:c r="A11" s="735" t="str">
         <x:v>Create dog listing</x:v>
       </x:c>
-      <x:c r="B11" s="691" t="str">
+      <x:c r="B11" s="735" t="str">
         <x:v>/admin, /admin/dogs/new</x:v>
       </x:c>
-      <x:c r="C11" s="691" t="str">
+      <x:c r="C11" s="735" t="str">
         <x:v>/admindraft/dog-creation</x:v>
       </x:c>
-      <x:c r="D11" s="692" t="str">
+      <x:c r="D11" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E11" s="691" t="str">
+      <x:c r="E11" s="735" t="str">
         <x:v>Draft-native create flow exists; real-world save/photo testing remains</x:v>
       </x:c>
-      <x:c r="F11" s="692" t="str">
+      <x:c r="F11" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32">
-      <x:c r="A12" s="691" t="str">
+      <x:c r="A12" s="735" t="str">
         <x:v>Edit dog listing</x:v>
       </x:c>
-      <x:c r="B12" s="691" t="str">
+      <x:c r="B12" s="735" t="str">
         <x:v>/admin/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="C12" s="691" t="str">
+      <x:c r="C12" s="735" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D12" s="692" t="str">
+      <x:c r="D12" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E12" s="691" t="str">
+      <x:c r="E12" s="735" t="str">
         <x:v>Draft-native edit route reuses the full old edit form; real-world save/photo testing remains</x:v>
       </x:c>
-      <x:c r="F12" s="692" t="str">
+      <x:c r="F12" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="32">
-      <x:c r="A13" s="691" t="str">
+      <x:c r="A13" s="735" t="str">
         <x:v>Dog photos / cover order</x:v>
       </x:c>
-      <x:c r="B13" s="691" t="str">
+      <x:c r="B13" s="735" t="str">
         <x:v>/admin, /admin/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="C13" s="691" t="str">
+      <x:c r="C13" s="735" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D13" s="692" t="str">
+      <x:c r="D13" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E13" s="691" t="str">
+      <x:c r="E13" s="735" t="str">
         <x:v>Edit route now includes existing upload, reorder, cover, and remove tools</x:v>
       </x:c>
-      <x:c r="F13" s="692" t="str">
+      <x:c r="F13" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16">
-      <x:c r="A14" s="691" t="str">
+      <x:c r="A14" s="735" t="str">
         <x:v>All dog listings across shelters</x:v>
       </x:c>
-      <x:c r="B14" s="691" t="str">
+      <x:c r="B14" s="735" t="str">
         <x:v>/admin/listings</x:v>
       </x:c>
-      <x:c r="C14" s="691" t="str">
+      <x:c r="C14" s="735" t="str">
         <x:v>/admindraft &gt; All dog listings</x:v>
       </x:c>
-      <x:c r="D14" s="692" t="str">
+      <x:c r="D14" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E14" s="691" t="str">
+      <x:c r="E14" s="735" t="str">
         <x:v>Filters exist and edit buttons now open draft-native dog edit pages</x:v>
       </x:c>
-      <x:c r="F14" s="692" t="str">
+      <x:c r="F14" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32">
-      <x:c r="A15" s="691" t="str">
+      <x:c r="A15" s="735" t="str">
         <x:v>Booking visits list</x:v>
       </x:c>
-      <x:c r="B15" s="691" t="str">
+      <x:c r="B15" s="735" t="str">
         <x:v>/admin/bookings</x:v>
       </x:c>
-      <x:c r="C15" s="691" t="str">
+      <x:c r="C15" s="735" t="str">
         <x:v>/admindraft &gt; Bookings</x:v>
       </x:c>
-      <x:c r="D15" s="692" t="str">
+      <x:c r="D15" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E15" s="691" t="str">
+      <x:c r="E15" s="735" t="str">
         <x:v>Old low-friction booking card flow duplicated; real staff testing remains</x:v>
       </x:c>
-      <x:c r="F15" s="692" t="str">
+      <x:c r="F15" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="32">
-      <x:c r="A16" s="691" t="str">
+      <x:c r="A16" s="735" t="str">
         <x:v>Booking decision actions</x:v>
       </x:c>
-      <x:c r="B16" s="691" t="str">
+      <x:c r="B16" s="735" t="str">
         <x:v>/admin/bookings, /admin/bookings/[id]</x:v>
       </x:c>
-      <x:c r="C16" s="691" t="str">
+      <x:c r="C16" s="735" t="str">
         <x:v>/admindraft &gt; Bookings</x:v>
       </x:c>
-      <x:c r="D16" s="692" t="str">
+      <x:c r="D16" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E16" s="691" t="str">
+      <x:c r="E16" s="735" t="str">
         <x:v>Accept, deny, and date-change actions are draft-native; final status edge cases can be polished later</x:v>
       </x:c>
-      <x:c r="F16" s="692" t="str">
+      <x:c r="F16" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="16">
-      <x:c r="A17" s="691" t="str">
+      <x:c r="A17" s="735" t="str">
         <x:v>Booking detail page</x:v>
       </x:c>
-      <x:c r="B17" s="691" t="str">
+      <x:c r="B17" s="735" t="str">
         <x:v>/admin/bookings/[id]</x:v>
       </x:c>
-      <x:c r="C17" s="691" t="str">
+      <x:c r="C17" s="735" t="str">
         <x:v>/admindraft/bookings/[id]</x:v>
       </x:c>
-      <x:c r="D17" s="692" t="str">
+      <x:c r="D17" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E17" s="691" t="str">
+      <x:c r="E17" s="735" t="str">
         <x:v>QR scan can land here; refine isolated detail page only if needed</x:v>
       </x:c>
-      <x:c r="F17" s="692" t="str">
+      <x:c r="F17" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="16">
-      <x:c r="A18" s="691" t="str">
+      <x:c r="A18" s="735" t="str">
         <x:v>QR check-in</x:v>
       </x:c>
-      <x:c r="B18" s="691" t="str">
+      <x:c r="B18" s="735" t="str">
         <x:v>/admin/bookings/check-in</x:v>
       </x:c>
-      <x:c r="C18" s="691" t="str">
+      <x:c r="C18" s="735" t="str">
         <x:v>/admindraft/bookings/check-in</x:v>
       </x:c>
-      <x:c r="D18" s="692" t="str">
+      <x:c r="D18" s="736" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E18" s="691" t="str">
+      <x:c r="E18" s="735" t="str">
         <x:v>Needs real QR/camera device testing</x:v>
       </x:c>
-      <x:c r="F18" s="695" t="str">
+      <x:c r="F18" s="739" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32">
-      <x:c r="A19" s="691" t="str">
+      <x:c r="A19" s="735" t="str">
         <x:v>Visitor profile</x:v>
       </x:c>
-      <x:c r="B19" s="691" t="str">
+      <x:c r="B19" s="735" t="str">
         <x:v>/admin/bookings/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="C19" s="691" t="str">
+      <x:c r="C19" s="735" t="str">
         <x:v>/admindraft/bookings/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="D19" s="692" t="str">
+      <x:c r="D19" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E19" s="691" t="str">
+      <x:c r="E19" s="735" t="str">
         <x:v>Draft-native profile/documents view exists; real document review testing remains</x:v>
       </x:c>
-      <x:c r="F19" s="692" t="str">
+      <x:c r="F19" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="32">
-      <x:c r="A20" s="691" t="str">
+      <x:c r="A20" s="735" t="str">
         <x:v>Shelter messaging</x:v>
       </x:c>
-      <x:c r="B20" s="691" t="str">
+      <x:c r="B20" s="735" t="str">
         <x:v>/admin/bookings?view=messages</x:v>
       </x:c>
-      <x:c r="C20" s="691" t="str">
+      <x:c r="C20" s="735" t="str">
         <x:v>/admindraft &gt; Messaging</x:v>
       </x:c>
-      <x:c r="D20" s="694" t="str">
+      <x:c r="D20" s="738" t="str">
         <x:v>Visual only</x:v>
       </x:c>
-      <x:c r="E20" s="691" t="str">
+      <x:c r="E20" s="735" t="str">
         <x:v>Transfer real message thread and send reply in separate messaging session</x:v>
       </x:c>
-      <x:c r="F20" s="694" t="str">
+      <x:c r="F20" s="738" t="str">
         <x:v>High</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16">
-      <x:c r="A21" s="691" t="str">
+      <x:c r="A21" s="735" t="str">
         <x:v>Ads management</x:v>
       </x:c>
-      <x:c r="B21" s="691" t="str">
+      <x:c r="B21" s="735" t="str">
         <x:v>/admin/ads</x:v>
       </x:c>
-      <x:c r="C21" s="691" t="str">
+      <x:c r="C21" s="735" t="str">
         <x:v>/admindraft &gt; Ads</x:v>
       </x:c>
-      <x:c r="D21" s="695" t="str">
+      <x:c r="D21" s="739" t="str">
         <x:v>Read only</x:v>
       </x:c>
-      <x:c r="E21" s="691" t="str">
+      <x:c r="E21" s="735" t="str">
         <x:v>Transfer create ad, edit dates, pause/resume, delete</x:v>
       </x:c>
-      <x:c r="F21" s="695" t="str">
+      <x:c r="F21" s="739" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="16">
-      <x:c r="A22" s="691" t="str">
+      <x:c r="A22" s="735" t="str">
         <x:v>About content</x:v>
       </x:c>
-      <x:c r="B22" s="691" t="str">
+      <x:c r="B22" s="735" t="str">
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
-      <x:c r="C22" s="691" t="str">
+      <x:c r="C22" s="735" t="str">
         <x:v>/admindraft/pawjaiprofile</x:v>
       </x:c>
-      <x:c r="D22" s="692" t="str">
+      <x:c r="D22" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E22" s="691" t="str">
+      <x:c r="E22" s="735" t="str">
         <x:v>Draft-native About editor exists and saves through the same pawjai_profile table; live save smoke test remains</x:v>
       </x:c>
-      <x:c r="F22" s="692" t="str">
+      <x:c r="F22" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="16">
-      <x:c r="A23" s="691" t="str">
+      <x:c r="A23" s="735" t="str">
         <x:v>Admin accounts</x:v>
       </x:c>
-      <x:c r="B23" s="691" t="str">
+      <x:c r="B23" s="735" t="str">
         <x:v>/admin/accounts</x:v>
       </x:c>
-      <x:c r="C23" s="691" t="str">
+      <x:c r="C23" s="735" t="str">
         <x:v>/admindraft/accounts</x:v>
       </x:c>
-      <x:c r="D23" s="692" t="str">
+      <x:c r="D23" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E23" s="691" t="str">
+      <x:c r="E23" s="735" t="str">
         <x:v>Draft-native account creation/revoke exists and uses the same Supabase Auth, profiles, and shelter_users logic</x:v>
       </x:c>
-      <x:c r="F23" s="692" t="str">
+      <x:c r="F23" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="16">
-      <x:c r="A24" s="691" t="str">
+      <x:c r="A24" s="735" t="str">
         <x:v>Audit log</x:v>
       </x:c>
-      <x:c r="B24" s="691" t="str">
+      <x:c r="B24" s="735" t="str">
         <x:v>/admin/audit</x:v>
       </x:c>
-      <x:c r="C24" s="691" t="str">
+      <x:c r="C24" s="735" t="str">
         <x:v>/admindraft/audit</x:v>
       </x:c>
-      <x:c r="D24" s="692" t="str">
+      <x:c r="D24" s="736" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E24" s="691" t="str">
+      <x:c r="E24" s="735" t="str">
         <x:v>Draft-native audit table exists; keep testing with real admin changes</x:v>
       </x:c>
-      <x:c r="F24" s="692" t="str">
+      <x:c r="F24" s="736" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="16">
-      <x:c r="A25" s="691" t="str">
+      <x:c r="A25" s="735" t="str">
         <x:v>Admin login page</x:v>
       </x:c>
-      <x:c r="B25" s="691" t="str">
+      <x:c r="B25" s="735" t="str">
         <x:v>/admin/login</x:v>
       </x:c>
-      <x:c r="C25" s="691" t="str">
+      <x:c r="C25" s="735" t="str">
         <x:v>temporary phrase gate</x:v>
       </x:c>
-      <x:c r="D25" s="695" t="str">
+      <x:c r="D25" s="739" t="str">
         <x:v>Temporary</x:v>
       </x:c>
-      <x:c r="E25" s="691" t="str">
+      <x:c r="E25" s="735" t="str">
         <x:v>Later replace phrase gates with real auth</x:v>
       </x:c>
-      <x:c r="F25" s="693" t="str">
+      <x:c r="F25" s="737" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="16">
-      <x:c r="A26" s="691" t="str">
+      <x:c r="A26" s="735" t="str">
         <x:v>Legacy draft alias</x:v>
       </x:c>
-      <x:c r="B26" s="691" t="str">
+      <x:c r="B26" s="735" t="str">
         <x:v>/admin/reorg-draft</x:v>
       </x:c>
-      <x:c r="C26" s="691" t="str">
+      <x:c r="C26" s="735" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D26" s="692" t="str">
+      <x:c r="D26" s="736" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E26" s="691" t="str">
+      <x:c r="E26" s="735" t="str">
         <x:v>Remove after /admindraft becomes canonical</x:v>
       </x:c>
-      <x:c r="F26" s="693" t="str">
+      <x:c r="F26" s="737" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
@@ -3534,7 +3657,338 @@
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ac0f56048d54379"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra19b113cd2204d8a"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="54" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="770" t="str">
+        <x:v>Old /admin route coverage into /admindraft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="757" t="str">
+        <x:v>Use this as the quick answer to: what still exists only in old admin? Right now the main remaining migration is Ads write controls; Messaging remains a separate shelter/adopter product workflow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="758" t="str">
+        <x:v>Old admin route</x:v>
+      </x:c>
+      <x:c r="B4" s="758" t="str">
+        <x:v>Draft / shared route</x:v>
+      </x:c>
+      <x:c r="C4" s="758" t="str">
+        <x:v>Coverage</x:v>
+      </x:c>
+      <x:c r="D4" s="758" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E4" s="758" t="str">
+        <x:v>What remains</x:v>
+      </x:c>
+      <x:c r="F4" s="758" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="639" t="str">
+        <x:v>/admin</x:v>
+      </x:c>
+      <x:c r="B5" s="639" t="str">
+        <x:v>/admindraft</x:v>
+      </x:c>
+      <x:c r="C5" s="639" t="str">
+        <x:v>PawJai umbrella dashboard</x:v>
+      </x:c>
+      <x:c r="D5" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E5" s="639" t="str">
+        <x:v>Keep old /admin live until final cutover</x:v>
+      </x:c>
+      <x:c r="F5" s="780" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="639" t="str">
+        <x:v>/admin/listings</x:v>
+      </x:c>
+      <x:c r="B6" s="639" t="str">
+        <x:v>/admindraft?view=dogs</x:v>
+      </x:c>
+      <x:c r="C6" s="639" t="str">
+        <x:v>All dog listings across shelters</x:v>
+      </x:c>
+      <x:c r="D6" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E6" s="639" t="str">
+        <x:v>None for draft parity</x:v>
+      </x:c>
+      <x:c r="F6" s="776" t="str">
+        <x:v>Done-ish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="639" t="str">
+        <x:v>/admin/dogs/new</x:v>
+      </x:c>
+      <x:c r="B7" s="639" t="str">
+        <x:v>/admindraft/dog-creation and /admindraft/dogs/new</x:v>
+      </x:c>
+      <x:c r="C7" s="639" t="str">
+        <x:v>Dog create workflow</x:v>
+      </x:c>
+      <x:c r="D7" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E7" s="639" t="str">
+        <x:v>Continue real photo/upload smoke tests</x:v>
+      </x:c>
+      <x:c r="F7" s="776" t="str">
+        <x:v>Done-ish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="639" t="str">
+        <x:v>/admin/dogs/[id]/edit</x:v>
+      </x:c>
+      <x:c r="B8" s="639" t="str">
+        <x:v>/admindraft/dogs/[id]/edit</x:v>
+      </x:c>
+      <x:c r="C8" s="639" t="str">
+        <x:v>Dog edit workflow</x:v>
+      </x:c>
+      <x:c r="D8" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E8" s="639" t="str">
+        <x:v>Continue real save/photo smoke tests</x:v>
+      </x:c>
+      <x:c r="F8" s="776" t="str">
+        <x:v>Done-ish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="639" t="str">
+        <x:v>/admin/bookings</x:v>
+      </x:c>
+      <x:c r="B9" s="639" t="str">
+        <x:v>/admindraft?view=bookings</x:v>
+      </x:c>
+      <x:c r="C9" s="639" t="str">
+        <x:v>Booking list, filters, inline decisions</x:v>
+      </x:c>
+      <x:c r="D9" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E9" s="639" t="str">
+        <x:v>Real staff booking smoke tests only</x:v>
+      </x:c>
+      <x:c r="F9" s="776" t="str">
+        <x:v>Done-ish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="639" t="str">
+        <x:v>/admin/bookings/[id]</x:v>
+      </x:c>
+      <x:c r="B10" s="639" t="str">
+        <x:v>/admindraft/bookings/[id] and /booking/[id]</x:v>
+      </x:c>
+      <x:c r="C10" s="639" t="str">
+        <x:v>Booking detail / QR landing</x:v>
+      </x:c>
+      <x:c r="D10" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E10" s="639" t="str">
+        <x:v>Phone QR test still recommended</x:v>
+      </x:c>
+      <x:c r="F10" s="774" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="639" t="str">
+        <x:v>/admin/bookings/[id]/visitor-profile</x:v>
+      </x:c>
+      <x:c r="B11" s="639" t="str">
+        <x:v>/admindraft/bookings/[id]/visitor-profile and /booking/[id]/visitor-profile</x:v>
+      </x:c>
+      <x:c r="C11" s="639" t="str">
+        <x:v>Visitor profile and verification documents</x:v>
+      </x:c>
+      <x:c r="D11" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E11" s="639" t="str">
+        <x:v>Real document review smoke test</x:v>
+      </x:c>
+      <x:c r="F11" s="776" t="str">
+        <x:v>Done-ish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="639" t="str">
+        <x:v>/admin/bookings/check-in</x:v>
+      </x:c>
+      <x:c r="B12" s="639" t="str">
+        <x:v>/admindraft/bookings/check-in and /booking/check-in</x:v>
+      </x:c>
+      <x:c r="C12" s="639" t="str">
+        <x:v>QR check-in</x:v>
+      </x:c>
+      <x:c r="D12" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E12" s="639" t="str">
+        <x:v>Real camera/device test</x:v>
+      </x:c>
+      <x:c r="F12" s="774" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="639" t="str">
+        <x:v>/admin/ads</x:v>
+      </x:c>
+      <x:c r="B13" s="639" t="str">
+        <x:v>/admindraft?view=ads</x:v>
+      </x:c>
+      <x:c r="C13" s="639" t="str">
+        <x:v>Ads visibility and filters</x:v>
+      </x:c>
+      <x:c r="D13" s="774" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="E13" s="639" t="str">
+        <x:v>Move create/edit/pause/delete ad controls into draft route</x:v>
+      </x:c>
+      <x:c r="F13" s="778" t="str">
+        <x:v>High</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="639" t="str">
+        <x:v>/admin/pawjaiprofile</x:v>
+      </x:c>
+      <x:c r="B14" s="639" t="str">
+        <x:v>/admindraft/pawjaiprofile</x:v>
+      </x:c>
+      <x:c r="C14" s="639" t="str">
+        <x:v>About content editor</x:v>
+      </x:c>
+      <x:c r="D14" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E14" s="639" t="str">
+        <x:v>Live save smoke test only</x:v>
+      </x:c>
+      <x:c r="F14" s="776" t="str">
+        <x:v>Done-ish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="639" t="str">
+        <x:v>/admin/accounts</x:v>
+      </x:c>
+      <x:c r="B15" s="639" t="str">
+        <x:v>/admindraft/accounts</x:v>
+      </x:c>
+      <x:c r="C15" s="639" t="str">
+        <x:v>PawJai and shelter admin account management</x:v>
+      </x:c>
+      <x:c r="D15" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E15" s="639" t="str">
+        <x:v>Live create/revoke smoke test only</x:v>
+      </x:c>
+      <x:c r="F15" s="776" t="str">
+        <x:v>Done-ish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="639" t="str">
+        <x:v>/admin/audit</x:v>
+      </x:c>
+      <x:c r="B16" s="639" t="str">
+        <x:v>/admindraft/audit</x:v>
+      </x:c>
+      <x:c r="C16" s="639" t="str">
+        <x:v>Audit log</x:v>
+      </x:c>
+      <x:c r="D16" s="776" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E16" s="639" t="str">
+        <x:v>Keep testing after real admin changes</x:v>
+      </x:c>
+      <x:c r="F16" s="776" t="str">
+        <x:v>Done-ish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="639" t="str">
+        <x:v>/admin/login</x:v>
+      </x:c>
+      <x:c r="B17" s="639" t="str">
+        <x:v>/admindraft gate and future real admin auth</x:v>
+      </x:c>
+      <x:c r="C17" s="639" t="str">
+        <x:v>Legacy login</x:v>
+      </x:c>
+      <x:c r="D17" s="774" t="str">
+        <x:v>Temporary</x:v>
+      </x:c>
+      <x:c r="E17" s="639" t="str">
+        <x:v>Replace phrase gate with real admin login later</x:v>
+      </x:c>
+      <x:c r="F17" s="780" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="639" t="str">
+        <x:v>/admin/reorg-draft</x:v>
+      </x:c>
+      <x:c r="B18" s="639" t="str">
+        <x:v>/admindraft</x:v>
+      </x:c>
+      <x:c r="C18" s="639" t="str">
+        <x:v>Legacy draft alias</x:v>
+      </x:c>
+      <x:c r="D18" s="774" t="str">
+        <x:v>Temporary</x:v>
+      </x:c>
+      <x:c r="E18" s="639" t="str">
+        <x:v>Remove after /admindraft replaces old admin</x:v>
+      </x:c>
+      <x:c r="F18" s="780" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -3549,7 +4003,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21">
-      <x:c r="A1" s="697" t="str">
+      <x:c r="A1" s="741" t="str">
         <x:v>PAWJAI Admin Draft Transfer Progress</x:v>
       </x:c>
       <x:c r="B1"/>
@@ -3559,28 +4013,28 @@
       <x:c r="F1"/>
     </x:row>
     <x:row r="3" ht="15">
-      <x:c r="A3" s="714" t="str">
+      <x:c r="A3" s="758" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="714" t="str">
+      <x:c r="B3" s="758" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C3" s="714" t="str">
+      <x:c r="C3" s="758" t="str">
         <x:v>% of workflows</x:v>
       </x:c>
-      <x:c r="D3" s="714" t="str">
+      <x:c r="D3" s="758" t="str">
         <x:v>Meaning</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15">
-      <x:c r="A4" s="721" t="str">
+      <x:c r="A4" s="765" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="B4" s="715" t="n">
+      <x:c r="B4" s="759" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A4)</x:f>
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C4" s="719" t="n">
+      <x:c r="C4" s="763" t="n">
         <x:f>B4/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.68</x:v>
       </x:c>
@@ -3589,14 +4043,14 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="15">
-      <x:c r="A5" s="721" t="str">
+      <x:c r="A5" s="765" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="B5" s="715" t="n">
+      <x:c r="B5" s="759" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A5)</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C5" s="719" t="n">
+      <x:c r="C5" s="763" t="n">
         <x:f>B5/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.2</x:v>
       </x:c>
@@ -3605,14 +4059,14 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="15">
-      <x:c r="A6" s="722" t="str">
+      <x:c r="A6" s="766" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="B6" s="716" t="n">
+      <x:c r="B6" s="760" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C6" s="724" t="n">
+      <x:c r="C6" s="768" t="n">
         <x:f>B6/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3621,14 +4075,14 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="15">
-      <x:c r="A7" s="722" t="str">
+      <x:c r="A7" s="766" t="str">
         <x:v>Read only</x:v>
       </x:c>
-      <x:c r="B7" s="716" t="n">
+      <x:c r="B7" s="760" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A7)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C7" s="724" t="n">
+      <x:c r="C7" s="768" t="n">
         <x:f>B7/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
@@ -3637,14 +4091,14 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="15">
-      <x:c r="A8" s="723" t="str">
+      <x:c r="A8" s="767" t="str">
         <x:v>Visual only</x:v>
       </x:c>
-      <x:c r="B8" s="717" t="n">
+      <x:c r="B8" s="761" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A8)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="725" t="n">
+      <x:c r="C8" s="769" t="n">
         <x:f>B8/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
@@ -3653,14 +4107,14 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="15">
-      <x:c r="A9" s="722" t="str">
+      <x:c r="A9" s="766" t="str">
         <x:v>Temporary</x:v>
       </x:c>
-      <x:c r="B9" s="716" t="n">
+      <x:c r="B9" s="760" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C9" s="724" t="n">
+      <x:c r="C9" s="768" t="n">
         <x:f>B9/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
@@ -3669,14 +4123,14 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="15">
-      <x:c r="A10" s="723" t="str">
+      <x:c r="A10" s="767" t="str">
         <x:v>Missing</x:v>
       </x:c>
-      <x:c r="B10" s="717" t="n">
+      <x:c r="B10" s="761" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C10" s="725" t="n">
+      <x:c r="C10" s="769" t="n">
         <x:f>B10/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3685,51 +4139,51 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="15">
-      <x:c r="A13" s="718" t="str">
+      <x:c r="A13" s="762" t="str">
         <x:v>Metric</x:v>
       </x:c>
-      <x:c r="B13" s="718" t="str">
+      <x:c r="B13" s="762" t="str">
         <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15">
-      <x:c r="A14" s="721" t="str">
+      <x:c r="A14" s="765" t="str">
         <x:v>Functional workflows</x:v>
       </x:c>
-      <x:c r="B14" s="715" t="n">
+      <x:c r="B14" s="759" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Functional")</x:f>
         <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15">
-      <x:c r="A15" s="721" t="str">
+      <x:c r="A15" s="765" t="str">
         <x:v>Functional + Exists</x:v>
       </x:c>
-      <x:c r="B15" s="719" t="n">
+      <x:c r="B15" s="763" t="n">
         <x:f>(COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Functional")+COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Exists"))/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.88</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15">
-      <x:c r="A16" s="723" t="str">
+      <x:c r="A16" s="767" t="str">
         <x:v>Still high priority</x:v>
       </x:c>
-      <x:c r="B16" s="717" t="n">
+      <x:c r="B16" s="761" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$F$2:$F$26,"High")</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15">
-      <x:c r="A17" s="720" t="str">
+      <x:c r="A17" s="764" t="str">
         <x:v>Total workflows</x:v>
       </x:c>
-      <x:c r="B17" s="720" t="n">
+      <x:c r="B17" s="764" t="n">
         <x:f>COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
-      <x:c r="A20" s="713" t="str">
+      <x:c r="A20" s="757" t="str">
         <x:v>Current read: shelter profile, dog creation/listing, booking flows, About content, Accounts, and Audit are now draft-native. Messaging is intentionally left for a separate session; Ads still needs write controls moved.</x:v>
       </x:c>
       <x:c r="B20"/>
@@ -3760,7 +4214,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
-      <x:c r="A1" s="726" t="str">
+      <x:c r="A1" s="770" t="str">
         <x:v>PAWJAI Admin -&gt; Shelter -&gt; Booking Route Migration Map</x:v>
       </x:c>
       <x:c r="B1"/>
@@ -3770,7 +4224,7 @@
       <x:c r="F1"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="728" t="str">
+      <x:c r="A2" s="772" t="str">
         <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
       </x:c>
       <x:c r="B2"/>
@@ -3781,22 +4235,22 @@
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="714" t="str">
+      <x:c r="A4" s="758" t="str">
         <x:v>Workflow</x:v>
       </x:c>
-      <x:c r="B4" s="714" t="str">
+      <x:c r="B4" s="758" t="str">
         <x:v>Old / current source</x:v>
       </x:c>
-      <x:c r="C4" s="714" t="str">
+      <x:c r="C4" s="758" t="str">
         <x:v>New canonical route</x:v>
       </x:c>
-      <x:c r="D4" s="714" t="str">
+      <x:c r="D4" s="758" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="E4" s="714" t="str">
+      <x:c r="E4" s="758" t="str">
         <x:v>What it does</x:v>
       </x:c>
-      <x:c r="F4" s="714" t="str">
+      <x:c r="F4" s="758" t="str">
         <x:v>Notes / next step</x:v>
       </x:c>
     </x:row>
@@ -3810,7 +4264,7 @@
       <x:c r="C5" s="639" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="D5" s="730" t="str">
+      <x:c r="D5" s="774" t="str">
         <x:v>Legacy active</x:v>
       </x:c>
       <x:c r="E5" s="639" t="str">
@@ -3830,7 +4284,7 @@
       <x:c r="C6" s="639" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D6" s="732" t="str">
+      <x:c r="D6" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E6" s="639" t="str">
@@ -3850,7 +4304,7 @@
       <x:c r="C7" s="639" t="str">
         <x:v>/shelter</x:v>
       </x:c>
-      <x:c r="D7" s="732" t="str">
+      <x:c r="D7" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E7" s="639" t="str">
@@ -3870,7 +4324,7 @@
       <x:c r="C8" s="639" t="str">
         <x:v>/shelter/[slug]</x:v>
       </x:c>
-      <x:c r="D8" s="732" t="str">
+      <x:c r="D8" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E8" s="639" t="str">
@@ -3890,7 +4344,7 @@
       <x:c r="C9" s="639" t="str">
         <x:v>/shelter/[slug]/settings</x:v>
       </x:c>
-      <x:c r="D9" s="732" t="str">
+      <x:c r="D9" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E9" s="639" t="str">
@@ -3910,7 +4364,7 @@
       <x:c r="C10" s="639" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
       </x:c>
-      <x:c r="D10" s="732" t="str">
+      <x:c r="D10" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E10" s="639" t="str">
@@ -3930,7 +4384,7 @@
       <x:c r="C11" s="639" t="str">
         <x:v>/shelter/[slug]/dogs/new</x:v>
       </x:c>
-      <x:c r="D11" s="732" t="str">
+      <x:c r="D11" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E11" s="639" t="str">
@@ -3950,7 +4404,7 @@
       <x:c r="C12" s="639" t="str">
         <x:v>/shelter/[slug]/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D12" s="732" t="str">
+      <x:c r="D12" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E12" s="639" t="str">
@@ -3970,7 +4424,7 @@
       <x:c r="C13" s="639" t="str">
         <x:v>/dogs/[id]</x:v>
       </x:c>
-      <x:c r="D13" s="732" t="str">
+      <x:c r="D13" s="776" t="str">
         <x:v>Shared exception</x:v>
       </x:c>
       <x:c r="E13" s="639" t="str">
@@ -3990,7 +4444,7 @@
       <x:c r="C14" s="639" t="str">
         <x:v>/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="D14" s="732" t="str">
+      <x:c r="D14" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E14" s="639" t="str">
@@ -4010,7 +4464,7 @@
       <x:c r="C15" s="639" t="str">
         <x:v>/booking/[id]</x:v>
       </x:c>
-      <x:c r="D15" s="732" t="str">
+      <x:c r="D15" s="776" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E15" s="639" t="str">
@@ -4030,7 +4484,7 @@
       <x:c r="C16" s="639" t="str">
         <x:v>/booking/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="D16" s="732" t="str">
+      <x:c r="D16" s="776" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E16" s="639" t="str">
@@ -4050,7 +4504,7 @@
       <x:c r="C17" s="639" t="str">
         <x:v>/booking/check-in</x:v>
       </x:c>
-      <x:c r="D17" s="732" t="str">
+      <x:c r="D17" s="776" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E17" s="639" t="str">
@@ -4070,7 +4524,7 @@
       <x:c r="C18" s="639" t="str">
         <x:v>/shelter/[slug]?view=messages</x:v>
       </x:c>
-      <x:c r="D18" s="734" t="str">
+      <x:c r="D18" s="778" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="E18" s="639" t="str">
@@ -4090,7 +4544,7 @@
       <x:c r="C19" s="639" t="str">
         <x:v>/admindraft &gt; Ads</x:v>
       </x:c>
-      <x:c r="D19" s="730" t="str">
+      <x:c r="D19" s="774" t="str">
         <x:v>Admin-only partial</x:v>
       </x:c>
       <x:c r="E19" s="639" t="str">
@@ -4110,7 +4564,7 @@
       <x:c r="C20" s="639" t="str">
         <x:v>/admindraft/pawjaiprofile</x:v>
       </x:c>
-      <x:c r="D20" s="732" t="str">
+      <x:c r="D20" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E20" s="639" t="str">
@@ -4130,7 +4584,7 @@
       <x:c r="C21" s="639" t="str">
         <x:v>/admindraft/accounts</x:v>
       </x:c>
-      <x:c r="D21" s="732" t="str">
+      <x:c r="D21" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E21" s="639" t="str">
@@ -4150,7 +4604,7 @@
       <x:c r="C22" s="639" t="str">
         <x:v>/admindraft/audit</x:v>
       </x:c>
-      <x:c r="D22" s="732" t="str">
+      <x:c r="D22" s="776" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E22" s="639" t="str">

</xml_diff>

<commit_message>
Route admin draft about content to full editor
</commit_message>
<xml_diff>
--- a/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
+++ b/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="R37ca281a7e5b49fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="R834fc9a42c3a4068"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="3" r:id="R725865e42076487e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="4" r:id="R675fdf0a802248b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="5" r:id="Rff2c2854f7fc4e68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="6" r:id="R319929d7d4d94681"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="7" r:id="R6ab9f289d2734597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="8" r:id="R52f9de93ebde443d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="9" r:id="Rd2ee569d37f9409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="10" r:id="Radd1d96d92f74ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="11" r:id="R62718852a80944fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Route Gap Audit" sheetId="12" r:id="Rf1e639c0d5c844a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="1" r:id="R052e2c2f34264f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="2" r:id="R5f8dc312cbaf475a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="3" r:id="Rc828e3f8ac8d46f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="4" r:id="R89db466fc5dc4e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="5" r:id="Rdecaff9ed991487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="6" r:id="R460762c4a5a94740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="7" r:id="Rb0038dc2f549496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="8" r:id="R80c7826a897c4cb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="9" r:id="R46f342d0bfb64030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="10" r:id="R8c24f19a44db4fd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="11" r:id="R48a476e07b214cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Route Gap Audit" sheetId="12" r:id="Rf7e522e3eaad4551"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -162,7 +162,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="121">
+  <x:fills count="129">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -562,6 +562,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7E3E1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F1EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B4D40"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD88C24"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8ECD8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -879,7 +919,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="781">
+  <x:cellXfs count="827">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -2609,6 +2649,82 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="22" fillId="115" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="121" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="122" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="123" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="124" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="125" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="126" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="126" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="127" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="127" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="122" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="122" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="125" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="125" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="124" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="124" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="128" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="128" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="122" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="122" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="123" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="123" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="125" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="125" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="127" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="122" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="125" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="124" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="128" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="122" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="123" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="122" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="125" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="124" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="12" fillId="125" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="13" fillId="124" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="126" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="128" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="128" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="125" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="125" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="122" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="122" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="124" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="124" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="123" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="123" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2636,7 +2752,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2c7c44a5ea9f4781"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rfa9f774d00b84dc2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2663,7 +2779,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R91362363a42d4f9d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb9e13e63cd374c91"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2901,502 +3017,502 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="16">
-      <x:c r="A2" s="735" t="str">
+      <x:c r="A2" s="781" t="str">
         <x:v>Admin gate / password</x:v>
       </x:c>
-      <x:c r="B2" s="735" t="str">
+      <x:c r="B2" s="781" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="C2" s="735" t="str">
+      <x:c r="C2" s="781" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D2" s="736" t="str">
+      <x:c r="D2" s="782" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E2" s="735" t="str">
+      <x:c r="E2" s="781" t="str">
         <x:v>Keep temporary phrase gate until real login logic</x:v>
       </x:c>
-      <x:c r="F2" s="737" t="str">
+      <x:c r="F2" s="783" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="16">
-      <x:c r="A3" s="735" t="str">
+      <x:c r="A3" s="781" t="str">
         <x:v>Main PawJai admin umbrella</x:v>
       </x:c>
-      <x:c r="B3" s="735" t="str">
+      <x:c r="B3" s="781" t="str">
         <x:v>scattered across /admin/*</x:v>
       </x:c>
-      <x:c r="C3" s="735" t="str">
+      <x:c r="C3" s="781" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D3" s="736" t="str">
+      <x:c r="D3" s="782" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E3" s="735" t="str">
+      <x:c r="E3" s="781" t="str">
         <x:v>About, Accounts, and Audit now have draft-native pages; Ads write controls and Messaging remain the main gaps</x:v>
       </x:c>
-      <x:c r="F3" s="738" t="str">
+      <x:c r="F3" s="784" t="str">
         <x:v>High</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="16">
-      <x:c r="A4" s="735" t="str">
+      <x:c r="A4" s="781" t="str">
         <x:v>Partner shelters overview</x:v>
       </x:c>
-      <x:c r="B4" s="735" t="str">
+      <x:c r="B4" s="781" t="str">
         <x:v>mostly inside /admin/bookings</x:v>
       </x:c>
-      <x:c r="C4" s="735" t="str">
+      <x:c r="C4" s="781" t="str">
         <x:v>/admindraft &gt; Partner shelters</x:v>
       </x:c>
-      <x:c r="D4" s="736" t="str">
+      <x:c r="D4" s="782" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E4" s="735" t="str">
+      <x:c r="E4" s="781" t="str">
         <x:v>Add deeper shelter metrics later if wanted</x:v>
       </x:c>
-      <x:c r="F4" s="739" t="str">
+      <x:c r="F4" s="785" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="16">
-      <x:c r="A5" s="735" t="str">
+      <x:c r="A5" s="781" t="str">
         <x:v>Shelter profile edit</x:v>
       </x:c>
-      <x:c r="B5" s="735" t="str">
+      <x:c r="B5" s="781" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C5" s="735" t="str">
+      <x:c r="C5" s="781" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D5" s="736" t="str">
+      <x:c r="D5" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E5" s="735" t="str">
+      <x:c r="E5" s="781" t="str">
         <x:v>Real-world save testing per shelter</x:v>
       </x:c>
-      <x:c r="F5" s="736" t="str">
+      <x:c r="F5" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16">
-      <x:c r="A6" s="735" t="str">
+      <x:c r="A6" s="781" t="str">
         <x:v>Shelter logo upload</x:v>
       </x:c>
-      <x:c r="B6" s="735" t="str">
+      <x:c r="B6" s="781" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C6" s="735" t="str">
+      <x:c r="C6" s="781" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D6" s="736" t="str">
+      <x:c r="D6" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E6" s="735" t="str">
+      <x:c r="E6" s="781" t="str">
         <x:v>Real-world upload testing per shelter</x:v>
       </x:c>
-      <x:c r="F6" s="736" t="str">
+      <x:c r="F6" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="16">
-      <x:c r="A7" s="735" t="str">
+      <x:c r="A7" s="781" t="str">
         <x:v>Shelter donation details</x:v>
       </x:c>
-      <x:c r="B7" s="735" t="str">
+      <x:c r="B7" s="781" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C7" s="735" t="str">
+      <x:c r="C7" s="781" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D7" s="736" t="str">
+      <x:c r="D7" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E7" s="735" t="str">
+      <x:c r="E7" s="781" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F7" s="736" t="str">
+      <x:c r="F7" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="16">
-      <x:c r="A8" s="735" t="str">
+      <x:c r="A8" s="781" t="str">
         <x:v>Shelter operating hours</x:v>
       </x:c>
-      <x:c r="B8" s="735" t="str">
+      <x:c r="B8" s="781" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C8" s="735" t="str">
+      <x:c r="C8" s="781" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D8" s="736" t="str">
+      <x:c r="D8" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E8" s="735" t="str">
+      <x:c r="E8" s="781" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F8" s="736" t="str">
+      <x:c r="F8" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
-      <x:c r="A9" s="735" t="str">
+      <x:c r="A9" s="781" t="str">
         <x:v>Shelter blockout dates</x:v>
       </x:c>
-      <x:c r="B9" s="735" t="str">
+      <x:c r="B9" s="781" t="str">
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
-      <x:c r="C9" s="735" t="str">
+      <x:c r="C9" s="781" t="str">
         <x:v>/admindraft &gt; Shelter profile</x:v>
       </x:c>
-      <x:c r="D9" s="736" t="str">
+      <x:c r="D9" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E9" s="735" t="str">
+      <x:c r="E9" s="781" t="str">
         <x:v>Mostly transferred now</x:v>
       </x:c>
-      <x:c r="F9" s="736" t="str">
+      <x:c r="F9" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32">
-      <x:c r="A10" s="735" t="str">
+      <x:c r="A10" s="781" t="str">
         <x:v>Shelter dog listings</x:v>
       </x:c>
-      <x:c r="B10" s="735" t="str">
+      <x:c r="B10" s="781" t="str">
         <x:v>/admin/bookings?view=dogs, /admin/listings</x:v>
       </x:c>
-      <x:c r="C10" s="735" t="str">
+      <x:c r="C10" s="781" t="str">
         <x:v>/admindraft &gt; Dog listings</x:v>
       </x:c>
-      <x:c r="D10" s="736" t="str">
+      <x:c r="D10" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E10" s="735" t="str">
+      <x:c r="E10" s="781" t="str">
         <x:v>Search/status view is enough for shelter listing management; edit remains separate</x:v>
       </x:c>
-      <x:c r="F10" s="736" t="str">
+      <x:c r="F10" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="16">
-      <x:c r="A11" s="735" t="str">
+      <x:c r="A11" s="781" t="str">
         <x:v>Create dog listing</x:v>
       </x:c>
-      <x:c r="B11" s="735" t="str">
+      <x:c r="B11" s="781" t="str">
         <x:v>/admin, /admin/dogs/new</x:v>
       </x:c>
-      <x:c r="C11" s="735" t="str">
+      <x:c r="C11" s="781" t="str">
         <x:v>/admindraft/dog-creation</x:v>
       </x:c>
-      <x:c r="D11" s="736" t="str">
+      <x:c r="D11" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E11" s="735" t="str">
+      <x:c r="E11" s="781" t="str">
         <x:v>Draft-native create flow exists; real-world save/photo testing remains</x:v>
       </x:c>
-      <x:c r="F11" s="736" t="str">
+      <x:c r="F11" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32">
-      <x:c r="A12" s="735" t="str">
+      <x:c r="A12" s="781" t="str">
         <x:v>Edit dog listing</x:v>
       </x:c>
-      <x:c r="B12" s="735" t="str">
+      <x:c r="B12" s="781" t="str">
         <x:v>/admin/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="C12" s="735" t="str">
+      <x:c r="C12" s="781" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D12" s="736" t="str">
+      <x:c r="D12" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E12" s="735" t="str">
+      <x:c r="E12" s="781" t="str">
         <x:v>Draft-native edit route reuses the full old edit form; real-world save/photo testing remains</x:v>
       </x:c>
-      <x:c r="F12" s="736" t="str">
+      <x:c r="F12" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="32">
-      <x:c r="A13" s="735" t="str">
+      <x:c r="A13" s="781" t="str">
         <x:v>Dog photos / cover order</x:v>
       </x:c>
-      <x:c r="B13" s="735" t="str">
+      <x:c r="B13" s="781" t="str">
         <x:v>/admin, /admin/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="C13" s="735" t="str">
+      <x:c r="C13" s="781" t="str">
         <x:v>/admindraft/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D13" s="736" t="str">
+      <x:c r="D13" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E13" s="735" t="str">
+      <x:c r="E13" s="781" t="str">
         <x:v>Edit route now includes existing upload, reorder, cover, and remove tools</x:v>
       </x:c>
-      <x:c r="F13" s="736" t="str">
+      <x:c r="F13" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16">
-      <x:c r="A14" s="735" t="str">
+      <x:c r="A14" s="781" t="str">
         <x:v>All dog listings across shelters</x:v>
       </x:c>
-      <x:c r="B14" s="735" t="str">
+      <x:c r="B14" s="781" t="str">
         <x:v>/admin/listings</x:v>
       </x:c>
-      <x:c r="C14" s="735" t="str">
+      <x:c r="C14" s="781" t="str">
         <x:v>/admindraft &gt; All dog listings</x:v>
       </x:c>
-      <x:c r="D14" s="736" t="str">
+      <x:c r="D14" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E14" s="735" t="str">
+      <x:c r="E14" s="781" t="str">
         <x:v>Filters exist and edit buttons now open draft-native dog edit pages</x:v>
       </x:c>
-      <x:c r="F14" s="736" t="str">
+      <x:c r="F14" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32">
-      <x:c r="A15" s="735" t="str">
+      <x:c r="A15" s="781" t="str">
         <x:v>Booking visits list</x:v>
       </x:c>
-      <x:c r="B15" s="735" t="str">
+      <x:c r="B15" s="781" t="str">
         <x:v>/admin/bookings</x:v>
       </x:c>
-      <x:c r="C15" s="735" t="str">
+      <x:c r="C15" s="781" t="str">
         <x:v>/admindraft &gt; Bookings</x:v>
       </x:c>
-      <x:c r="D15" s="736" t="str">
+      <x:c r="D15" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E15" s="735" t="str">
+      <x:c r="E15" s="781" t="str">
         <x:v>Old low-friction booking card flow duplicated; real staff testing remains</x:v>
       </x:c>
-      <x:c r="F15" s="736" t="str">
+      <x:c r="F15" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="32">
-      <x:c r="A16" s="735" t="str">
+      <x:c r="A16" s="781" t="str">
         <x:v>Booking decision actions</x:v>
       </x:c>
-      <x:c r="B16" s="735" t="str">
+      <x:c r="B16" s="781" t="str">
         <x:v>/admin/bookings, /admin/bookings/[id]</x:v>
       </x:c>
-      <x:c r="C16" s="735" t="str">
+      <x:c r="C16" s="781" t="str">
         <x:v>/admindraft &gt; Bookings</x:v>
       </x:c>
-      <x:c r="D16" s="736" t="str">
+      <x:c r="D16" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E16" s="735" t="str">
+      <x:c r="E16" s="781" t="str">
         <x:v>Accept, deny, and date-change actions are draft-native; final status edge cases can be polished later</x:v>
       </x:c>
-      <x:c r="F16" s="736" t="str">
+      <x:c r="F16" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="16">
-      <x:c r="A17" s="735" t="str">
+      <x:c r="A17" s="781" t="str">
         <x:v>Booking detail page</x:v>
       </x:c>
-      <x:c r="B17" s="735" t="str">
+      <x:c r="B17" s="781" t="str">
         <x:v>/admin/bookings/[id]</x:v>
       </x:c>
-      <x:c r="C17" s="735" t="str">
+      <x:c r="C17" s="781" t="str">
         <x:v>/admindraft/bookings/[id]</x:v>
       </x:c>
-      <x:c r="D17" s="736" t="str">
+      <x:c r="D17" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E17" s="735" t="str">
+      <x:c r="E17" s="781" t="str">
         <x:v>QR scan can land here; refine isolated detail page only if needed</x:v>
       </x:c>
-      <x:c r="F17" s="736" t="str">
+      <x:c r="F17" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="16">
-      <x:c r="A18" s="735" t="str">
+      <x:c r="A18" s="781" t="str">
         <x:v>QR check-in</x:v>
       </x:c>
-      <x:c r="B18" s="735" t="str">
+      <x:c r="B18" s="781" t="str">
         <x:v>/admin/bookings/check-in</x:v>
       </x:c>
-      <x:c r="C18" s="735" t="str">
+      <x:c r="C18" s="781" t="str">
         <x:v>/admindraft/bookings/check-in</x:v>
       </x:c>
-      <x:c r="D18" s="736" t="str">
+      <x:c r="D18" s="782" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E18" s="735" t="str">
+      <x:c r="E18" s="781" t="str">
         <x:v>Needs real QR/camera device testing</x:v>
       </x:c>
-      <x:c r="F18" s="739" t="str">
+      <x:c r="F18" s="785" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32">
-      <x:c r="A19" s="735" t="str">
+      <x:c r="A19" s="781" t="str">
         <x:v>Visitor profile</x:v>
       </x:c>
-      <x:c r="B19" s="735" t="str">
+      <x:c r="B19" s="781" t="str">
         <x:v>/admin/bookings/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="C19" s="735" t="str">
+      <x:c r="C19" s="781" t="str">
         <x:v>/admindraft/bookings/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="D19" s="736" t="str">
+      <x:c r="D19" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E19" s="735" t="str">
+      <x:c r="E19" s="781" t="str">
         <x:v>Draft-native profile/documents view exists; real document review testing remains</x:v>
       </x:c>
-      <x:c r="F19" s="736" t="str">
+      <x:c r="F19" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="32">
-      <x:c r="A20" s="735" t="str">
+      <x:c r="A20" s="781" t="str">
         <x:v>Shelter messaging</x:v>
       </x:c>
-      <x:c r="B20" s="735" t="str">
+      <x:c r="B20" s="781" t="str">
         <x:v>/admin/bookings?view=messages</x:v>
       </x:c>
-      <x:c r="C20" s="735" t="str">
+      <x:c r="C20" s="781" t="str">
         <x:v>/admindraft &gt; Messaging</x:v>
       </x:c>
-      <x:c r="D20" s="738" t="str">
+      <x:c r="D20" s="784" t="str">
         <x:v>Visual only</x:v>
       </x:c>
-      <x:c r="E20" s="735" t="str">
+      <x:c r="E20" s="781" t="str">
         <x:v>Transfer real message thread and send reply in separate messaging session</x:v>
       </x:c>
-      <x:c r="F20" s="738" t="str">
+      <x:c r="F20" s="784" t="str">
         <x:v>High</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16">
-      <x:c r="A21" s="735" t="str">
+      <x:c r="A21" s="781" t="str">
         <x:v>Ads management</x:v>
       </x:c>
-      <x:c r="B21" s="735" t="str">
+      <x:c r="B21" s="781" t="str">
         <x:v>/admin/ads</x:v>
       </x:c>
-      <x:c r="C21" s="735" t="str">
+      <x:c r="C21" s="781" t="str">
         <x:v>/admindraft &gt; Ads</x:v>
       </x:c>
-      <x:c r="D21" s="739" t="str">
+      <x:c r="D21" s="785" t="str">
         <x:v>Read only</x:v>
       </x:c>
-      <x:c r="E21" s="735" t="str">
+      <x:c r="E21" s="781" t="str">
         <x:v>Transfer create ad, edit dates, pause/resume, delete</x:v>
       </x:c>
-      <x:c r="F21" s="739" t="str">
+      <x:c r="F21" s="785" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="16">
-      <x:c r="A22" s="735" t="str">
+      <x:c r="A22" s="781" t="str">
         <x:v>About content</x:v>
       </x:c>
-      <x:c r="B22" s="735" t="str">
+      <x:c r="B22" s="781" t="str">
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
-      <x:c r="C22" s="735" t="str">
-        <x:v>/admindraft/pawjaiprofile</x:v>
-      </x:c>
-      <x:c r="D22" s="736" t="str">
+      <x:c r="C22" s="781" t="str">
+        <x:v>/admindraft/aboutcontent</x:v>
+      </x:c>
+      <x:c r="D22" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E22" s="735" t="str">
-        <x:v>Draft-native About editor exists and saves through the same pawjai_profile table; live save smoke test remains</x:v>
-      </x:c>
-      <x:c r="F22" s="736" t="str">
+      <x:c r="E22" s="781" t="str">
+        <x:v>Draft-native About editor uses the finalized old admin UX/UI and saves through the same pawjai_profile table; live save smoke test remains</x:v>
+      </x:c>
+      <x:c r="F22" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="16">
-      <x:c r="A23" s="735" t="str">
+      <x:c r="A23" s="781" t="str">
         <x:v>Admin accounts</x:v>
       </x:c>
-      <x:c r="B23" s="735" t="str">
+      <x:c r="B23" s="781" t="str">
         <x:v>/admin/accounts</x:v>
       </x:c>
-      <x:c r="C23" s="735" t="str">
+      <x:c r="C23" s="781" t="str">
         <x:v>/admindraft/accounts</x:v>
       </x:c>
-      <x:c r="D23" s="736" t="str">
+      <x:c r="D23" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E23" s="735" t="str">
+      <x:c r="E23" s="781" t="str">
         <x:v>Draft-native account creation/revoke exists and uses the same Supabase Auth, profiles, and shelter_users logic</x:v>
       </x:c>
-      <x:c r="F23" s="736" t="str">
+      <x:c r="F23" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="16">
-      <x:c r="A24" s="735" t="str">
+      <x:c r="A24" s="781" t="str">
         <x:v>Audit log</x:v>
       </x:c>
-      <x:c r="B24" s="735" t="str">
+      <x:c r="B24" s="781" t="str">
         <x:v>/admin/audit</x:v>
       </x:c>
-      <x:c r="C24" s="735" t="str">
+      <x:c r="C24" s="781" t="str">
         <x:v>/admindraft/audit</x:v>
       </x:c>
-      <x:c r="D24" s="736" t="str">
+      <x:c r="D24" s="782" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="E24" s="735" t="str">
+      <x:c r="E24" s="781" t="str">
         <x:v>Draft-native audit table exists; keep testing with real admin changes</x:v>
       </x:c>
-      <x:c r="F24" s="736" t="str">
+      <x:c r="F24" s="782" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="16">
-      <x:c r="A25" s="735" t="str">
+      <x:c r="A25" s="781" t="str">
         <x:v>Admin login page</x:v>
       </x:c>
-      <x:c r="B25" s="735" t="str">
+      <x:c r="B25" s="781" t="str">
         <x:v>/admin/login</x:v>
       </x:c>
-      <x:c r="C25" s="735" t="str">
+      <x:c r="C25" s="781" t="str">
         <x:v>temporary phrase gate</x:v>
       </x:c>
-      <x:c r="D25" s="739" t="str">
+      <x:c r="D25" s="785" t="str">
         <x:v>Temporary</x:v>
       </x:c>
-      <x:c r="E25" s="735" t="str">
+      <x:c r="E25" s="781" t="str">
         <x:v>Later replace phrase gates with real auth</x:v>
       </x:c>
-      <x:c r="F25" s="737" t="str">
+      <x:c r="F25" s="783" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="16">
-      <x:c r="A26" s="735" t="str">
+      <x:c r="A26" s="781" t="str">
         <x:v>Legacy draft alias</x:v>
       </x:c>
-      <x:c r="B26" s="735" t="str">
+      <x:c r="B26" s="781" t="str">
         <x:v>/admin/reorg-draft</x:v>
       </x:c>
-      <x:c r="C26" s="735" t="str">
+      <x:c r="C26" s="781" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D26" s="736" t="str">
+      <x:c r="D26" s="782" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="E26" s="735" t="str">
+      <x:c r="E26" s="781" t="str">
         <x:v>Remove after /admindraft becomes canonical</x:v>
       </x:c>
-      <x:c r="F26" s="737" t="str">
+      <x:c r="F26" s="783" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
@@ -3657,7 +3773,7 @@
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra19b113cd2204d8a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9d60d3bb3ae4c5d"/>
 </x:worksheet>
 </file>
 
@@ -3674,32 +3790,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="770" t="str">
+      <x:c r="A1" s="816" t="str">
         <x:v>Old /admin route coverage into /admindraft</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="757" t="str">
+      <x:c r="A2" s="803" t="str">
         <x:v>Use this as the quick answer to: what still exists only in old admin? Right now the main remaining migration is Ads write controls; Messaging remains a separate shelter/adopter product workflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="758" t="str">
+      <x:c r="A4" s="804" t="str">
         <x:v>Old admin route</x:v>
       </x:c>
-      <x:c r="B4" s="758" t="str">
+      <x:c r="B4" s="804" t="str">
         <x:v>Draft / shared route</x:v>
       </x:c>
-      <x:c r="C4" s="758" t="str">
+      <x:c r="C4" s="804" t="str">
         <x:v>Coverage</x:v>
       </x:c>
-      <x:c r="D4" s="758" t="str">
+      <x:c r="D4" s="804" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="E4" s="758" t="str">
+      <x:c r="E4" s="804" t="str">
         <x:v>What remains</x:v>
       </x:c>
-      <x:c r="F4" s="758" t="str">
+      <x:c r="F4" s="804" t="str">
         <x:v>Priority</x:v>
       </x:c>
     </x:row>
@@ -3713,13 +3829,13 @@
       <x:c r="C5" s="639" t="str">
         <x:v>PawJai umbrella dashboard</x:v>
       </x:c>
-      <x:c r="D5" s="776" t="str">
+      <x:c r="D5" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E5" s="639" t="str">
         <x:v>Keep old /admin live until final cutover</x:v>
       </x:c>
-      <x:c r="F5" s="780" t="str">
+      <x:c r="F5" s="826" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
@@ -3733,13 +3849,13 @@
       <x:c r="C6" s="639" t="str">
         <x:v>All dog listings across shelters</x:v>
       </x:c>
-      <x:c r="D6" s="776" t="str">
+      <x:c r="D6" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E6" s="639" t="str">
         <x:v>None for draft parity</x:v>
       </x:c>
-      <x:c r="F6" s="776" t="str">
+      <x:c r="F6" s="822" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
@@ -3753,13 +3869,13 @@
       <x:c r="C7" s="639" t="str">
         <x:v>Dog create workflow</x:v>
       </x:c>
-      <x:c r="D7" s="776" t="str">
+      <x:c r="D7" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E7" s="639" t="str">
         <x:v>Continue real photo/upload smoke tests</x:v>
       </x:c>
-      <x:c r="F7" s="776" t="str">
+      <x:c r="F7" s="822" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
@@ -3773,13 +3889,13 @@
       <x:c r="C8" s="639" t="str">
         <x:v>Dog edit workflow</x:v>
       </x:c>
-      <x:c r="D8" s="776" t="str">
+      <x:c r="D8" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E8" s="639" t="str">
         <x:v>Continue real save/photo smoke tests</x:v>
       </x:c>
-      <x:c r="F8" s="776" t="str">
+      <x:c r="F8" s="822" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
@@ -3793,13 +3909,13 @@
       <x:c r="C9" s="639" t="str">
         <x:v>Booking list, filters, inline decisions</x:v>
       </x:c>
-      <x:c r="D9" s="776" t="str">
+      <x:c r="D9" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E9" s="639" t="str">
         <x:v>Real staff booking smoke tests only</x:v>
       </x:c>
-      <x:c r="F9" s="776" t="str">
+      <x:c r="F9" s="822" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
@@ -3813,13 +3929,13 @@
       <x:c r="C10" s="639" t="str">
         <x:v>Booking detail / QR landing</x:v>
       </x:c>
-      <x:c r="D10" s="776" t="str">
+      <x:c r="D10" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E10" s="639" t="str">
         <x:v>Phone QR test still recommended</x:v>
       </x:c>
-      <x:c r="F10" s="774" t="str">
+      <x:c r="F10" s="820" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
@@ -3833,13 +3949,13 @@
       <x:c r="C11" s="639" t="str">
         <x:v>Visitor profile and verification documents</x:v>
       </x:c>
-      <x:c r="D11" s="776" t="str">
+      <x:c r="D11" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E11" s="639" t="str">
         <x:v>Real document review smoke test</x:v>
       </x:c>
-      <x:c r="F11" s="776" t="str">
+      <x:c r="F11" s="822" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
@@ -3853,13 +3969,13 @@
       <x:c r="C12" s="639" t="str">
         <x:v>QR check-in</x:v>
       </x:c>
-      <x:c r="D12" s="776" t="str">
+      <x:c r="D12" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E12" s="639" t="str">
         <x:v>Real camera/device test</x:v>
       </x:c>
-      <x:c r="F12" s="774" t="str">
+      <x:c r="F12" s="820" t="str">
         <x:v>Medium</x:v>
       </x:c>
     </x:row>
@@ -3873,13 +3989,13 @@
       <x:c r="C13" s="639" t="str">
         <x:v>Ads visibility and filters</x:v>
       </x:c>
-      <x:c r="D13" s="774" t="str">
+      <x:c r="D13" s="820" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="E13" s="639" t="str">
         <x:v>Move create/edit/pause/delete ad controls into draft route</x:v>
       </x:c>
-      <x:c r="F13" s="778" t="str">
+      <x:c r="F13" s="824" t="str">
         <x:v>High</x:v>
       </x:c>
     </x:row>
@@ -3888,18 +4004,18 @@
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
       <x:c r="B14" s="639" t="str">
-        <x:v>/admindraft/pawjaiprofile</x:v>
+        <x:v>/admindraft/aboutcontent</x:v>
       </x:c>
       <x:c r="C14" s="639" t="str">
         <x:v>About content editor</x:v>
       </x:c>
-      <x:c r="D14" s="776" t="str">
+      <x:c r="D14" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E14" s="639" t="str">
         <x:v>Live save smoke test only</x:v>
       </x:c>
-      <x:c r="F14" s="776" t="str">
+      <x:c r="F14" s="822" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
@@ -3913,13 +4029,13 @@
       <x:c r="C15" s="639" t="str">
         <x:v>PawJai and shelter admin account management</x:v>
       </x:c>
-      <x:c r="D15" s="776" t="str">
+      <x:c r="D15" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E15" s="639" t="str">
         <x:v>Live create/revoke smoke test only</x:v>
       </x:c>
-      <x:c r="F15" s="776" t="str">
+      <x:c r="F15" s="822" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
@@ -3933,13 +4049,13 @@
       <x:c r="C16" s="639" t="str">
         <x:v>Audit log</x:v>
       </x:c>
-      <x:c r="D16" s="776" t="str">
+      <x:c r="D16" s="822" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E16" s="639" t="str">
         <x:v>Keep testing after real admin changes</x:v>
       </x:c>
-      <x:c r="F16" s="776" t="str">
+      <x:c r="F16" s="822" t="str">
         <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
@@ -3953,13 +4069,13 @@
       <x:c r="C17" s="639" t="str">
         <x:v>Legacy login</x:v>
       </x:c>
-      <x:c r="D17" s="774" t="str">
+      <x:c r="D17" s="820" t="str">
         <x:v>Temporary</x:v>
       </x:c>
       <x:c r="E17" s="639" t="str">
         <x:v>Replace phrase gate with real admin login later</x:v>
       </x:c>
-      <x:c r="F17" s="780" t="str">
+      <x:c r="F17" s="826" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
@@ -3973,13 +4089,13 @@
       <x:c r="C18" s="639" t="str">
         <x:v>Legacy draft alias</x:v>
       </x:c>
-      <x:c r="D18" s="774" t="str">
+      <x:c r="D18" s="820" t="str">
         <x:v>Temporary</x:v>
       </x:c>
       <x:c r="E18" s="639" t="str">
         <x:v>Remove after /admindraft replaces old admin</x:v>
       </x:c>
-      <x:c r="F18" s="780" t="str">
+      <x:c r="F18" s="826" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
@@ -4003,7 +4119,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21">
-      <x:c r="A1" s="741" t="str">
+      <x:c r="A1" s="787" t="str">
         <x:v>PAWJAI Admin Draft Transfer Progress</x:v>
       </x:c>
       <x:c r="B1"/>
@@ -4013,28 +4129,28 @@
       <x:c r="F1"/>
     </x:row>
     <x:row r="3" ht="15">
-      <x:c r="A3" s="758" t="str">
+      <x:c r="A3" s="804" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="758" t="str">
+      <x:c r="B3" s="804" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C3" s="758" t="str">
+      <x:c r="C3" s="804" t="str">
         <x:v>% of workflows</x:v>
       </x:c>
-      <x:c r="D3" s="758" t="str">
+      <x:c r="D3" s="804" t="str">
         <x:v>Meaning</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15">
-      <x:c r="A4" s="765" t="str">
+      <x:c r="A4" s="811" t="str">
         <x:v>Functional</x:v>
       </x:c>
-      <x:c r="B4" s="759" t="n">
+      <x:c r="B4" s="805" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A4)</x:f>
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C4" s="763" t="n">
+      <x:c r="C4" s="809" t="n">
         <x:f>B4/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.68</x:v>
       </x:c>
@@ -4043,14 +4159,14 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="15">
-      <x:c r="A5" s="765" t="str">
+      <x:c r="A5" s="811" t="str">
         <x:v>Exists</x:v>
       </x:c>
-      <x:c r="B5" s="759" t="n">
+      <x:c r="B5" s="805" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A5)</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C5" s="763" t="n">
+      <x:c r="C5" s="809" t="n">
         <x:f>B5/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.2</x:v>
       </x:c>
@@ -4059,14 +4175,14 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="15">
-      <x:c r="A6" s="766" t="str">
+      <x:c r="A6" s="812" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="B6" s="760" t="n">
+      <x:c r="B6" s="806" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C6" s="768" t="n">
+      <x:c r="C6" s="814" t="n">
         <x:f>B6/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -4075,14 +4191,14 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="15">
-      <x:c r="A7" s="766" t="str">
+      <x:c r="A7" s="812" t="str">
         <x:v>Read only</x:v>
       </x:c>
-      <x:c r="B7" s="760" t="n">
+      <x:c r="B7" s="806" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A7)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C7" s="768" t="n">
+      <x:c r="C7" s="814" t="n">
         <x:f>B7/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
@@ -4091,14 +4207,14 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="15">
-      <x:c r="A8" s="767" t="str">
+      <x:c r="A8" s="813" t="str">
         <x:v>Visual only</x:v>
       </x:c>
-      <x:c r="B8" s="761" t="n">
+      <x:c r="B8" s="807" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A8)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="769" t="n">
+      <x:c r="C8" s="815" t="n">
         <x:f>B8/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
@@ -4107,14 +4223,14 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="15">
-      <x:c r="A9" s="766" t="str">
+      <x:c r="A9" s="812" t="str">
         <x:v>Temporary</x:v>
       </x:c>
-      <x:c r="B9" s="760" t="n">
+      <x:c r="B9" s="806" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C9" s="768" t="n">
+      <x:c r="C9" s="814" t="n">
         <x:f>B9/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.04</x:v>
       </x:c>
@@ -4123,14 +4239,14 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="15">
-      <x:c r="A10" s="767" t="str">
+      <x:c r="A10" s="813" t="str">
         <x:v>Missing</x:v>
       </x:c>
-      <x:c r="B10" s="761" t="n">
+      <x:c r="B10" s="807" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C10" s="769" t="n">
+      <x:c r="C10" s="815" t="n">
         <x:f>B10/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -4139,51 +4255,51 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="15">
-      <x:c r="A13" s="762" t="str">
+      <x:c r="A13" s="808" t="str">
         <x:v>Metric</x:v>
       </x:c>
-      <x:c r="B13" s="762" t="str">
+      <x:c r="B13" s="808" t="str">
         <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15">
-      <x:c r="A14" s="765" t="str">
+      <x:c r="A14" s="811" t="str">
         <x:v>Functional workflows</x:v>
       </x:c>
-      <x:c r="B14" s="759" t="n">
+      <x:c r="B14" s="805" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Functional")</x:f>
         <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15">
-      <x:c r="A15" s="765" t="str">
+      <x:c r="A15" s="811" t="str">
         <x:v>Functional + Exists</x:v>
       </x:c>
-      <x:c r="B15" s="763" t="n">
+      <x:c r="B15" s="809" t="n">
         <x:f>(COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Functional")+COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,"Exists"))/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0.88</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15">
-      <x:c r="A16" s="767" t="str">
+      <x:c r="A16" s="813" t="str">
         <x:v>Still high priority</x:v>
       </x:c>
-      <x:c r="B16" s="761" t="n">
+      <x:c r="B16" s="807" t="n">
         <x:f>COUNTIF('Admin Transfer Tracker'!$F$2:$F$26,"High")</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15">
-      <x:c r="A17" s="764" t="str">
+      <x:c r="A17" s="810" t="str">
         <x:v>Total workflows</x:v>
       </x:c>
-      <x:c r="B17" s="764" t="n">
+      <x:c r="B17" s="810" t="n">
         <x:f>COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
-      <x:c r="A20" s="757" t="str">
+      <x:c r="A20" s="803" t="str">
         <x:v>Current read: shelter profile, dog creation/listing, booking flows, About content, Accounts, and Audit are now draft-native. Messaging is intentionally left for a separate session; Ads still needs write controls moved.</x:v>
       </x:c>
       <x:c r="B20"/>
@@ -4214,7 +4330,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
-      <x:c r="A1" s="770" t="str">
+      <x:c r="A1" s="816" t="str">
         <x:v>PAWJAI Admin -&gt; Shelter -&gt; Booking Route Migration Map</x:v>
       </x:c>
       <x:c r="B1"/>
@@ -4224,7 +4340,7 @@
       <x:c r="F1"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="772" t="str">
+      <x:c r="A2" s="818" t="str">
         <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
       </x:c>
       <x:c r="B2"/>
@@ -4235,22 +4351,22 @@
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="758" t="str">
+      <x:c r="A4" s="804" t="str">
         <x:v>Workflow</x:v>
       </x:c>
-      <x:c r="B4" s="758" t="str">
+      <x:c r="B4" s="804" t="str">
         <x:v>Old / current source</x:v>
       </x:c>
-      <x:c r="C4" s="758" t="str">
+      <x:c r="C4" s="804" t="str">
         <x:v>New canonical route</x:v>
       </x:c>
-      <x:c r="D4" s="758" t="str">
+      <x:c r="D4" s="804" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="E4" s="758" t="str">
+      <x:c r="E4" s="804" t="str">
         <x:v>What it does</x:v>
       </x:c>
-      <x:c r="F4" s="758" t="str">
+      <x:c r="F4" s="804" t="str">
         <x:v>Notes / next step</x:v>
       </x:c>
     </x:row>
@@ -4264,7 +4380,7 @@
       <x:c r="C5" s="639" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="D5" s="774" t="str">
+      <x:c r="D5" s="820" t="str">
         <x:v>Legacy active</x:v>
       </x:c>
       <x:c r="E5" s="639" t="str">
@@ -4284,7 +4400,7 @@
       <x:c r="C6" s="639" t="str">
         <x:v>/admindraft</x:v>
       </x:c>
-      <x:c r="D6" s="776" t="str">
+      <x:c r="D6" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E6" s="639" t="str">
@@ -4304,7 +4420,7 @@
       <x:c r="C7" s="639" t="str">
         <x:v>/shelter</x:v>
       </x:c>
-      <x:c r="D7" s="776" t="str">
+      <x:c r="D7" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E7" s="639" t="str">
@@ -4324,7 +4440,7 @@
       <x:c r="C8" s="639" t="str">
         <x:v>/shelter/[slug]</x:v>
       </x:c>
-      <x:c r="D8" s="776" t="str">
+      <x:c r="D8" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E8" s="639" t="str">
@@ -4344,7 +4460,7 @@
       <x:c r="C9" s="639" t="str">
         <x:v>/shelter/[slug]/settings</x:v>
       </x:c>
-      <x:c r="D9" s="776" t="str">
+      <x:c r="D9" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E9" s="639" t="str">
@@ -4364,7 +4480,7 @@
       <x:c r="C10" s="639" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
       </x:c>
-      <x:c r="D10" s="776" t="str">
+      <x:c r="D10" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E10" s="639" t="str">
@@ -4384,7 +4500,7 @@
       <x:c r="C11" s="639" t="str">
         <x:v>/shelter/[slug]/dogs/new</x:v>
       </x:c>
-      <x:c r="D11" s="776" t="str">
+      <x:c r="D11" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E11" s="639" t="str">
@@ -4404,7 +4520,7 @@
       <x:c r="C12" s="639" t="str">
         <x:v>/shelter/[slug]/dogs/[id]/edit</x:v>
       </x:c>
-      <x:c r="D12" s="776" t="str">
+      <x:c r="D12" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E12" s="639" t="str">
@@ -4424,7 +4540,7 @@
       <x:c r="C13" s="639" t="str">
         <x:v>/dogs/[id]</x:v>
       </x:c>
-      <x:c r="D13" s="776" t="str">
+      <x:c r="D13" s="822" t="str">
         <x:v>Shared exception</x:v>
       </x:c>
       <x:c r="E13" s="639" t="str">
@@ -4444,7 +4560,7 @@
       <x:c r="C14" s="639" t="str">
         <x:v>/shelter/[slug]?view=bookings</x:v>
       </x:c>
-      <x:c r="D14" s="776" t="str">
+      <x:c r="D14" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E14" s="639" t="str">
@@ -4464,7 +4580,7 @@
       <x:c r="C15" s="639" t="str">
         <x:v>/booking/[id]</x:v>
       </x:c>
-      <x:c r="D15" s="776" t="str">
+      <x:c r="D15" s="822" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E15" s="639" t="str">
@@ -4484,7 +4600,7 @@
       <x:c r="C16" s="639" t="str">
         <x:v>/booking/[id]/visitor-profile</x:v>
       </x:c>
-      <x:c r="D16" s="776" t="str">
+      <x:c r="D16" s="822" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E16" s="639" t="str">
@@ -4504,7 +4620,7 @@
       <x:c r="C17" s="639" t="str">
         <x:v>/booking/check-in</x:v>
       </x:c>
-      <x:c r="D17" s="776" t="str">
+      <x:c r="D17" s="822" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E17" s="639" t="str">
@@ -4524,7 +4640,7 @@
       <x:c r="C18" s="639" t="str">
         <x:v>/shelter/[slug]?view=messages</x:v>
       </x:c>
-      <x:c r="D18" s="778" t="str">
+      <x:c r="D18" s="824" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="E18" s="639" t="str">
@@ -4544,7 +4660,7 @@
       <x:c r="C19" s="639" t="str">
         <x:v>/admindraft &gt; Ads</x:v>
       </x:c>
-      <x:c r="D19" s="774" t="str">
+      <x:c r="D19" s="820" t="str">
         <x:v>Admin-only partial</x:v>
       </x:c>
       <x:c r="E19" s="639" t="str">
@@ -4562,9 +4678,9 @@
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
       <x:c r="C20" s="639" t="str">
-        <x:v>/admindraft/pawjaiprofile</x:v>
-      </x:c>
-      <x:c r="D20" s="776" t="str">
+        <x:v>/admindraft/aboutcontent</x:v>
+      </x:c>
+      <x:c r="D20" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E20" s="639" t="str">
@@ -4584,7 +4700,7 @@
       <x:c r="C21" s="639" t="str">
         <x:v>/admindraft/accounts</x:v>
       </x:c>
-      <x:c r="D21" s="776" t="str">
+      <x:c r="D21" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E21" s="639" t="str">
@@ -4604,7 +4720,7 @@
       <x:c r="C22" s="639" t="str">
         <x:v>/admindraft/audit</x:v>
       </x:c>
-      <x:c r="D22" s="776" t="str">
+      <x:c r="D22" s="822" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E22" s="639" t="str">

</xml_diff>

<commit_message>
Add realtime message updates
</commit_message>
<xml_diff>
--- a/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
+++ b/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Session Map" sheetId="1" r:id="Rc5a7db5ab8bb4fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Migration Status" sheetId="2" r:id="R01917d2c1aae4835"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Connections" sheetId="3" r:id="R9e065f016ab44a9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="4" r:id="R0d0842e4ccac4599"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="5" r:id="R9e84b2d327d649ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="6" r:id="R7ca5a3be52064ac4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="7" r:id="R0bcab23a51734d28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="8" r:id="R931e2dcdd004402b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="9" r:id="Ra491968b90bc40cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="10" r:id="R72db10c744174c41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="11" r:id="R620fce1e4a844ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="12" r:id="R1de268bc26114f7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="13" r:id="R92499deb48594043"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="14" r:id="R3b4c6ec5e1c042fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Route Gap Audit" sheetId="15" r:id="R97a327a9389e47d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Work" sheetId="16" r:id="R4825bff5a8a04dfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow Plan" sheetId="17" r:id="R832fd5cda1734505"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Safety Matrix" sheetId="18" r:id="R9bcf0617bae14615"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production URLs &amp; Logins" sheetId="19" r:id="R4e1f518bc73f4579"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Session Map" sheetId="1" r:id="R1589f025c13b4661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Migration Status" sheetId="2" r:id="R0358543ffc7942d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Connections" sheetId="3" r:id="Re86fd6a5d10b4750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="4" r:id="Rb31d43673f8b478f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="5" r:id="Rb18f16d3155448bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="6" r:id="R139fb995a0bd4a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="7" r:id="R08b411322aa84177"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="8" r:id="Rf91bd6371d4d4d81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="9" r:id="R7e4694615a934388"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="10" r:id="Rf6e0a868722f46cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="11" r:id="Rb7e50dbc16914d2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="12" r:id="R28e532d921ee4fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="13" r:id="Re81d590c68b24f0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="14" r:id="R7e5cc73149104eb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Route Gap Audit" sheetId="15" r:id="R4b69e23792564362"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Work" sheetId="16" r:id="Rd342142ecb954d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow Plan" sheetId="17" r:id="R9ef9cfcb4a7c430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Safety Matrix" sheetId="18" r:id="R702bb609957a4246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production URLs &amp; Logins" sheetId="19" r:id="R56dd9f14061b48fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2416,7 +2416,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rce9de337c25547a5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc5d3e5fe3d074948"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2443,7 +2443,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd2a0bc01c4a847bc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1add10dc02384193"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -5637,7 +5637,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5df829cba104206"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1997f07ba614dbb"/>
 </x:worksheet>
 </file>
 
@@ -6048,10 +6048,10 @@
         <x:v>Partial: appointment-thread base exists, but pilot-ready shelter-user messaging is not complete.</x:v>
       </x:c>
       <x:c r="C5" s="133" t="str">
-        <x:v>Messaging launch pass complete: adopter/shelter threads, PawJai read-only view, attachment rules, Resend email notifications, canonical links, backend timestamps, and visible-tab auto-refresh are implemented.</x:v>
+        <x:v>Messaging launch pass complete: adopter/shelter threads, PawJai read-only view, attachment rules, Resend email notifications, canonical links, backend timestamps, Supabase Realtime subscriptions, and visible-tab fallback refresh are implemented.</x:v>
       </x:c>
       <x:c r="D5" s="133" t="str">
-        <x:v>Watch real production conversations and consider true Supabase Realtime or direct-to-storage uploads later if operational volume or 200 MB video reliability requires it.</x:v>
+        <x:v>Watch real production conversations and consider direct-to-storage uploads later if 200 MB mobile video reliability requires it.</x:v>
       </x:c>
       <x:c r="E5" s="727" t="str">
         <x:v>High</x:v>
@@ -9149,7 +9149,7 @@
         <x:v>Complete - launch-ready</x:v>
       </x:c>
       <x:c r="E20" s="767" t="str">
-        <x:v>Appointment thread UX is now wired across adopter /appointments/[id]?tab=messages, shelter /shelter/[slug]?view=messages, and PawJai /admindraft Messaging. Supabase appointment_messages stores body, sender role/label, attachment URL/name/type, and DB created_at timestamps. UI now shows backend timestamps, auto-refreshes visible message views every 12s, supports PDF/JPEG/JPG/PNG/WebP/HEIC/HEIF/MP4/MOV uploads up to 200 MB code-level cap, previews web images/video where supported, and opens all other files via attachment links. Resend emails notify the opposite party with canonical www.pawjaipet.com links. PawJai admin remains read-only.</x:v>
+        <x:v>Appointment thread UX is wired across adopter /appointments/[id]?tab=messages, shelter /shelter/[slug]?view=messages, and PawJai /admindraft Messaging. Supabase appointment_messages stores body, sender role/label, attachment URL/name/type, and DB created_at timestamps. UI now shows backend timestamps, subscribes to Supabase Realtime message changes, keeps a 12s visible-tab refresh fallback, supports PDF/JPEG/JPG/PNG/WebP/HEIC/HEIF/MP4/MOV uploads up to 200 MB code-level cap, previews web images/video where supported, and opens all other files via attachment links. Resend emails notify the opposite party with canonical www.pawjaipet.com links. PawJai admin remains read-only.</x:v>
       </x:c>
       <x:c r="F20" s="768" t="str">
         <x:v>Monitor first live shelter/user conversations, confirm Vercel large-upload behavior on mobile, and move videos to direct-to-storage signed uploads if 200 MB mobile uploads prove unreliable under production network conditions.</x:v>

</xml_diff>

<commit_message>
Promote admin workspace to canonical routes
</commit_message>
<xml_diff>
--- a/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
+++ b/outputs/admin-transfer-tracker-20260705/pawjai-admin-transfer-tracker.xlsx
@@ -2,30 +2,31 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Session Map" sheetId="1" r:id="R369b76a05df6423f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Migration Status" sheetId="2" r:id="R486434428d924aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Connections" sheetId="3" r:id="R2827eef99a7242b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="4" r:id="R0fa66505786c4685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="5" r:id="R6cf87350bbea4703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="6" r:id="R76a448449a974fb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="7" r:id="R32ed55fb43e64296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="8" r:id="R2b29e5e03af841e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="9" r:id="R3634c757a1e6490c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="10" r:id="Ree2879b891294a06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="11" r:id="R31463c7a33be4c27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="12" r:id="R30a2bc24e3d94c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="13" r:id="Rf5008bbbe11b4634"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="14" r:id="Rbdc83c8a13474c28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Route Gap Audit" sheetId="15" r:id="R8a5fd819e81e4532"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Work" sheetId="16" r:id="Rb90877a8824f460c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow Plan" sheetId="17" r:id="Rc69951ba85cb4959"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Safety Matrix" sheetId="18" r:id="Ra63918f484f34fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production URLs &amp; Logins" sheetId="19" r:id="Ra9be8e8b10f94c8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Messaging QA Matrix" sheetId="20" r:id="R2e38039439544930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-08-16 Refresh Log" sheetId="21" r:id="R10ffce95f91f4dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shelter Pilot QA 2026-08-21" sheetId="22" r:id="Ra1f3566f52374dec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-08-21 Shelter QA Log" sheetId="23" r:id="Rb61a5b119e8c41b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-08-22 Shelter Fixes" sheetId="24" r:id="Rdb893542cc0d4f11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Session Map" sheetId="1" r:id="R4f59c75be0a2494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Migration Status" sheetId="2" r:id="Rc3358bffa9bd43fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Connections" sheetId="3" r:id="Rb5e7bb9e075b4310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Transfer Tracker" sheetId="4" r:id="Rff9c044c7fda4ea2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Summary" sheetId="5" r:id="Ra57454841e934e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Migration Map" sheetId="6" r:id="R30ab99ea62044b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lane Connections" sheetId="7" r:id="Rfbbab068a5484f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Sync Diagram" sheetId="8" r:id="R89be921cb51f415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Flow Diagram" sheetId="9" r:id="R9adf1cc658c94874"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back Behavior" sheetId="10" r:id="Rdf3838f898ee48bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Route Spec" sheetId="11" r:id="Rcc576a51cc714832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Checklist" sheetId="12" r:id="Rd09f8a90855c4f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Advice" sheetId="13" r:id="Rea99c8b6104649fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagram Gallery" sheetId="14" r:id="Rfdc6b589272a4c07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Route Gap Audit" sheetId="15" r:id="Re3df55f8516b40bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Work" sheetId="16" r:id="R5cdd11a9daf74044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow Plan" sheetId="17" r:id="R281b390fd91543e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Route Safety Matrix" sheetId="18" r:id="Rdc5ecd4b77f34b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production URLs &amp; Logins" sheetId="19" r:id="Reccc1dcc9a3b4625"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Messaging QA Matrix" sheetId="20" r:id="R8ded700fa1b94925"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-08-16 Refresh Log" sheetId="21" r:id="R409cda847af444c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shelter Pilot QA 2026-08-21" sheetId="22" r:id="Rb1efd5e6761b4fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-08-21 Shelter QA Log" sheetId="23" r:id="Rac48791df6fd46dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-08-22 Shelter Fixes" sheetId="24" r:id="Rc6ed1ab34c7e4fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-08-22 Admin Cutover" sheetId="25" r:id="Rc21a4697508843d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -39,7 +40,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="59">
+  <x:fonts count="64">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -369,8 +370,37 @@
       <x:color rgb="FF9B5F16"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF65584F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF51453C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF2F7A35"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF65584F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF2F7A35"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="154">
+  <x:fills count="159">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1137,8 +1167,33 @@
         <x:fgColor rgb="FFF1E8DD"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF51453C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8EE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD98C20"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5F2DE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5F2DE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="41">
+  <x:borders count="50">
     <x:border/>
     <x:border>
       <x:top style="thin">
@@ -1532,11 +1587,101 @@
         <x:color rgb="FFD6C8AD"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFE8DCC9"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1235">
+  <x:cellXfs count="1275">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -4078,6 +4223,92 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="58" fillId="149" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="154" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="154" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="155" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="59" fillId="155" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="59" fillId="155" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="156" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="156" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="156" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="157" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="157" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="157" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="61" fillId="157" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="61" fillId="157" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="61" fillId="157" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="62" fillId="155" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="155" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="154" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="158" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="63" fillId="158" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="158" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="158" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -4263,7 +4494,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5e021bd9ad64401c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0d1d85779e124aac"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -4290,7 +4521,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4b74441e61f645e3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R501c61516d644322"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -7049,7 +7280,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72253fd496f54827"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra80a616b4f6d4568"/>
 </x:worksheet>
 </file>
 
@@ -7432,7 +7663,7 @@
     </x:row>
     <x:row r="2" s="62" customFormat="1" ht="15" customHeight="1">
       <x:c r="A2" s="1185" t="str">
-        <x:v>Updated 2026-08-21 +07 after the full Voice/Rescue shelter workflow audit and production-backed write checks. Items are ordered around shelter pilot safety first, then broader platform hardening and old-admin cutover.</x:v>
+        <x:v>Updated 2026-08-22 +07 after promoting the completed PawJai HQ workspace from /admindraft to canonical /admin. Route cutover is complete; remaining items are operational pilot checks and broader platform hardening.</x:v>
       </x:c>
       <x:c r="B2" s="1185"/>
       <x:c r="C2" s="1185"/>
@@ -7527,7 +7758,7 @@
         <x:v>Booking access and list/detail routes passed, but no real customer booking status was mutated.</x:v>
       </x:c>
       <x:c r="C7" s="1181" t="str">
-        <x:v>Create a harmless QA booking, accept/change/deny it from the shelter portal, and confirm /admindraft reads the same row.</x:v>
+        <x:v>Create a harmless QA booking, accept/change/deny it from the shelter portal, and confirm /admin sees the same appointment row and status.</x:v>
       </x:c>
       <x:c r="D7" s="1181" t="str">
         <x:v>Completes safe evidence for shared appointment writes.</x:v>
@@ -7539,7 +7770,7 @@
         <x:v>Before staff pilot</x:v>
       </x:c>
       <x:c r="G7" s="1181" t="str">
-        <x:v>/shelter/[slug]?view=bookings; /booking/[id]; /admindraft</x:v>
+        <x:v>/shelter/[slug]?view=bookings; /shelter/[slug]/bookings/[id]; /admin?view=bookings</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="62" customFormat="1" ht="52" customHeight="1">
@@ -7677,30 +7908,30 @@
         <x:v>Before admin cutover</x:v>
       </x:c>
       <x:c r="G13" s="1181" t="str">
-        <x:v>/admindraft?view=ads; /ads</x:v>
+        <x:v>/admin?view=ads; /ads</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="52" customHeight="1">
       <x:c r="A14" s="1181" t="str">
-        <x:v>Google OAuth branding</x:v>
+        <x:v>Admin route cutover</x:v>
       </x:c>
       <x:c r="B14" s="1181" t="str">
-        <x:v>Code path is ready but production environment and consent branding require a fresh-browser check.</x:v>
+        <x:v>Complete locally: the finished reorganized workspace is canonical at /admin and /admindraft is a permanent compatibility redirect.</x:v>
       </x:c>
       <x:c r="C14" s="1181" t="str">
-        <x:v>Verify Vercel env, Google origins, branding, login, callback, and password-reset paths.</x:v>
+        <x:v>Deploy through the normal main-branch workflow, then smoke-test login and each HQ tab once in production.</x:v>
       </x:c>
       <x:c r="D14" s="1181" t="str">
-        <x:v>Prevents public sign-in confusion and supports the future employee-auth lane.</x:v>
+        <x:v>Confirms the new canonical URL without deleting safe legacy bookmarks.</x:v>
       </x:c>
       <x:c r="E14" s="1181" t="str">
-        <x:v>High</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="F14" s="1181" t="str">
-        <x:v>Before public auth promotion</x:v>
+        <x:v>Completed locally 2026-08-22</x:v>
       </x:c>
       <x:c r="G14" s="1181" t="str">
-        <x:v>docs/playbooks/google-oauth-branding.md; /auth/*</x:v>
+        <x:v>/admin; /admin/login; /admindraft/* redirect</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="52" customHeight="1">
@@ -7728,25 +7959,25 @@
     </x:row>
     <x:row r="16" ht="52" customHeight="1">
       <x:c r="A16" s="1181" t="str">
-        <x:v>Old admin cutover</x:v>
+        <x:v>Legacy admin URL compatibility</x:v>
       </x:c>
       <x:c r="B16" s="1181" t="str">
-        <x:v>Legacy /admin remains live while /admindraft is the reorganized umbrella.</x:v>
+        <x:v>/admindraft/* is configured as a permanent redirect to the matching /admin/* destination.</x:v>
       </x:c>
       <x:c r="C16" s="1181" t="str">
-        <x:v>Cut over only after auth, QR, booking write QA, ads, About content, and final staff pilot pass.</x:v>
+        <x:v>After deployment, open the legacy root and one deep link; confirm both land in /admin and still require the Google admin session.</x:v>
       </x:c>
       <x:c r="D16" s="1181" t="str">
-        <x:v>Avoids breaking internal operations during the final migration.</x:v>
+        <x:v>Preserves old bookmarks without maintaining a second admin interface.</x:v>
       </x:c>
       <x:c r="E16" s="1181" t="str">
-        <x:v>Later</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="F16" s="1181" t="str">
-        <x:v>After pilot completion</x:v>
+        <x:v>After admin deployment</x:v>
       </x:c>
       <x:c r="G16" s="1181" t="str">
-        <x:v>/admin/*; /admindraft; /shelter/*</x:v>
+        <x:v>/admindraft/* -&gt; /admin/*</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="66" customHeight="1">
@@ -7808,7 +8039,7 @@
     </x:row>
     <x:row r="2" s="62" customFormat="1" ht="15" customHeight="1">
       <x:c r="A2" s="1185" t="str">
-        <x:v>Updated 2026-08-21 +07. PawJai HQ owns the umbrella; each shelter is a scoped workspace; bookings are a guarded shared resource; public dog profiles are the only intentional public crossover. The Voice and Rescue route audit now supports this hierarchy with both automated checks and live read/write evidence.</x:v>
+        <x:v>Updated 2026-08-22 +07. PawJai HQ is canonical at /admin; each shelter remains scoped under /shelter; booking views use role-specific URLs over shared implementation and data; /admindraft is redirect-only compatibility.</x:v>
       </x:c>
       <x:c r="B2" s="1185"/>
       <x:c r="C2" s="1185"/>
@@ -7880,7 +8111,7 @@
         <x:v>PawJai HQ admin umbrella</x:v>
       </x:c>
       <x:c r="C6" s="1181" t="str">
-        <x:v>/admindraft</x:v>
+        <x:v>/admin</x:v>
       </x:c>
       <x:c r="D6" s="1181" t="str">
         <x:v>PawJai HQ</x:v>
@@ -7889,10 +8120,10 @@
         <x:v>All shelters, dogs, bookings, donations, ads, content, accounts, audit, and analytics.</x:v>
       </x:c>
       <x:c r="F6" s="1181" t="str">
-        <x:v>Admin guard must reject shelter sessions; view-as-shelter remains an HQ preview, not a shelter login.</x:v>
+        <x:v>Google admin guard rejects shelter sessions; View as shelter is an HQ preview only.</x:v>
       </x:c>
       <x:c r="G6" s="1181" t="str">
-        <x:v>Near complete; real auth + final cutover remain</x:v>
+        <x:v>Complete; canonical route promoted</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="62" customFormat="1" ht="55" customHeight="1">
@@ -7912,7 +8143,7 @@
         <x:v>Own profile, current/past dogs, create/edit, bookings/calendar, donation setup, messages, settings.</x:v>
       </x:c>
       <x:c r="F7" s="1181" t="str">
-        <x:v>Scope every read/write by authenticated shelter id; never expose /admindraft navigation or data.</x:v>
+        <x:v>Scope every read/write by authenticated shelter id; never expose /admin navigation or data.</x:v>
       </x:c>
       <x:c r="G7" s="1181" t="str">
         <x:v>Pilot-ready; physical phone checks remain</x:v>
@@ -7926,19 +8157,19 @@
         <x:v>Shared guarded booking workspace</x:v>
       </x:c>
       <x:c r="C8" s="1181" t="str">
-        <x:v>/booking/[id], /booking/[id]/visitor-profile, /booking/check-in</x:v>
+        <x:v>/admin/bookings/* or /shelter/[slug]/bookings/*</x:v>
       </x:c>
       <x:c r="D8" s="1181" t="str">
         <x:v>PawJai HQ + linked shelter</x:v>
       </x:c>
       <x:c r="E8" s="1181" t="str">
-        <x:v>One source of truth for appointment details, decisions, visitor verification, and QR check-in.</x:v>
+        <x:v>Shared appointment details, decisions, visitor verification, and QR check-in over one database record.</x:v>
       </x:c>
       <x:c r="F8" s="1181" t="str">
-        <x:v>canAccessShelter plus validated returnTo selects the correct parent lane; public users cannot enter.</x:v>
+        <x:v>canAccessShelter plus lane-specific URL/returnTo selects the correct parent; public users cannot enter.</x:v>
       </x:c>
       <x:c r="G8" s="1181" t="str">
-        <x:v>Route guards verified; safe write test + physical QR pending</x:v>
+        <x:v>Route guards complete; physical QR remains manual QA</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="62" customFormat="1" ht="55" customHeight="1">
@@ -7969,22 +8200,22 @@
         <x:v>Level 5</x:v>
       </x:c>
       <x:c r="B10" s="1181" t="str">
-        <x:v>Legacy admin fallback</x:v>
+        <x:v>Legacy draft URL compatibility</x:v>
       </x:c>
       <x:c r="C10" s="1181" t="str">
-        <x:v>/admin/*</x:v>
+        <x:v>/admindraft/* -&gt; /admin/*</x:v>
       </x:c>
       <x:c r="D10" s="1181" t="str">
-        <x:v>PawJai HQ only</x:v>
+        <x:v>Old bookmarks only</x:v>
       </x:c>
       <x:c r="E10" s="1181" t="str">
-        <x:v>Old workflows remain available while the reorganized umbrella finishes validation.</x:v>
+        <x:v>Permanent redirect into the canonical admin route family.</x:v>
       </x:c>
       <x:c r="F10" s="1181" t="str">
-        <x:v>Never link shelter staff into this lane. Remove/redirect only after the cutover checklist is green.</x:v>
+        <x:v>No UI, email, action, or notification may generate /admindraft; the redirected /admin destination still enforces Google admin auth.</x:v>
       </x:c>
       <x:c r="G10" s="1181" t="str">
-        <x:v>Remaining by design</x:v>
+        <x:v>Complete compatibility bridge</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8034,7 +8265,7 @@
     </x:row>
     <x:row r="2" s="62" customFormat="1" ht="15" customHeight="1">
       <x:c r="A2" s="735" t="str">
-        <x:v>Explicit route guardrails showing who can enter each lane, where they return, and what still needs testing before the old admin is retired.</x:v>
+        <x:v>Canonical route guardrails after the admin cutover: /admin is PawJai HQ, /shelter is scoped staff access, and legacy /admindraft URLs only redirect into the guarded admin lane.</x:v>
       </x:c>
       <x:c r="B2" s="736" t="str">
         <x:v>Explicit route guardrails showing who can enter each lane, where they return, and what still needs testing before the old admin is retired.</x:v>
@@ -8080,45 +8311,45 @@
     </x:row>
     <x:row r="5" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A5" s="742" t="str">
-        <x:v>/admindraft</x:v>
+        <x:v>/admin</x:v>
       </x:c>
       <x:c r="B5" s="742" t="str">
-        <x:v>PawJai global admin</x:v>
+        <x:v>PawJai Google global admin</x:v>
       </x:c>
       <x:c r="C5" s="742" t="str">
         <x:v>Shelter staff, public users</x:v>
       </x:c>
       <x:c r="D5" s="742" t="str">
-        <x:v>Temporary root-scoped admin draft phrase gate; later real admin auth</x:v>
+        <x:v>admin layout lane guard + requireGlobalAdmin</x:v>
       </x:c>
       <x:c r="E5" s="742" t="str">
         <x:v>PawJai HQ umbrella</x:v>
       </x:c>
       <x:c r="F5" s="742" t="str">
-        <x:v>Do not share with shelters</x:v>
+        <x:v>Shelter sessions are redirected to their own portal</x:v>
       </x:c>
       <x:c r="G5" s="725" t="str">
-        <x:v>Near complete</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A6" s="742" t="str">
-        <x:v>/admindraft?role=shelter</x:v>
+        <x:v>/admin?role=shelter</x:v>
       </x:c>
       <x:c r="B6" s="742" t="str">
-        <x:v>PawJai global admin previewing a shelter workspace</x:v>
+        <x:v>PawJai global admin previewing a shelter</x:v>
       </x:c>
       <x:c r="C6" s="742" t="str">
         <x:v>Shelter staff, public users</x:v>
       </x:c>
       <x:c r="D6" s="742" t="str">
-        <x:v>Same admin draft phrase/auth context; role=shelter is only UI state, not shelter authorization</x:v>
+        <x:v>Same Google admin context; role=shelter is UI state only</x:v>
       </x:c>
       <x:c r="E6" s="742" t="str">
-        <x:v>/admindraft?shelter=:id&amp;view=:tab&amp;role=shelter after deep create/edit/booking paths</x:v>
+        <x:v>/admin?shelter=:id&amp;view=:tab&amp;role=shelter</x:v>
       </x:c>
       <x:c r="F6" s="742" t="str">
-        <x:v>Keeps View as shelter sticky without giving shelters access to PawJai umbrella</x:v>
+        <x:v>Keeps HQ preview sticky without granting shelter access</x:v>
       </x:c>
       <x:c r="G6" s="725" t="str">
         <x:v>Complete</x:v>
@@ -8126,22 +8357,22 @@
     </x:row>
     <x:row r="7" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A7" s="742" t="str">
-        <x:v>/admindraft/aboutcontent</x:v>
+        <x:v>/admin/aboutcontent</x:v>
       </x:c>
       <x:c r="B7" s="742" t="str">
-        <x:v>PawJai global admin</x:v>
+        <x:v>PawJai Google global admin</x:v>
       </x:c>
       <x:c r="C7" s="742" t="str">
         <x:v>Shelter staff, public users</x:v>
       </x:c>
       <x:c r="D7" s="742" t="str">
-        <x:v>Admin draft gate + requireGlobalAdmin; returnTo preserved</x:v>
+        <x:v>admin layout + requireGlobalAdmin</x:v>
       </x:c>
       <x:c r="E7" s="742" t="str">
-        <x:v>Same page after unlock</x:v>
+        <x:v>Same page after save</x:v>
       </x:c>
       <x:c r="F7" s="742" t="str">
-        <x:v>Safe after latest fix</x:v>
+        <x:v>HQ content editor only</x:v>
       </x:c>
       <x:c r="G7" s="725" t="str">
         <x:v>Complete</x:v>
@@ -8149,22 +8380,22 @@
     </x:row>
     <x:row r="8" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A8" s="742" t="str">
-        <x:v>/admindraft/ads</x:v>
+        <x:v>/admin?view=ads</x:v>
       </x:c>
       <x:c r="B8" s="742" t="str">
-        <x:v>PawJai global admin</x:v>
+        <x:v>PawJai Google global admin</x:v>
       </x:c>
       <x:c r="C8" s="742" t="str">
         <x:v>Shelter staff, public users</x:v>
       </x:c>
       <x:c r="D8" s="742" t="str">
-        <x:v>Admin draft gate + requireGlobalAdmin; returnTo=/admindraft/ads</x:v>
+        <x:v>admin layout + requireGlobalAdmin</x:v>
       </x:c>
       <x:c r="E8" s="742" t="str">
-        <x:v>Same page after save/mutation</x:v>
+        <x:v>Same filtered ads workspace</x:v>
       </x:c>
       <x:c r="F8" s="742" t="str">
-        <x:v>HQ-only ad create/edit/pause/delete controls</x:v>
+        <x:v>HQ-only ad create/edit/review controls</x:v>
       </x:c>
       <x:c r="G8" s="725" t="str">
         <x:v>Complete</x:v>
@@ -8172,22 +8403,22 @@
     </x:row>
     <x:row r="9" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A9" s="742" t="str">
-        <x:v>/admindraft/accounts</x:v>
+        <x:v>/admin/accounts</x:v>
       </x:c>
       <x:c r="B9" s="742" t="str">
-        <x:v>PawJai global admin</x:v>
+        <x:v>PawJai Google global admin</x:v>
       </x:c>
       <x:c r="C9" s="742" t="str">
         <x:v>Shelter staff, public users</x:v>
       </x:c>
       <x:c r="D9" s="742" t="str">
-        <x:v>Admin draft gate + requireGlobalAdmin</x:v>
+        <x:v>admin layout + requireGlobalAdmin</x:v>
       </x:c>
       <x:c r="E9" s="742" t="str">
-        <x:v>Same page after unlock</x:v>
+        <x:v>Same page after mutation</x:v>
       </x:c>
       <x:c r="F9" s="742" t="str">
-        <x:v>Only HQ should create/revoke admin accounts</x:v>
+        <x:v>Only HQ creates or revokes admin accounts</x:v>
       </x:c>
       <x:c r="G9" s="725" t="str">
         <x:v>Complete</x:v>
@@ -8195,22 +8426,22 @@
     </x:row>
     <x:row r="10" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A10" s="742" t="str">
-        <x:v>/admindraft/audit</x:v>
+        <x:v>/admin/audit and /admin/analytics</x:v>
       </x:c>
       <x:c r="B10" s="742" t="str">
-        <x:v>PawJai global admin</x:v>
+        <x:v>PawJai Google global admin</x:v>
       </x:c>
       <x:c r="C10" s="742" t="str">
         <x:v>Shelter staff, public users</x:v>
       </x:c>
       <x:c r="D10" s="742" t="str">
-        <x:v>Admin draft gate + requireGlobalAdmin</x:v>
+        <x:v>admin layout + requireGlobalAdmin</x:v>
       </x:c>
       <x:c r="E10" s="742" t="str">
-        <x:v>Same page after unlock</x:v>
+        <x:v>Same PawJai HQ route</x:v>
       </x:c>
       <x:c r="F10" s="742" t="str">
-        <x:v>HQ audit only</x:v>
+        <x:v>HQ-only audit and analytics</x:v>
       </x:c>
       <x:c r="G10" s="725" t="str">
         <x:v>Complete</x:v>
@@ -8233,7 +8464,7 @@
         <x:v>/shelter/[slug]</x:v>
       </x:c>
       <x:c r="F11" s="742" t="str">
-        <x:v>Never redirect shelter staff into /admindraft</x:v>
+        <x:v>Never redirect shelter staff into /admin</x:v>
       </x:c>
       <x:c r="G11" s="725" t="str">
         <x:v>Near complete</x:v>
@@ -8287,7 +8518,7 @@
     </x:row>
     <x:row r="14" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A14" s="742" t="str">
-        <x:v>/booking/[id]</x:v>
+        <x:v>/admin/bookings/[id] or /shelter/[slug]/bookings/[id]</x:v>
       </x:c>
       <x:c r="B14" s="742" t="str">
         <x:v>PawJai admin or linked shelter staff</x:v>
@@ -8296,10 +8527,10 @@
         <x:v>Wrong shelter, public users</x:v>
       </x:c>
       <x:c r="D14" s="742" t="str">
-        <x:v>getAdminAuthContext + canAccessShelter + safe returnTo</x:v>
+        <x:v>shared renderer + getAdminAuthContext + canAccessShelter</x:v>
       </x:c>
       <x:c r="E14" s="742" t="str">
-        <x:v>Allowed admin/shelter booking list</x:v>
+        <x:v>Correct lane booking list</x:v>
       </x:c>
       <x:c r="F14" s="742" t="str">
         <x:v>Shared page is good because data is one appointment row</x:v>
@@ -8310,7 +8541,7 @@
     </x:row>
     <x:row r="15" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A15" s="742" t="str">
-        <x:v>/booking/[id]/visitor-profile</x:v>
+        <x:v>.../bookings/[id]/visitor-profile</x:v>
       </x:c>
       <x:c r="B15" s="742" t="str">
         <x:v>PawJai admin or linked shelter staff</x:v>
@@ -8319,10 +8550,10 @@
         <x:v>Wrong shelter, public users</x:v>
       </x:c>
       <x:c r="D15" s="742" t="str">
-        <x:v>canAccessShelter on appointment.shelter_id</x:v>
+        <x:v>shared renderer + canAccessShelter on appointment.shelter_id</x:v>
       </x:c>
       <x:c r="E15" s="742" t="str">
-        <x:v>/booking/[id] or booking list</x:v>
+        <x:v>Correct lane booking detail or list</x:v>
       </x:c>
       <x:c r="F15" s="742" t="str">
         <x:v>Protect adopter documents</x:v>
@@ -8333,7 +8564,7 @@
     </x:row>
     <x:row r="16" s="62" customFormat="1" ht="54" customHeight="1">
       <x:c r="A16" s="742" t="str">
-        <x:v>/booking/check-in</x:v>
+        <x:v>.../bookings/check-in</x:v>
       </x:c>
       <x:c r="B16" s="742" t="str">
         <x:v>PawJai admin or linked shelter staff with QR token</x:v>
@@ -8342,10 +8573,10 @@
         <x:v>Wrong shelter, public users</x:v>
       </x:c>
       <x:c r="D16" s="742" t="str">
-        <x:v>Signed token + appointment shelter access</x:v>
+        <x:v>signed token + appointment shelter access</x:v>
       </x:c>
       <x:c r="E16" s="742" t="str">
-        <x:v>/booking/[id]</x:v>
+        <x:v>Correct lane booking detail</x:v>
       </x:c>
       <x:c r="F16" s="742" t="str">
         <x:v>Needs real phone camera test</x:v>
@@ -8379,25 +8610,25 @@
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
       <x:c r="A18" s="742" t="str">
+        <x:v>/admindraft/*</x:v>
+      </x:c>
+      <x:c r="B18" s="742" t="str">
+        <x:v>Anyone with an old bookmark; destination still requires admin auth</x:v>
+      </x:c>
+      <x:c r="C18" s="742" t="str">
+        <x:v>Shelter/public access to destination</x:v>
+      </x:c>
+      <x:c r="D18" s="742" t="str">
+        <x:v>Permanent Next.js redirect to /admin/*, then normal admin guard</x:v>
+      </x:c>
+      <x:c r="E18" s="742" t="str">
         <x:v>/admin/*</x:v>
       </x:c>
-      <x:c r="B18" s="742" t="str">
-        <x:v>PawJai internal during migration</x:v>
-      </x:c>
-      <x:c r="C18" s="742" t="str">
-        <x:v>Shelter staff</x:v>
-      </x:c>
-      <x:c r="D18" s="742" t="str">
-        <x:v>Legacy gate / redirects depending route</x:v>
-      </x:c>
-      <x:c r="E18" s="742" t="str">
-        <x:v>Old admin or draft</x:v>
-      </x:c>
       <x:c r="F18" s="742" t="str">
-        <x:v>Keep until cutover; then redirect/remove</x:v>
+        <x:v>Compatibility only; product must never generate this URL</x:v>
       </x:c>
       <x:c r="G18" s="723" t="str">
-        <x:v>Remaining</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8437,7 +8668,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1115" t="str">
-        <x:v>Updated 2026-08-16 +07. Canonical domain is pawjaipet.com. Temporary/shared pilot gates should be replaced with real account-based auth before broad shelter rollout. No secrets are stored in this tracker.</x:v>
+        <x:v>Updated 2026-08-22 +07. Canonical PawJai HQ route is /admin with Google-only authentication. /admindraft is retained only as a permanent compatibility redirect. No secrets are stored in this tracker.</x:v>
       </x:c>
       <x:c r="B2" s="1115"/>
       <x:c r="C2" s="1115"/>
@@ -8693,80 +8924,80 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1170" t="str">
-        <x:v>PawJai admin draft umbrella</x:v>
+        <x:v>PawJai admin umbrella</x:v>
       </x:c>
       <x:c r="B13" s="1170" t="str">
-        <x:v>https://www.pawjaipet.com/admindraft</x:v>
+        <x:v>https://www.pawjaipet.com/admin</x:v>
       </x:c>
       <x:c r="C13" s="1170" t="str">
         <x:v>PawJai HQ only</x:v>
       </x:c>
       <x:c r="D13" s="1171" t="str">
-        <x:v>Canonical draft admin</x:v>
+        <x:v>Canonical admin</x:v>
       </x:c>
       <x:c r="E13" s="1170" t="str">
-        <x:v>Sees all shelters, dogs, bookings, ads, About content, accounts, audit.</x:v>
+        <x:v>Finished reorganized workspace with all HQ tabs and View as shelter.</x:v>
       </x:c>
       <x:c r="F13" s="1125" t="str">
         <x:v>Plan admin reorg</x:v>
       </x:c>
       <x:c r="G13" s="1125" t="str">
-        <x:v>Pilot QA and real auth before broad use</x:v>
+        <x:v>Production smoke test after deployment</x:v>
       </x:c>
       <x:c r="H13" s="1125" t="str">
-        <x:v>2026-08-16</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1170" t="str">
-        <x:v>Legacy admin</x:v>
+        <x:v>Legacy admin draft alias</x:v>
       </x:c>
       <x:c r="B14" s="1170" t="str">
-        <x:v>https://www.pawjaipet.com/admin/*</x:v>
+        <x:v>https://www.pawjaipet.com/admindraft/*</x:v>
       </x:c>
       <x:c r="C14" s="1170" t="str">
-        <x:v>PawJai internal only</x:v>
+        <x:v>Old bookmarks only</x:v>
       </x:c>
       <x:c r="D14" s="1159" t="str">
-        <x:v>Legacy fallback</x:v>
+        <x:v>Permanent redirect</x:v>
       </x:c>
       <x:c r="E14" s="1170" t="str">
-        <x:v>Keep until admindraft cutover is complete.</x:v>
+        <x:v>Redirects to the matching /admin/* destination; no product UI generates this URL.</x:v>
       </x:c>
       <x:c r="F14" s="1125" t="str">
         <x:v>Plan admin reorg</x:v>
       </x:c>
       <x:c r="G14" s="1125" t="str">
-        <x:v>Decide redirect/remove later</x:v>
+        <x:v>Verify one legacy deep-link redirect after deployment</x:v>
       </x:c>
       <x:c r="H14" s="1125" t="str">
-        <x:v>2026-08-16</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1170" t="str">
-        <x:v>Admin profile editor</x:v>
+        <x:v>Admin About content editor</x:v>
       </x:c>
       <x:c r="B15" s="1170" t="str">
-        <x:v>https://www.pawjaipet.com/admin/pawjaiprofile</x:v>
+        <x:v>https://www.pawjaipet.com/admin/aboutcontent</x:v>
       </x:c>
       <x:c r="C15" s="1170" t="str">
         <x:v>PawJai HQ only</x:v>
       </x:c>
       <x:c r="D15" s="1159" t="str">
-        <x:v>Needs smoke test</x:v>
+        <x:v>Canonical / guarded</x:v>
       </x:c>
       <x:c r="E15" s="1170" t="str">
-        <x:v>Code no longer shows exported-object server-action bug, but save flow should be tested.</x:v>
+        <x:v>Uses the finalized editor and the canonical admin login/return path.</x:v>
       </x:c>
       <x:c r="F15" s="1125" t="str">
         <x:v>Plan admin reorg</x:v>
       </x:c>
       <x:c r="G15" s="1125" t="str">
-        <x:v>Save About content once safely</x:v>
+        <x:v>Safe content save smoke test</x:v>
       </x:c>
       <x:c r="H15" s="1125" t="str">
-        <x:v>2026-08-16</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -8826,16 +9057,16 @@
         <x:v>Booking detail</x:v>
       </x:c>
       <x:c r="B18" s="1125" t="str">
-        <x:v>https://www.pawjaipet.com/booking/[id]</x:v>
+        <x:v>https://www.pawjaipet.com/admin/bookings/[id] or /shelter/[slug]/bookings/[id]</x:v>
       </x:c>
       <x:c r="C18" s="1125" t="str">
         <x:v>PawJai admin + linked shelter</x:v>
       </x:c>
       <x:c r="D18" s="1125" t="str">
-        <x:v>Shared guarded internal route</x:v>
+        <x:v>Shared implementation / role-specific route</x:v>
       </x:c>
       <x:c r="E18" s="1125" t="str">
-        <x:v>Validated access and returnTo keep users in correct lane.</x:v>
+        <x:v>Same appointment record; lane-aware access and returnTo keep each user in the correct workspace.</x:v>
       </x:c>
       <x:c r="F18" s="1125" t="str">
         <x:v>BACKEND related</x:v>
@@ -8844,7 +9075,7 @@
         <x:v>Pilot booking decision QA</x:v>
       </x:c>
       <x:c r="H18" s="1125" t="str">
-        <x:v>2026-08-16</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -8852,16 +9083,16 @@
         <x:v>Visitor profile</x:v>
       </x:c>
       <x:c r="B19" s="1125" t="str">
-        <x:v>https://www.pawjaipet.com/booking/[id]/visitor-profile</x:v>
+        <x:v>https://www.pawjaipet.com/admin/bookings/[id]/visitor-profile or /shelter/[slug]/bookings/[id]/visitor-profile</x:v>
       </x:c>
       <x:c r="C19" s="1125" t="str">
         <x:v>PawJai admin + linked shelter</x:v>
       </x:c>
       <x:c r="D19" s="1125" t="str">
-        <x:v>Shared guarded internal route</x:v>
+        <x:v>Shared implementation / role-specific route</x:v>
       </x:c>
       <x:c r="E19" s="1125" t="str">
-        <x:v>Contains adopter/visitor context; protect access.</x:v>
+        <x:v>Same adopter/document records; wrong shelters and public users are blocked.</x:v>
       </x:c>
       <x:c r="F19" s="1125" t="str">
         <x:v>BACKEND related</x:v>
@@ -8870,7 +9101,7 @@
         <x:v>Route denial QA</x:v>
       </x:c>
       <x:c r="H19" s="1125" t="str">
-        <x:v>2026-08-16</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -11663,6 +11894,294 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="1270" t="str">
+        <x:v>PAWJAI /admin Canonical Route Cutover</x:v>
+      </x:c>
+      <x:c r="B1" s="1270"/>
+      <x:c r="C1" s="1270"/>
+      <x:c r="D1" s="1270"/>
+      <x:c r="E1" s="1270"/>
+      <x:c r="F1" s="1270"/>
+      <x:c r="G1" s="1270"/>
+    </x:row>
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A2" s="1239" t="str">
+        <x:v>Implemented and locally verified 2026-08-22 +07. This sheet records the URL promotion only; the database schema and storage buckets are unchanged.</x:v>
+      </x:c>
+      <x:c r="B2" s="1239"/>
+      <x:c r="C2" s="1239"/>
+      <x:c r="D2" s="1239"/>
+      <x:c r="E2" s="1239"/>
+      <x:c r="F2" s="1239"/>
+      <x:c r="G2" s="1239"/>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="1242" t="str">
+        <x:v>Area</x:v>
+      </x:c>
+      <x:c r="B4" s="1242" t="str">
+        <x:v>Previous route</x:v>
+      </x:c>
+      <x:c r="C4" s="1242" t="str">
+        <x:v>Canonical route</x:v>
+      </x:c>
+      <x:c r="D4" s="1242" t="str">
+        <x:v>Implementation</x:v>
+      </x:c>
+      <x:c r="E4" s="1242" t="str">
+        <x:v>Safety behavior</x:v>
+      </x:c>
+      <x:c r="F4" s="1242" t="str">
+        <x:v>Verification</x:v>
+      </x:c>
+      <x:c r="G4" s="1242" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A5" s="1253" t="str">
+        <x:v>HQ umbrella</x:v>
+      </x:c>
+      <x:c r="B5" s="1254" t="str">
+        <x:v>/admindraft</x:v>
+      </x:c>
+      <x:c r="C5" s="1254" t="str">
+        <x:v>/admin</x:v>
+      </x:c>
+      <x:c r="D5" s="1254" t="str">
+        <x:v>Finished workspace now renders from app/admin</x:v>
+      </x:c>
+      <x:c r="E5" s="1254" t="str">
+        <x:v>Google global-admin guard</x:v>
+      </x:c>
+      <x:c r="F5" s="1254" t="str">
+        <x:v>Route/auth source tests</x:v>
+      </x:c>
+      <x:c r="G5" s="1265" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A6" s="1256" t="str">
+        <x:v>Admin login</x:v>
+      </x:c>
+      <x:c r="B6" s="1257" t="str">
+        <x:v>/admindraft gate / legacy admin</x:v>
+      </x:c>
+      <x:c r="C6" s="1257" t="str">
+        <x:v>/admin/login</x:v>
+      </x:c>
+      <x:c r="D6" s="1257" t="str">
+        <x:v>Google-only PawJai account with sanitized next</x:v>
+      </x:c>
+      <x:c r="E6" s="1257" t="str">
+        <x:v>Shelter sessions redirect to /shelter/[slug]</x:v>
+      </x:c>
+      <x:c r="F6" s="1257" t="str">
+        <x:v>Auth contract tests</x:v>
+      </x:c>
+      <x:c r="G6" s="1266" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A7" s="1256" t="str">
+        <x:v>Dog create/edit</x:v>
+      </x:c>
+      <x:c r="B7" s="1257" t="str">
+        <x:v>/admindraft/dogs/*</x:v>
+      </x:c>
+      <x:c r="C7" s="1257" t="str">
+        <x:v>/admin/dogs/*</x:v>
+      </x:c>
+      <x:c r="D7" s="1257" t="str">
+        <x:v>Same production forms, actions, photos, traits, and buckets</x:v>
+      </x:c>
+      <x:c r="E7" s="1257" t="str">
+        <x:v>requireGlobalAdmin; shelter owns separate scoped URLs</x:v>
+      </x:c>
+      <x:c r="F7" s="1257" t="str">
+        <x:v>Form + route tests</x:v>
+      </x:c>
+      <x:c r="G7" s="1266" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A8" s="1256" t="str">
+        <x:v>Bookings</x:v>
+      </x:c>
+      <x:c r="B8" s="1257" t="str">
+        <x:v>/admindraft/bookings/*</x:v>
+      </x:c>
+      <x:c r="C8" s="1257" t="str">
+        <x:v>/admin/bookings/*</x:v>
+      </x:c>
+      <x:c r="D8" s="1257" t="str">
+        <x:v>Admin aliases reuse shared guarded booking renderers</x:v>
+      </x:c>
+      <x:c r="E8" s="1257" t="str">
+        <x:v>Lane-aware returnTo and shelter access checks</x:v>
+      </x:c>
+      <x:c r="F8" s="1257" t="str">
+        <x:v>Booking route tests</x:v>
+      </x:c>
+      <x:c r="G8" s="1266" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A9" s="1256" t="str">
+        <x:v>Ads</x:v>
+      </x:c>
+      <x:c r="B9" s="1257" t="str">
+        <x:v>/admindraft?view=ads</x:v>
+      </x:c>
+      <x:c r="C9" s="1257" t="str">
+        <x:v>/admin?view=ads</x:v>
+      </x:c>
+      <x:c r="D9" s="1257" t="str">
+        <x:v>Canonical tab plus /admin/ads redirect</x:v>
+      </x:c>
+      <x:c r="E9" s="1257" t="str">
+        <x:v>Global admin only</x:v>
+      </x:c>
+      <x:c r="F9" s="1257" t="str">
+        <x:v>Ad action tests</x:v>
+      </x:c>
+      <x:c r="G9" s="1266" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A10" s="1256" t="str">
+        <x:v>About/accounts/audit/analytics</x:v>
+      </x:c>
+      <x:c r="B10" s="1257" t="str">
+        <x:v>/admindraft/*</x:v>
+      </x:c>
+      <x:c r="C10" s="1257" t="str">
+        <x:v>/admin/*</x:v>
+      </x:c>
+      <x:c r="D10" s="1257" t="str">
+        <x:v>Unified branded admin shell</x:v>
+      </x:c>
+      <x:c r="E10" s="1257" t="str">
+        <x:v>Global admin only</x:v>
+      </x:c>
+      <x:c r="F10" s="1257" t="str">
+        <x:v>Admin workspace tests</x:v>
+      </x:c>
+      <x:c r="G10" s="1266" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A11" s="1256" t="str">
+        <x:v>Emails and mutations</x:v>
+      </x:c>
+      <x:c r="B11" s="1257" t="str">
+        <x:v>Mixed draft return URLs</x:v>
+      </x:c>
+      <x:c r="C11" s="1257" t="str">
+        <x:v>/admin return URLs</x:v>
+      </x:c>
+      <x:c r="D11" s="1257" t="str">
+        <x:v>Revalidation, links, and redirects canonicalized</x:v>
+      </x:c>
+      <x:c r="E11" s="1257" t="str">
+        <x:v>Legacy inputs are normalized before redirect</x:v>
+      </x:c>
+      <x:c r="F11" s="1257" t="str">
+        <x:v>156 automated tests</x:v>
+      </x:c>
+      <x:c r="G11" s="1266" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="66" hidden="0" customHeight="1">
+      <x:c r="A12" s="1256" t="str">
+        <x:v>Legacy URL</x:v>
+      </x:c>
+      <x:c r="B12" s="1257" t="str">
+        <x:v>/admindraft/*</x:v>
+      </x:c>
+      <x:c r="C12" s="1257" t="str">
+        <x:v>/admin/*</x:v>
+      </x:c>
+      <x:c r="D12" s="1257" t="str">
+        <x:v>Permanent Next.js compatibility redirect</x:v>
+      </x:c>
+      <x:c r="E12" s="1257" t="str">
+        <x:v>Destination re-enters normal admin guard</x:v>
+      </x:c>
+      <x:c r="F12" s="1257" t="str">
+        <x:v>Redirect contract test</x:v>
+      </x:c>
+      <x:c r="G12" s="1266" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A13" s="1259" t="str">
+        <x:v>Tracked-source typecheck</x:v>
+      </x:c>
+      <x:c r="B13" s="1260" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C13" s="1260" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="D13" s="1260" t="str">
+        <x:v>Isolated TypeScript check excluding unrelated untracked duplicate backup files</x:v>
+      </x:c>
+      <x:c r="E13" s="1260" t="str">
+        <x:v>No route implementation errors</x:v>
+      </x:c>
+      <x:c r="F13" s="1260" t="str">
+        <x:v>npx tsc --noEmit</x:v>
+      </x:c>
+      <x:c r="G13" s="1267" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14"/>
+    <x:row r="15" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A15" s="1269" t="str">
+        <x:v>Deployment note: production changes appear after this code is committed and pushed to main. Smoke-test /admin, /admin/login, one deep dog route, one booking route, and one /admindraft redirect after Vercel finishes.</x:v>
+      </x:c>
+      <x:c r="B15" s="1269"/>
+      <x:c r="C15" s="1269"/>
+      <x:c r="D15" s="1269"/>
+      <x:c r="E15" s="1269"/>
+      <x:c r="F15" s="1269"/>
+      <x:c r="G15" s="1269"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A15:G15"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -12177,7 +12696,7 @@
         <x:v>Old Admin Route</x:v>
       </x:c>
       <x:c r="C1" s="1" t="str">
-        <x:v>New Admin Draft Location</x:v>
+        <x:v>Canonical Admin Location</x:v>
       </x:c>
       <x:c r="D1" s="1" t="str">
         <x:v>Status</x:v>
@@ -12191,22 +12710,22 @@
     </x:row>
     <x:row r="2" s="62" customFormat="1" ht="48" customHeight="1">
       <x:c r="A2" s="684" t="str">
-        <x:v>Admin draft gate / password</x:v>
+        <x:v>PawJai admin Google login</x:v>
       </x:c>
       <x:c r="B2" s="684" t="str">
-        <x:v>/admin</x:v>
+        <x:v>/admin/login</x:v>
       </x:c>
       <x:c r="C2" s="684" t="str">
-        <x:v>/admindraft</x:v>
-      </x:c>
-      <x:c r="D2" s="685" t="str">
-        <x:v>Temporary</x:v>
+        <x:v>/admin/login</x:v>
+      </x:c>
+      <x:c r="D2" s="1272" t="str">
+        <x:v>Functional</x:v>
       </x:c>
       <x:c r="E2" s="684" t="str">
-        <x:v>Direct draft pages preserve returnTo, role=shelter preview state, and the temporary 8-hour unlock now persists across /admindraft, /booking, and legacy /admin hops; replace the phrase gate with real PawJai admin login later</x:v>
+        <x:v>Google-only PawJai HQ authentication is canonical. Legacy phrase cookies are cleared and no longer authorize admin access.</x:v>
       </x:c>
       <x:c r="F2" s="686" t="str">
-        <x:v>Later</x:v>
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="62" customFormat="1" ht="48" customHeight="1">
@@ -12214,19 +12733,19 @@
         <x:v>Main PawJai admin umbrella</x:v>
       </x:c>
       <x:c r="B3" s="684" t="str">
-        <x:v>scattered across /admin/*</x:v>
+        <x:v>scattered across legacy /admin/* and /admindraft</x:v>
       </x:c>
       <x:c r="C3" s="684" t="str">
-        <x:v>/admindraft</x:v>
+        <x:v>/admin</x:v>
       </x:c>
       <x:c r="D3" s="687" t="str">
-        <x:v>Exists</x:v>
+        <x:v>Functional</x:v>
       </x:c>
       <x:c r="E3" s="684" t="str">
-        <x:v>About, Accounts, Audit, dogs, shelter profile, bookings, Messaging, and Ads are draft-native; View as shelter now stays sticky through deep create/edit/booking routes; pilot QA, real admin auth, and old-admin cutover remain the main gaps</x:v>
-      </x:c>
-      <x:c r="F3" s="688" t="str">
-        <x:v>High</x:v>
+        <x:v>The completed reorganized workspace is now canonical at /admin with shelters, dogs, bookings, donations, ads, content, accounts, audit, analytics, and View as shelter.</x:v>
+      </x:c>
+      <x:c r="F3" s="1272" t="str">
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="62" customFormat="1" ht="32" customHeight="1">
@@ -12237,10 +12756,10 @@
         <x:v>mostly inside /admin/bookings</x:v>
       </x:c>
       <x:c r="C4" s="684" t="str">
-        <x:v>/admindraft &gt; Partner shelters</x:v>
-      </x:c>
-      <x:c r="D4" s="687" t="str">
-        <x:v>Exists</x:v>
+        <x:v>/admin?view=shelters</x:v>
+      </x:c>
+      <x:c r="D4" s="1272" t="str">
+        <x:v>Functional</x:v>
       </x:c>
       <x:c r="E4" s="684" t="str">
         <x:v>Add deeper shelter metrics and operational health summaries later if useful</x:v>
@@ -12257,7 +12776,7 @@
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
       <x:c r="C5" s="684" t="str">
-        <x:v>/admindraft &gt; Shelter profile</x:v>
+        <x:v>/admin?shelter=:id&amp;view=profile</x:v>
       </x:c>
       <x:c r="D5" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12277,7 +12796,7 @@
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
       <x:c r="C6" s="684" t="str">
-        <x:v>/admindraft &gt; Shelter profile</x:v>
+        <x:v>/admin?shelter=:id&amp;view=profile</x:v>
       </x:c>
       <x:c r="D6" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12297,7 +12816,7 @@
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
       <x:c r="C7" s="684" t="str">
-        <x:v>/admindraft &gt; Shelter profile</x:v>
+        <x:v>/admin?shelter=:id&amp;view=donations</x:v>
       </x:c>
       <x:c r="D7" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12317,7 +12836,7 @@
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
       <x:c r="C8" s="684" t="str">
-        <x:v>/admindraft &gt; Shelter profile</x:v>
+        <x:v>/admin?shelter=:id&amp;view=profile</x:v>
       </x:c>
       <x:c r="D8" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12337,7 +12856,7 @@
         <x:v>/admin/bookings?view=profile</x:v>
       </x:c>
       <x:c r="C9" s="684" t="str">
-        <x:v>/admindraft &gt; Shelter profile</x:v>
+        <x:v>/admin?shelter=:id&amp;view=bookings&amp;bookingView=calendar</x:v>
       </x:c>
       <x:c r="D9" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12357,7 +12876,7 @@
         <x:v>/admin/bookings?view=dogs, /admin/listings</x:v>
       </x:c>
       <x:c r="C10" s="684" t="str">
-        <x:v>/admindraft &gt; Dog listings</x:v>
+        <x:v>/admin?shelter=:id&amp;view=dogs</x:v>
       </x:c>
       <x:c r="D10" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12377,13 +12896,13 @@
         <x:v>/admin, /admin/dogs/new</x:v>
       </x:c>
       <x:c r="C11" s="684" t="str">
-        <x:v>/admindraft/dog-creation</x:v>
+        <x:v>/admin/dogs/new?shelter=:id</x:v>
       </x:c>
       <x:c r="D11" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E11" s="684" t="str">
-        <x:v>Draft-native create flow exists; role=shelter return paths now send View as shelter users back to the selected shelter dog list; real-world save/photo testing remains</x:v>
+        <x:v>Canonical /admin create flow uses the production form, actions, dog table, traits, and media buckets; final phone photo QA remains operational testing.</x:v>
       </x:c>
       <x:c r="F11" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12397,13 +12916,13 @@
         <x:v>/admin/dogs/[id]/edit</x:v>
       </x:c>
       <x:c r="C12" s="684" t="str">
-        <x:v>/admindraft/dogs/[id]/edit</x:v>
+        <x:v>/admin/dogs/[id]/edit</x:v>
       </x:c>
       <x:c r="D12" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E12" s="684" t="str">
-        <x:v>Draft-native edit route reuses the full old edit form; role=shelter return paths now keep View as shelter users in the same selected shelter dog list; real-world save/photo testing remains</x:v>
+        <x:v>Canonical /admin edit route uses the production form and shared records; final phone photo/reorder QA remains operational testing.</x:v>
       </x:c>
       <x:c r="F12" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12417,7 +12936,7 @@
         <x:v>/admin, /admin/dogs/[id]/edit</x:v>
       </x:c>
       <x:c r="C13" s="684" t="str">
-        <x:v>/admindraft/dogs/[id]/edit</x:v>
+        <x:v>/admin/dogs/[id]/edit</x:v>
       </x:c>
       <x:c r="D13" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12437,13 +12956,13 @@
         <x:v>/admin/listings</x:v>
       </x:c>
       <x:c r="C14" s="684" t="str">
-        <x:v>/admindraft &gt; All dog listings</x:v>
+        <x:v>/admin?view=dogs</x:v>
       </x:c>
       <x:c r="D14" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E14" s="684" t="str">
-        <x:v>Filters exist and edit buttons now open draft-native dog edit pages</x:v>
+        <x:v>Search and shelter/status filters are live; edit buttons open canonical /admin dog edit pages.</x:v>
       </x:c>
       <x:c r="F14" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12457,7 +12976,7 @@
         <x:v>/admin/bookings</x:v>
       </x:c>
       <x:c r="C15" s="684" t="str">
-        <x:v>/admindraft &gt; Bookings</x:v>
+        <x:v>/admin?view=bookings</x:v>
       </x:c>
       <x:c r="D15" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12477,13 +12996,13 @@
         <x:v>/admin/bookings, /admin/bookings/[id]</x:v>
       </x:c>
       <x:c r="C16" s="684" t="str">
-        <x:v>/admindraft &gt; Bookings</x:v>
+        <x:v>/admin?view=bookings or /admin/bookings/[id]</x:v>
       </x:c>
       <x:c r="D16" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E16" s="684" t="str">
-        <x:v>Accept, deny, and date-change actions are draft-native; final status edge cases can be polished later</x:v>
+        <x:v>Accept, deny, and date-change actions are canonical under /admin; harmless booking mutation QA remains an operational check.</x:v>
       </x:c>
       <x:c r="F16" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12497,7 +13016,7 @@
         <x:v>/admin/bookings/[id]</x:v>
       </x:c>
       <x:c r="C17" s="684" t="str">
-        <x:v>/admindraft/bookings/[id]</x:v>
+        <x:v>/admin/bookings/[id]</x:v>
       </x:c>
       <x:c r="D17" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12517,7 +13036,7 @@
         <x:v>/admin/bookings/check-in</x:v>
       </x:c>
       <x:c r="C18" s="684" t="str">
-        <x:v>/admindraft/bookings/check-in and /booking/check-in</x:v>
+        <x:v>/admin/bookings/check-in</x:v>
       </x:c>
       <x:c r="D18" s="687" t="str">
         <x:v>Functional</x:v>
@@ -12537,13 +13056,13 @@
         <x:v>/admin/bookings/[id]/visitor-profile</x:v>
       </x:c>
       <x:c r="C19" s="684" t="str">
-        <x:v>/admindraft/bookings/[id]/visitor-profile</x:v>
+        <x:v>/admin/bookings/[id]/visitor-profile</x:v>
       </x:c>
       <x:c r="D19" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E19" s="684" t="str">
-        <x:v>Draft-native profile/documents view exists; real document review testing remains</x:v>
+        <x:v>Canonical admin visitor profile and document view reuses the guarded shared renderer; live document review QA remains.</x:v>
       </x:c>
       <x:c r="F19" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12557,7 +13076,7 @@
         <x:v>/admin/bookings?view=messages</x:v>
       </x:c>
       <x:c r="C20" s="684" t="str">
-        <x:v>/admindraft &gt; Messaging and /shelter/[slug]?view=messages</x:v>
+        <x:v>/admin?view=messages</x:v>
       </x:c>
       <x:c r="D20" s="766" t="str">
         <x:v>Complete - QA passed</x:v>
@@ -12577,13 +13096,13 @@
         <x:v>/admin/ads</x:v>
       </x:c>
       <x:c r="C21" s="684" t="str">
-        <x:v>/admindraft/ads</x:v>
+        <x:v>/admin?view=ads</x:v>
       </x:c>
       <x:c r="D21" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E21" s="684" t="str">
-        <x:v>Draft-native create ad, edit dates, pause/resume, and delete controls now use the same ads table and media upload flow; live upload smoke test remains</x:v>
+        <x:v>Canonical /admin ads tab uses the same ads table and media flow; disposable live upload smoke test remains.</x:v>
       </x:c>
       <x:c r="F21" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12597,13 +13116,13 @@
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
       <x:c r="C22" s="684" t="str">
-        <x:v>/admindraft/aboutcontent</x:v>
+        <x:v>/admin/aboutcontent</x:v>
       </x:c>
       <x:c r="D22" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E22" s="684" t="str">
-        <x:v>Draft-native About editor now uses the finalized old admin UX/UI, saves through pawjai_profile, and no longer bounces back to /admindraft after unlock; live save smoke test remains</x:v>
+        <x:v>Canonical /admin/aboutcontent uses the finalized editor, saves through pawjai_profile, and returns to the same route after mutation.</x:v>
       </x:c>
       <x:c r="F22" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12617,13 +13136,13 @@
         <x:v>/admin/accounts</x:v>
       </x:c>
       <x:c r="C23" s="684" t="str">
-        <x:v>/admindraft/accounts</x:v>
+        <x:v>/admin/accounts</x:v>
       </x:c>
       <x:c r="D23" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E23" s="684" t="str">
-        <x:v>Draft-native account creation/revoke exists and uses the same Supabase Auth, profiles, and shelter_users logic</x:v>
+        <x:v>Canonical /admin/accounts uses the same Supabase Auth, profiles, and shelter_users logic.</x:v>
       </x:c>
       <x:c r="F23" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12637,13 +13156,13 @@
         <x:v>/admin/audit</x:v>
       </x:c>
       <x:c r="C24" s="684" t="str">
-        <x:v>/admindraft/audit</x:v>
+        <x:v>/admin/audit</x:v>
       </x:c>
       <x:c r="D24" s="687" t="str">
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="E24" s="684" t="str">
-        <x:v>Draft-native audit table exists; keep testing with real admin changes</x:v>
+        <x:v>Canonical /admin/audit reads the existing admin_audit_events table and remains HQ-only.</x:v>
       </x:c>
       <x:c r="F24" s="687" t="str">
         <x:v>Done-ish</x:v>
@@ -12651,42 +13170,42 @@
     </x:row>
     <x:row r="25" s="62" customFormat="1" ht="32" customHeight="1">
       <x:c r="A25" s="684" t="str">
-        <x:v>Admin login page</x:v>
+        <x:v>User analytics</x:v>
       </x:c>
       <x:c r="B25" s="684" t="str">
-        <x:v>/admin/login</x:v>
+        <x:v>new during admin reorganization</x:v>
       </x:c>
       <x:c r="C25" s="684" t="str">
-        <x:v>temporary root-scoped phrase gate</x:v>
-      </x:c>
-      <x:c r="D25" s="685" t="str">
-        <x:v>Temporary</x:v>
+        <x:v>/admin/analytics</x:v>
+      </x:c>
+      <x:c r="D25" s="1272" t="str">
+        <x:v>Functional</x:v>
       </x:c>
       <x:c r="E25" s="684" t="str">
-        <x:v>Later replace phrase gates with real PawJai admin auth and employee-level shelter accounts</x:v>
+        <x:v>Canonical HQ-only analytics route is inside the unified admin shell; continue monitoring launch traffic and event coverage.</x:v>
       </x:c>
       <x:c r="F25" s="686" t="str">
-        <x:v>Later</x:v>
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
     <x:row r="26" s="62" customFormat="1" ht="16" customHeight="1">
       <x:c r="A26" s="684" t="str">
-        <x:v>Legacy draft alias</x:v>
+        <x:v>Legacy draft URL compatibility</x:v>
       </x:c>
       <x:c r="B26" s="684" t="str">
-        <x:v>/admin/reorg-draft</x:v>
+        <x:v>/admindraft/*</x:v>
       </x:c>
       <x:c r="C26" s="684" t="str">
-        <x:v>/admindraft</x:v>
+        <x:v>/admin/*</x:v>
       </x:c>
       <x:c r="D26" s="687" t="str">
-        <x:v>Exists</x:v>
+        <x:v>Functional</x:v>
       </x:c>
       <x:c r="E26" s="684" t="str">
-        <x:v>Remove after /admindraft becomes canonical</x:v>
+        <x:v>Permanent redirects preserve old bookmarks while auth next paths and server actions canonicalize every return to /admin. Product UI no longer generates /admindraft links.</x:v>
       </x:c>
       <x:c r="F26" s="686" t="str">
-        <x:v>Later</x:v>
+        <x:v>Done-ish</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12706,7 +13225,7 @@
   <x:sheetData>
     <x:row r="1" s="62" customFormat="1" ht="21" customHeight="1">
       <x:c r="A1" s="1195" t="str">
-        <x:v>PAWJAI Admin Draft Transfer Progress</x:v>
+        <x:v>PAWJAI Admin Canonical Route Progress</x:v>
       </x:c>
       <x:c r="B1" s="1196"/>
       <x:c r="C1" s="1196"/>
@@ -12716,7 +13235,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1198" t="str">
-        <x:v>Updated 2026-08-21 +07. The shelter lane is now production-backed and route-audited for Voice and Rescue, with Thai, historical dog status, profile/donation/calendar saves, dog create/edit/storage, and route separation verified. Remaining pilot gates are recorded in Pilot Checklist and Shelter Pilot QA 2026-08-21.</x:v>
+        <x:v>Updated 2026-08-22 +07. The completed admin draft has been promoted to canonical /admin. All HQ tabs, dog and booking deep routes, auth returns, mutations, notifications, and view-as-shelter links now use /admin; /admindraft is compatibility redirect only.</x:v>
       </x:c>
       <x:c r="B2" s="1198"/>
       <x:c r="C2" s="1198"/>
@@ -12743,13 +13262,13 @@
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="B4" s="708" t="n">
-        <x:v>20</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C4" s="712" t="n">
-        <x:v>0.8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D4" s="117" t="str">
-        <x:v>Moved into draft and connected enough to use/test; messaging stress-tested 2026-07-24</x:v>
+        <x:v>Canonical /admin routes are connected; all automated route/auth tests pass</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12757,15 +13276,13 @@
         <x:v>Exists</x:v>
       </x:c>
       <x:c r="B5" s="708" t="n">
-        <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A5)</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="712" t="n">
-        <x:f>B5/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
-        <x:v>0.12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="117" t="str">
-        <x:v>Present in draft, but may still need deeper behavior</x:v>
+        <x:v>Present but not fully transferred</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12773,15 +13290,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="709" t="n">
-        <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="717" t="n">
-        <x:f>B6/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="117" t="str">
-        <x:v>Some behavior moved, still depends on old admin or missing pieces</x:v>
+        <x:v>Some behavior still depends on a previous admin route</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12789,15 +13304,13 @@
         <x:v>Read only</x:v>
       </x:c>
       <x:c r="B7" s="709" t="n">
-        <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="717" t="n">
-        <x:f>B7/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="117" t="str">
-        <x:v>Real data visible, write controls not transferred</x:v>
+        <x:v>Real data visible without write controls</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12805,11 +13318,9 @@
         <x:v>Visual only</x:v>
       </x:c>
       <x:c r="B8" s="710" t="n">
-        <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="718" t="n">
-        <x:f>B8/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="117" t="str">
@@ -12821,15 +13332,13 @@
         <x:v>Temporary</x:v>
       </x:c>
       <x:c r="B9" s="709" t="n">
-        <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A9)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="717" t="n">
-        <x:f>B9/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
-        <x:v>0.08</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="117" t="str">
-        <x:v>Temporary bridge until real auth/login</x:v>
+        <x:v>Temporary route or phrase-gate bridge</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12837,15 +13346,13 @@
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="B10" s="710" t="n">
-        <x:f>COUNTIF('Admin Transfer Tracker'!$D$2:$D$26,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="718" t="n">
-        <x:f>B10/COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="117" t="str">
-        <x:v>Not moved yet</x:v>
+        <x:v>Not transferred</x:v>
       </x:c>
     </x:row>
     <x:row r="13" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12861,7 +13368,7 @@
         <x:v>Functional workflows</x:v>
       </x:c>
       <x:c r="B14" s="708" t="n">
-        <x:v>20</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12869,7 +13376,7 @@
         <x:v>Functional + Exists</x:v>
       </x:c>
       <x:c r="B15" s="712" t="n">
-        <x:v>0.92</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12885,20 +13392,19 @@
         <x:v>Total workflows</x:v>
       </x:c>
       <x:c r="B17" s="713" t="n">
-        <x:f>COUNTA('Admin Transfer Tracker'!$A$2:$A$26)</x:f>
         <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="20" s="62" customFormat="1" ht="48" customHeight="1">
       <x:c r="A20" s="859" t="str">
-        <x:v>Messaging QA note</x:v>
+        <x:v>Admin route cutover</x:v>
       </x:c>
       <x:c r="B20" s="88" t="str">
-        <x:v>Passed 2026-07-24</x:v>
+        <x:v>Passed locally 2026-08-22</x:v>
       </x:c>
       <x:c r="C20" s="88"/>
       <x:c r="D20" s="88" t="str">
-        <x:v>File matrix and cleanup evidence recorded on Messaging QA Matrix.</x:v>
+        <x:v>156 automated tests pass; isolated tracked-source typecheck passes. Production activation follows the normal commit/push deployment.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12926,12 +13432,12 @@
   <x:sheetData>
     <x:row r="1" s="62" customFormat="1" ht="19.25" customHeight="1">
       <x:c r="A1" s="719" t="str">
-        <x:v>PAWJAI Admin -&gt; Shelter -&gt; Booking Route Migration Map</x:v>
+        <x:v>PAWJAI Admin -&gt; Shelter -&gt; Booking Canonical Route Map</x:v>
       </x:c>
     </x:row>
     <x:row r="2" s="62" customFormat="1" ht="15" customHeight="1">
       <x:c r="A2" s="721" t="str">
-        <x:v>Tracks what has moved from old /admin to /admindraft, what now belongs under /shelter, and what is shared through /booking.</x:v>
+        <x:v>The reorganized HQ workspace is canonical at /admin. Shelter staff remain under /shelter, while shared booking implementations expose role-specific admin and shelter URLs backed by the same records.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="62" customFormat="1" ht="15" customHeight="1">
@@ -12956,22 +13462,22 @@
     </x:row>
     <x:row r="5" s="62" customFormat="1" ht="26.25" customHeight="1">
       <x:c r="A5" s="133" t="str">
-        <x:v>Old production admin</x:v>
+        <x:v>Canonical PawJai admin</x:v>
       </x:c>
       <x:c r="B5" s="133" t="str">
-        <x:v>/admin</x:v>
+        <x:v>/admindraft and legacy /admin/*</x:v>
       </x:c>
       <x:c r="C5" s="133" t="str">
         <x:v>/admin</x:v>
       </x:c>
       <x:c r="D5" s="723" t="str">
-        <x:v>Legacy active</x:v>
+        <x:v>Canonical / live</x:v>
       </x:c>
       <x:c r="E5" s="133" t="str">
-        <x:v>Current live admin remains usable until /admindraft fully replaces it</x:v>
+        <x:v>PawJai HQ sees all shelters, dogs, bookings, donations, ads, content, accounts, audit, and analytics.</x:v>
       </x:c>
       <x:c r="F5" s="133" t="str">
-        <x:v>Do not delete until every workflow is verified in /admindraft and /shelter</x:v>
+        <x:v>All generated links and return paths use /admin.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="62" customFormat="1" ht="26.25" customHeight="1">
@@ -12979,39 +13485,39 @@
         <x:v>PawJai umbrella dashboard</x:v>
       </x:c>
       <x:c r="B6" s="133" t="str">
+        <x:v>/admindraft</x:v>
+      </x:c>
+      <x:c r="C6" s="133" t="str">
         <x:v>/admin</x:v>
       </x:c>
-      <x:c r="C6" s="133" t="str">
-        <x:v>/admindraft</x:v>
-      </x:c>
       <x:c r="D6" s="725" t="str">
-        <x:v>Moved / live</x:v>
+        <x:v>Canonical / live</x:v>
       </x:c>
       <x:c r="E6" s="133" t="str">
-        <x:v>PawJai HQ sees all shelters, dogs, bookings, ads, about content, accounts, and audit</x:v>
+        <x:v>The finished reorganized hierarchy is the production admin umbrella.</x:v>
       </x:c>
       <x:c r="F6" s="133" t="str">
-        <x:v>Keep as the admin umbrella; do not make shelter staff use this route</x:v>
+        <x:v>Shelter accounts are redirected to their own /shelter/[slug] portal.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="62" customFormat="1" ht="15" customHeight="1">
       <x:c r="A7" s="133" t="str">
-        <x:v>Admin draft gate</x:v>
+        <x:v>PawJai admin login</x:v>
       </x:c>
       <x:c r="B7" s="133" t="str">
+        <x:v>phrase-gated draft and old admin login</x:v>
+      </x:c>
+      <x:c r="C7" s="133" t="str">
         <x:v>/admin/login</x:v>
       </x:c>
-      <x:c r="C7" s="133" t="str">
-        <x:v>/admindraft gate</x:v>
-      </x:c>
       <x:c r="D7" s="723" t="str">
-        <x:v>Temporary</x:v>
+        <x:v>Canonical / live</x:v>
       </x:c>
       <x:c r="E7" s="133" t="str">
-        <x:v>Shared phrase gate unlocks PawJai HQ draft pages for 8 hours across /admindraft, /booking, and legacy /admin hops</x:v>
+        <x:v>Google-only PawJai HQ sign-in with sanitized deep-link return.</x:v>
       </x:c>
       <x:c r="F7" s="133" t="str">
-        <x:v>Preserves returnTo for direct pages such as /admindraft/aboutcontent and tolerates/clears older path-scoped cookies; replace with real admin auth later</x:v>
+        <x:v>Legacy /admindraft next paths canonicalize to /admin before redirect.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="62" customFormat="1" ht="26.25" customHeight="1">
@@ -13039,7 +13545,7 @@
         <x:v>Shelter workspace</x:v>
       </x:c>
       <x:c r="B9" s="133" t="str">
-        <x:v>/admindraft view-as-shelter</x:v>
+        <x:v>/admin?role=shelter</x:v>
       </x:c>
       <x:c r="C9" s="133" t="str">
         <x:v>/shelter/[slug]</x:v>
@@ -13079,7 +13585,7 @@
         <x:v>Dog listings inside shelter</x:v>
       </x:c>
       <x:c r="B11" s="133" t="str">
-        <x:v>/admindraft?view=dogs</x:v>
+        <x:v>/admin?view=dogs</x:v>
       </x:c>
       <x:c r="C11" s="133" t="str">
         <x:v>/shelter/[slug]?view=dogs</x:v>
@@ -13099,7 +13605,7 @@
         <x:v>Create dog</x:v>
       </x:c>
       <x:c r="B12" s="133" t="str">
-        <x:v>/admindraft/dog-creation?shelter=:id</x:v>
+        <x:v>/admin/dogs/new?shelter=:id</x:v>
       </x:c>
       <x:c r="C12" s="133" t="str">
         <x:v>/shelter/[slug]/dogs/new</x:v>
@@ -13119,7 +13625,7 @@
         <x:v>Edit dog</x:v>
       </x:c>
       <x:c r="B13" s="133" t="str">
-        <x:v>/admindraft/dogs/[id]/edit</x:v>
+        <x:v>/admin/dogs/[id]/edit</x:v>
       </x:c>
       <x:c r="C13" s="133" t="str">
         <x:v>/shelter/[slug]/dogs/[id]/edit</x:v>
@@ -13159,7 +13665,7 @@
         <x:v>Booking list</x:v>
       </x:c>
       <x:c r="B15" s="133" t="str">
-        <x:v>/admindraft?view=bookings</x:v>
+        <x:v>/admin?view=bookings</x:v>
       </x:c>
       <x:c r="C15" s="133" t="str">
         <x:v>/shelter/[slug]?view=bookings</x:v>
@@ -13168,10 +13674,10 @@
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E15" s="133" t="str">
-        <x:v>Shelter booking list remains inside shelter workspace</x:v>
+        <x:v>Shelter booking list remains inside its scoped workspace; PawJai sees the cross-shelter list at /admin?view=bookings.</x:v>
       </x:c>
       <x:c r="F15" s="133" t="str">
-        <x:v>Links open shared /booking detail with safe returnTo</x:v>
+        <x:v>Role-specific links open the guarded shared renderer and return to the correct lane.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="62" customFormat="1" ht="15" customHeight="1">
@@ -13179,19 +13685,19 @@
         <x:v>Booking detail</x:v>
       </x:c>
       <x:c r="B16" s="133" t="str">
-        <x:v>/admindraft/bookings/[id]</x:v>
+        <x:v>shared booking renderer + appointments row</x:v>
       </x:c>
       <x:c r="C16" s="133" t="str">
-        <x:v>/booking/[id]</x:v>
+        <x:v>/admin/bookings/[id] or /shelter/[slug]/bookings/[id]</x:v>
       </x:c>
       <x:c r="D16" s="725" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E16" s="133" t="str">
-        <x:v>Single internal booking detail page for PawJai admin and linked shelter</x:v>
+        <x:v>One booking detail implementation reads the same appointments, adopters, dogs, and shelters records through admin or shelter aliases.</x:v>
       </x:c>
       <x:c r="F16" s="133" t="str">
-        <x:v>No new SQL table; reads same appointments/adopters/dogs/shelters</x:v>
+        <x:v>The visible URL remains in the caller's lane; no duplicate SQL table or booking record.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="62" customFormat="1" ht="15" customHeight="1">
@@ -13199,19 +13705,19 @@
         <x:v>Visitor profile / verification</x:v>
       </x:c>
       <x:c r="B17" s="133" t="str">
-        <x:v>/admindraft/bookings/[id]/visitor-profile</x:v>
+        <x:v>shared visitor renderer + adopter documents</x:v>
       </x:c>
       <x:c r="C17" s="133" t="str">
-        <x:v>/booking/[id]/visitor-profile</x:v>
+        <x:v>/admin/bookings/[id]/visitor-profile or /shelter/[slug]/bookings/[id]/visitor-profile</x:v>
       </x:c>
       <x:c r="D17" s="725" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E17" s="133" t="str">
-        <x:v>Single internal visitor profile and verification document page</x:v>
+        <x:v>One visitor/verification implementation reads the same adopter and document records through admin or shelter aliases.</x:v>
       </x:c>
       <x:c r="F17" s="133" t="str">
-        <x:v>Back links use safe returnTo</x:v>
+        <x:v>Back links and authorization are lane-aware.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="62" customFormat="1" ht="15" customHeight="1">
@@ -13219,19 +13725,19 @@
         <x:v>QR check-in</x:v>
       </x:c>
       <x:c r="B18" s="133" t="str">
-        <x:v>/admindraft/bookings/check-in</x:v>
+        <x:v>shared QR resolver + appointment access</x:v>
       </x:c>
       <x:c r="C18" s="133" t="str">
-        <x:v>/booking/check-in</x:v>
+        <x:v>/admin/bookings/check-in or /shelter/[slug]/bookings/check-in</x:v>
       </x:c>
       <x:c r="D18" s="725" t="str">
         <x:v>Shared route live</x:v>
       </x:c>
       <x:c r="E18" s="133" t="str">
-        <x:v>QR token resolves to shared booking detail</x:v>
+        <x:v>One QR resolver checks the signed token and appointment shelter before opening the lane-specific booking detail.</x:v>
       </x:c>
       <x:c r="F18" s="133" t="str">
-        <x:v>Generated QR URLs now use /booking/check-in</x:v>
+        <x:v>Physical camera permission remains a manual phone test.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" s="62" customFormat="1" ht="48" customHeight="1">
@@ -13239,7 +13745,7 @@
         <x:v>Messaging</x:v>
       </x:c>
       <x:c r="B19" s="133" t="str">
-        <x:v>/admindraft shelter workspace</x:v>
+        <x:v>/admin?view=messages</x:v>
       </x:c>
       <x:c r="C19" s="133" t="str">
         <x:v>/shelter/[slug]?view=messages</x:v>
@@ -13248,10 +13754,10 @@
         <x:v>Launch-ready</x:v>
       </x:c>
       <x:c r="E19" s="133" t="str">
-        <x:v>Appointment-thread messaging is live across adopter, shelter, and PawJai admin read-only routes.</x:v>
+        <x:v>Appointment-thread messaging remains live for adopter and shelter, with PawJai admin read-only visibility.</x:v>
       </x:c>
       <x:c r="F19" s="133" t="str">
-        <x:v>Production QA passed for realtime, attachments, admin visibility, and cleanup; monitor first live conversations.</x:v>
+        <x:v>Production QA passed; monitor first live conversations.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" s="62" customFormat="1" ht="15" customHeight="1">
@@ -13259,19 +13765,19 @@
         <x:v>Ads</x:v>
       </x:c>
       <x:c r="B20" s="133" t="str">
-        <x:v>/admin/ads</x:v>
+        <x:v>/admin?view=ads</x:v>
       </x:c>
       <x:c r="C20" s="133" t="str">
-        <x:v>/admindraft/ads</x:v>
+        <x:v>/admin?view=ads</x:v>
       </x:c>
       <x:c r="D20" s="725" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E20" s="133" t="str">
-        <x:v>PawJai-managed ads can now be created, date-edited, paused/resumed, and deleted in the draft umbrella</x:v>
+        <x:v>PawJai-managed ads use the same ads table, B2 media upload, and public feed revalidation.</x:v>
       </x:c>
       <x:c r="F20" s="133" t="str">
-        <x:v>Uses the same ads table, B2 upload flow, and public ad feed revalidation</x:v>
+        <x:v>Canonical review surface is /admin?view=ads.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" s="62" customFormat="1" ht="31" customHeight="1">
@@ -13282,16 +13788,16 @@
         <x:v>/admin/pawjaiprofile</x:v>
       </x:c>
       <x:c r="C21" s="133" t="str">
-        <x:v>/admindraft/aboutcontent</x:v>
+        <x:v>/admin/aboutcontent</x:v>
       </x:c>
       <x:c r="D21" s="725" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E21" s="133" t="str">
-        <x:v>Full PawJai public content editor and save action</x:v>
+        <x:v>Full PawJai public content editor saves through pawjai_profile and revalidates /about.</x:v>
       </x:c>
       <x:c r="F21" s="133" t="str">
-        <x:v>Uses the same pawjai_profile table, revalidates /about, and unlock returns to /admindraft/aboutcontent</x:v>
+        <x:v>Canonical editor and return path are /admin/aboutcontent.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" s="62" customFormat="1" ht="16" customHeight="1">
@@ -13302,16 +13808,16 @@
         <x:v>/admin/accounts</x:v>
       </x:c>
       <x:c r="C22" s="133" t="str">
-        <x:v>/admindraft/accounts</x:v>
+        <x:v>/admin/accounts</x:v>
       </x:c>
       <x:c r="D22" s="725" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E22" s="133" t="str">
-        <x:v>PawJai/shelter admin account creation and revoke controls</x:v>
+        <x:v>PawJai and shelter account administration uses Supabase Auth, profiles, and shelter_users.</x:v>
       </x:c>
       <x:c r="F22" s="133" t="str">
-        <x:v>Uses Supabase Auth, profiles, and shelter_users</x:v>
+        <x:v>Canonical HQ-only route is /admin/accounts.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" s="62" customFormat="1" ht="16" customHeight="1">
@@ -13322,16 +13828,16 @@
         <x:v>/admin/audit</x:v>
       </x:c>
       <x:c r="C23" s="133" t="str">
-        <x:v>/admindraft/audit</x:v>
+        <x:v>/admin/audit</x:v>
       </x:c>
       <x:c r="D23" s="725" t="str">
         <x:v>Moved / live</x:v>
       </x:c>
       <x:c r="E23" s="133" t="str">
-        <x:v>Privileged admin activity table</x:v>
+        <x:v>Privileged admin activity reads admin_audit_events and scopes by admin context.</x:v>
       </x:c>
       <x:c r="F23" s="133" t="str">
-        <x:v>Reads admin_audit_events and scopes by admin context</x:v>
+        <x:v>Canonical HQ-only route is /admin/audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>